<commit_message>
Barranquita: interior nivelado (NPT 184.65, cuneta 184.60, area verde 184.55), cunetas al ras del patio de maniobra 184.50, D2 como pase
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -631,7 +631,7 @@
         <v/>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.832</v>
+        <v>0.894</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
@@ -658,7 +658,7 @@
         <v/>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.853</v>
+        <v>0.922</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
@@ -685,11 +685,11 @@
         <v/>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.734</v>
+        <v>0.796</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>D2: Cerco norte (x = 965.5): poza de salida que rebalsa a nivel del fondo de la hondonada natural (baja a la quebrada del norte)</t>
+          <t>D2: Cerco norte (x = 965.5): pase en el cimiento del cerco al terreno exterior que baja a la quebrada del norte</t>
         </is>
       </c>
     </row>
@@ -770,14 +770,14 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>4. Rasante: NTN +184.50 en la plataforma; en el resto del area dentro del cerco, el terreno de las curvas recortado a +184.50.</t>
+          <t>4. Interior del cerco nivelado: pisos y pasadizos NPT +184.65; borde de cuneta +184.60; areas verdes +184.55; patio de maniobra +184.50 (cuneta al ras, con rejilla). Fuera del cerco, el terreno natural.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>5. D1, D3 y D4 salen por un pase en el cimiento del cerco; D2 por una poza de salida (0.80 x 0.80 m) que rebalsa a nivel del terreno. Fuera del cerco no hay obra.</t>
+          <t>5. D1, D2, D3 y D4 salen por un pase en el cimiento del cerco. Fuera del cerco no hay obra.</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>minima 0.50 % (R-02 P-04-P-05); maxima 47.52 %</t>
+          <t>minima 0.50 % (R-01 P-01-P-02); maxima 20.16 %</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>inicio 0.30 a 0.30; minima 0.25 (R-01); maxima 0.85 (R-07, prog 82.5)</t>
+          <t>inicio 0.30 a 0.30; minima 0.25 (R-01); maxima 0.92 (R-07, prog 96.2)</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>15 empalmes; caida maxima 0.34 m (R-11 en P-26)</t>
+          <t>15 empalmes; caida maxima 0.34 m (R-16 en P-44)</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>D1 C.F. 183.465: pase en el cimiento del cerco; el terreno exterior queda bajo la C.F. a 0.8 m del cerco; D2 C.F. 180.154: poza de salida: rebalsa a 180.62 (fondo de la hondonada); afuera el fondo no sube y baja 0.25 m a 11.8 m; D3 C.F. 183.482: pase en el cimiento del cerco; el terreno exterior queda bajo la C.F. a 1.8 m del cerco; D4 C.F. 183.999: pase en el cimiento del cerco; el terreno exterior queda bajo la C.F. a 0.8 m del cerco</t>
+          <t>D1 C.F. 183.660: pase en el cimiento del cerco; el terreno exterior queda bajo la C.F. a 0.5 m del cerco; D2 C.F. 183.704: pase en el cimiento del cerco; el terreno exterior queda bajo la C.F. a 0.2 m del cerco; D3 C.F. 183.576: pase en el cimiento del cerco; el terreno exterior queda bajo la C.F. a 1.0 m del cerco; D4 C.F. 184.099: pase en el cimiento del cerco; el terreno exterior queda bajo la C.F. a 0.5 m del cerco</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Borde de la cuneta por debajo del NPT de los bloques vecinos</t>
+          <t>Borde de la cuneta 0.05 m bajo el NPT (+184.65) y 0.05 m sobre el area verde (+184.55)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>41 rotulos NPT revisados (bloques a menos de 5 m de una cuneta); NPT de 183.50 a 184.65; borde de cuneta &lt;= NPT en todos</t>
+          <t>borde de cuneta +184.60 en la red dentro del cerco (NPT +184.65, area verde +184.55); junto al patio de maniobra (NTN +184.50) borde al ras +184.50 en 292 puntos</t>
         </is>
       </c>
     </row>
@@ -1012,11 +1012,11 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>I = 211 mm/h, C = 0.80, area total 9393 m2; menor borde libre 0.072 m en R-12 P-43-P-44 (Q 134.8 l/s, y 0.185, h 0.26)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
+          <t>I = 211 mm/h, C = 0.80, area total 9393 m2; menor borde libre 0.115 m en R-01 P-03-D1 (Q 190.8 l/s, y 0.135, h 0.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="11" t="n">
         <v>9</v>
       </c>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>tramos de fuerte pendiente con V &gt; 3.0 m/s: R-01 P-03-D1 (S 19.1 %, V 5.28), R-12 P-40-P-41 (S 18.7 %, V 4.25), R-12 P-42-P-43 (S 6.9 %, V 3.33), R-15 P-53-P-41 (S 47.5 %, V 3.43) -&gt; gradas (escalones) de concreto</t>
+          <t>tramos de fuerte pendiente con V &gt; 3.0 m/s: R-01 P-03-D1 (S 8.0 %, V 3.91), R-07 P-30-D3 (S 17.2 %, V 4.37) -&gt; gradas (escalones) de concreto</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>ningun borde de cuneta pasa el cerco; solo las 3 salidas lo atraviesan</t>
+          <t>ningun borde de cuneta pasa el cerco; solo las 4 salidas lo atraviesan</t>
         </is>
       </c>
     </row>
@@ -1109,11 +1109,11 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>183.465</v>
+        <v>183.66</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>pase en el cimiento del cerco: el terreno exterior queda bajo la C.F. a 0.8 m (perfilado maximo 0.30 m, sin obra)</t>
+          <t>pase en el cimiento del cerco: el terreno exterior queda bajo la C.F. a 0.5 m (perfilado maximo 0.11 m, sin obra)</t>
         </is>
       </c>
     </row>
@@ -1125,11 +1125,11 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>180.154</v>
+        <v>183.704</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>poza de salida: rebalsa a 180.62; el fondo exterior no sube y baja 0.25 m a 11.8 m</t>
+          <t>pase en el cimiento del cerco: el terreno exterior queda bajo la C.F. a 0.2 m (perfilado maximo 0.00 m, sin obra)</t>
         </is>
       </c>
     </row>
@@ -1141,11 +1141,11 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>183.482</v>
+        <v>183.576</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>pase en el cimiento del cerco: el terreno exterior queda bajo la C.F. a 1.8 m (perfilado maximo 0.26 m, sin obra)</t>
+          <t>pase en el cimiento del cerco: el terreno exterior queda bajo la C.F. a 1.0 m (perfilado maximo 0.16 m, sin obra)</t>
         </is>
       </c>
     </row>
@@ -1157,11 +1157,11 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>183.999</v>
+        <v>184.099</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>pase en el cimiento del cerco: el terreno exterior queda bajo la C.F. a 0.8 m (perfilado maximo 0.25 m, sin obra)</t>
+          <t>pase en el cimiento del cerco: el terreno exterior queda bajo la C.F. a 0.5 m (perfilado maximo 0.15 m, sin obra)</t>
         </is>
       </c>
     </row>
@@ -1350,11 +1350,11 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>NTN de la plataforma de los bloques</t>
+          <t>Borde superior de la cuneta (rasante)</t>
         </is>
       </c>
       <c r="B11" s="14" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Rotulos NTN del plano de arquitectura</t>
+          <t>Indicacion del usuario: NPT +184.65 (pisos y pasadizos), area verde +184.55</t>
         </is>
       </c>
     </row>
@@ -1596,20 +1596,20 @@
         <v/>
       </c>
       <c r="F11" s="18" t="n">
-        <v>0.93</v>
+        <v>0.5</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>0.077</v>
+        <v>0.095</v>
       </c>
       <c r="H11" s="18" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="I11" s="20">
         <f>H11-G11</f>
         <v/>
       </c>
       <c r="J11" s="6" t="n">
-        <v>1.03</v>
+        <v>0.84</v>
       </c>
       <c r="K11" s="21">
         <f>IF(I11&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1645,20 +1645,20 @@
         <v/>
       </c>
       <c r="F12" s="18" t="n">
-        <v>15.15</v>
+        <v>20.16</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>0.032</v>
+        <v>0.029</v>
       </c>
       <c r="H12" s="18" t="n">
-        <v>0.25</v>
+        <v>0.46</v>
       </c>
       <c r="I12" s="20">
         <f>H12-G12</f>
         <v/>
       </c>
       <c r="J12" s="6" t="n">
-        <v>2.58</v>
+        <v>2.82</v>
       </c>
       <c r="K12" s="21">
         <f>IF(I12&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1694,20 +1694,20 @@
         <v/>
       </c>
       <c r="F13" s="18" t="n">
-        <v>19.13</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0.1</v>
+        <v>0.135</v>
       </c>
       <c r="H13" s="18" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="I13" s="20">
         <f>H13-G13</f>
         <v/>
       </c>
       <c r="J13" s="6" t="n">
-        <v>5.28</v>
+        <v>3.91</v>
       </c>
       <c r="K13" s="21">
         <f>IF(I13&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1949,7 +1949,7 @@
         <v>0.339</v>
       </c>
       <c r="H18" s="18" t="n">
-        <v>0.42</v>
+        <v>0.83</v>
       </c>
       <c r="I18" s="20">
         <f>H18-G18</f>
@@ -2880,7 +2880,7 @@
         <v>0.256</v>
       </c>
       <c r="H37" s="18" t="n">
-        <v>0.72</v>
+        <v>0.79</v>
       </c>
       <c r="I37" s="20">
         <f>H37-G37</f>
@@ -2929,7 +2929,7 @@
         <v>0.258</v>
       </c>
       <c r="H38" s="18" t="n">
-        <v>0.72</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="I38" s="20">
         <f>H38-G38</f>
@@ -2972,20 +2972,20 @@
         <v/>
       </c>
       <c r="F39" s="18" t="n">
-        <v>1.14</v>
+        <v>0.5</v>
       </c>
       <c r="G39" s="19" t="n">
-        <v>0.19</v>
+        <v>0.26</v>
       </c>
       <c r="H39" s="18" t="n">
-        <v>0.27</v>
+        <v>0.85</v>
       </c>
       <c r="I39" s="20">
         <f>H39-G39</f>
         <v/>
       </c>
       <c r="J39" s="6" t="n">
-        <v>1.68</v>
+        <v>1.23</v>
       </c>
       <c r="K39" s="21">
         <f>IF(I39&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3021,20 +3021,20 @@
         <v/>
       </c>
       <c r="F40" s="18" t="n">
-        <v>1.13</v>
+        <v>0.5</v>
       </c>
       <c r="G40" s="19" t="n">
-        <v>0.195</v>
+        <v>0.266</v>
       </c>
       <c r="H40" s="18" t="n">
-        <v>0.27</v>
+        <v>0.88</v>
       </c>
       <c r="I40" s="20">
         <f>H40-G40</f>
         <v/>
       </c>
       <c r="J40" s="6" t="n">
-        <v>1.68</v>
+        <v>1.24</v>
       </c>
       <c r="K40" s="21">
         <f>IF(I40&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3070,20 +3070,20 @@
         <v/>
       </c>
       <c r="F41" s="18" t="n">
-        <v>0.5</v>
+        <v>17.21</v>
       </c>
       <c r="G41" s="19" t="n">
-        <v>0.266</v>
+        <v>0.075</v>
       </c>
       <c r="H41" s="18" t="n">
-        <v>0.34</v>
+        <v>0.25</v>
       </c>
       <c r="I41" s="20">
         <f>H41-G41</f>
         <v/>
       </c>
       <c r="J41" s="6" t="n">
-        <v>1.24</v>
+        <v>4.37</v>
       </c>
       <c r="K41" s="21">
         <f>IF(I41&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3093,7 +3093,11 @@
         <f>IF(J41&lt;=$B$7,"CUMPLE","GRADAS")</f>
         <v/>
       </c>
-      <c r="M41" s="22" t="inlineStr"/>
+      <c r="M41" s="22" t="inlineStr">
+        <is>
+          <t>gradas de concreto (escalones) en este tramo</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
@@ -3615,7 +3619,7 @@
         <v>0.161</v>
       </c>
       <c r="H52" s="18" t="n">
-        <v>0.67</v>
+        <v>0.57</v>
       </c>
       <c r="I52" s="20">
         <f>H52-G52</f>
@@ -3658,20 +3662,20 @@
         <v/>
       </c>
       <c r="F53" s="18" t="n">
-        <v>18.72</v>
+        <v>0.5</v>
       </c>
       <c r="G53" s="19" t="n">
-        <v>0.065</v>
+        <v>0.235</v>
       </c>
       <c r="H53" s="18" t="n">
-        <v>0.25</v>
+        <v>0.62</v>
       </c>
       <c r="I53" s="20">
         <f>H53-G53</f>
         <v/>
       </c>
       <c r="J53" s="6" t="n">
-        <v>4.25</v>
+        <v>1.19</v>
       </c>
       <c r="K53" s="21">
         <f>IF(I53&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3681,11 +3685,7 @@
         <f>IF(J53&lt;=$B$7,"CUMPLE","GRADAS")</f>
         <v/>
       </c>
-      <c r="M53" s="22" t="inlineStr">
-        <is>
-          <t>gradas de concreto (escalones) en este tramo</t>
-        </is>
-      </c>
+      <c r="M53" s="22" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
@@ -3711,20 +3711,20 @@
         <v/>
       </c>
       <c r="F54" s="18" t="n">
-        <v>5.03</v>
+        <v>0.5</v>
       </c>
       <c r="G54" s="19" t="n">
-        <v>0.12</v>
+        <v>0.282</v>
       </c>
       <c r="H54" s="18" t="n">
-        <v>0.25</v>
+        <v>0.68</v>
       </c>
       <c r="I54" s="20">
         <f>H54-G54</f>
         <v/>
       </c>
       <c r="J54" s="6" t="n">
-        <v>2.94</v>
+        <v>1.26</v>
       </c>
       <c r="K54" s="21">
         <f>IF(I54&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3760,20 +3760,20 @@
         <v/>
       </c>
       <c r="F55" s="18" t="n">
-        <v>6.92</v>
+        <v>0.5</v>
       </c>
       <c r="G55" s="19" t="n">
-        <v>0.111</v>
+        <v>0.294</v>
       </c>
       <c r="H55" s="18" t="n">
-        <v>0.26</v>
+        <v>0.72</v>
       </c>
       <c r="I55" s="20">
         <f>H55-G55</f>
         <v/>
       </c>
       <c r="J55" s="6" t="n">
-        <v>3.33</v>
+        <v>1.28</v>
       </c>
       <c r="K55" s="21">
         <f>IF(I55&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3783,11 +3783,7 @@
         <f>IF(J55&lt;=$B$7,"CUMPLE","GRADAS")</f>
         <v/>
       </c>
-      <c r="M55" s="22" t="inlineStr">
-        <is>
-          <t>gradas de concreto (escalones) en este tramo</t>
-        </is>
-      </c>
+      <c r="M55" s="22" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
@@ -3813,20 +3809,20 @@
         <v/>
       </c>
       <c r="F56" s="18" t="n">
-        <v>1.69</v>
+        <v>0.5</v>
       </c>
       <c r="G56" s="19" t="n">
-        <v>0.185</v>
+        <v>0.295</v>
       </c>
       <c r="H56" s="18" t="n">
-        <v>0.26</v>
+        <v>0.78</v>
       </c>
       <c r="I56" s="20">
         <f>H56-G56</f>
         <v/>
       </c>
       <c r="J56" s="6" t="n">
-        <v>2.02</v>
+        <v>1.28</v>
       </c>
       <c r="K56" s="21">
         <f>IF(I56&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3862,20 +3858,20 @@
         <v/>
       </c>
       <c r="F57" s="18" t="n">
-        <v>11.71</v>
+        <v>0.5</v>
       </c>
       <c r="G57" s="19" t="n">
-        <v>0.106</v>
+        <v>0.344</v>
       </c>
       <c r="H57" s="18" t="n">
-        <v>0.4</v>
+        <v>0.79</v>
       </c>
       <c r="I57" s="20">
         <f>H57-G57</f>
         <v/>
       </c>
       <c r="J57" s="6" t="n">
-        <v>4.25</v>
+        <v>1.33</v>
       </c>
       <c r="K57" s="21">
         <f>IF(I57&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4064,7 +4060,7 @@
         <v>0.089</v>
       </c>
       <c r="H61" s="18" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="I61" s="20">
         <f>H61-G61</f>
@@ -4113,7 +4109,7 @@
         <v>0.112</v>
       </c>
       <c r="H62" s="18" t="n">
-        <v>0.51</v>
+        <v>0.41</v>
       </c>
       <c r="I62" s="20">
         <f>H62-G62</f>
@@ -4162,7 +4158,7 @@
         <v>0.114</v>
       </c>
       <c r="H63" s="18" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="I63" s="20">
         <f>H63-G63</f>
@@ -4303,20 +4299,20 @@
         <v/>
       </c>
       <c r="F66" s="18" t="n">
-        <v>47.52</v>
+        <v>0.5</v>
       </c>
       <c r="G66" s="19" t="n">
-        <v>0.02</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="H66" s="18" t="n">
-        <v>0.25</v>
+        <v>0.38</v>
       </c>
       <c r="I66" s="20">
         <f>H66-G66</f>
         <v/>
       </c>
       <c r="J66" s="6" t="n">
-        <v>3.43</v>
+        <v>0.79</v>
       </c>
       <c r="K66" s="21">
         <f>IF(I66&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4326,11 +4322,7 @@
         <f>IF(J66&lt;=$B$7,"CUMPLE","GRADAS")</f>
         <v/>
       </c>
-      <c r="M66" s="22" t="inlineStr">
-        <is>
-          <t>gradas de concreto (escalones) en este tramo</t>
-        </is>
-      </c>
+      <c r="M66" s="22" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
@@ -4405,20 +4397,20 @@
         <v/>
       </c>
       <c r="F68" s="18" t="n">
-        <v>11.05</v>
+        <v>0.5</v>
       </c>
       <c r="G68" s="19" t="n">
-        <v>0.029</v>
+        <v>0.081</v>
       </c>
       <c r="H68" s="18" t="n">
-        <v>0.25</v>
+        <v>0.46</v>
       </c>
       <c r="I68" s="20">
         <f>H68-G68</f>
         <v/>
       </c>
       <c r="J68" s="6" t="n">
-        <v>2.11</v>
+        <v>0.77</v>
       </c>
       <c r="K68" s="21">
         <f>IF(I68&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4454,20 +4446,20 @@
         <v/>
       </c>
       <c r="F69" s="18" t="n">
-        <v>21.72</v>
+        <v>0.5</v>
       </c>
       <c r="G69" s="19" t="n">
-        <v>0.027</v>
+        <v>0.094</v>
       </c>
       <c r="H69" s="18" t="n">
-        <v>0.25</v>
+        <v>0.45</v>
       </c>
       <c r="I69" s="20">
         <f>H69-G69</f>
         <v/>
       </c>
       <c r="J69" s="6" t="n">
-        <v>2.84</v>
+        <v>0.83</v>
       </c>
       <c r="K69" s="21">
         <f>IF(I69&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4984,16 +4976,16 @@
         <v>31.9</v>
       </c>
       <c r="F5" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>184.155</v>
+        <v>184.6</v>
       </c>
       <c r="H5" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I5" s="25" t="n">
-        <v>183.905</v>
+        <v>184.141</v>
       </c>
       <c r="J5" s="26">
         <f>F5-H5</f>
@@ -5051,16 +5043,16 @@
         <v>2.15</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>184.155</v>
+        <v>184.6</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>184.024</v>
+        <v>184.6</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>183.905</v>
+        <v>184.141</v>
       </c>
       <c r="I6" s="25" t="n">
-        <v>183.579</v>
+        <v>183.708</v>
       </c>
       <c r="J6" s="26">
         <f>F6-H6</f>
@@ -5118,16 +5110,16 @@
         <v>0.6</v>
       </c>
       <c r="F7" s="24" t="n">
-        <v>184.024</v>
+        <v>184.6</v>
       </c>
       <c r="G7" s="24" t="n">
         <v>183.91</v>
       </c>
       <c r="H7" s="25" t="n">
-        <v>183.579</v>
+        <v>183.708</v>
       </c>
       <c r="I7" s="25" t="n">
-        <v>183.465</v>
+        <v>183.66</v>
       </c>
       <c r="J7" s="26">
         <f>F7-H7</f>
@@ -5185,16 +5177,16 @@
         <v>32.42</v>
       </c>
       <c r="F8" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H8" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I8" s="25" t="n">
-        <v>184.038</v>
+        <v>184.138</v>
       </c>
       <c r="J8" s="26">
         <f>F8-H8</f>
@@ -5252,16 +5244,16 @@
         <v>11.53</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H9" s="25" t="n">
-        <v>184.038</v>
+        <v>184.138</v>
       </c>
       <c r="I9" s="25" t="n">
-        <v>183.98</v>
+        <v>184.08</v>
       </c>
       <c r="J9" s="26">
         <f>F9-H9</f>
@@ -5319,16 +5311,16 @@
         <v>8.68</v>
       </c>
       <c r="F10" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>183.98</v>
+        <v>184.08</v>
       </c>
       <c r="I10" s="25" t="n">
-        <v>183.726</v>
+        <v>183.826</v>
       </c>
       <c r="J10" s="26">
         <f>F10-H10</f>
@@ -5386,16 +5378,16 @@
         <v>11.47</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H11" s="25" t="n">
-        <v>183.726</v>
+        <v>183.826</v>
       </c>
       <c r="I11" s="25" t="n">
-        <v>183.668</v>
+        <v>183.768</v>
       </c>
       <c r="J11" s="26">
         <f>F11-H11</f>
@@ -5453,16 +5445,16 @@
         <v>12.1</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>184.024</v>
+        <v>184.6</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>183.668</v>
+        <v>183.768</v>
       </c>
       <c r="I12" s="25" t="n">
-        <v>183.608</v>
+        <v>183.708</v>
       </c>
       <c r="J12" s="26">
         <f>F12-H12</f>
@@ -5520,16 +5512,16 @@
         <v>32.31</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G13" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H13" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>184.038</v>
+        <v>184.138</v>
       </c>
       <c r="J13" s="26">
         <f>F13-H13</f>
@@ -5587,16 +5579,16 @@
         <v>26.1</v>
       </c>
       <c r="F14" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G14" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I14" s="25" t="n">
-        <v>184.07</v>
+        <v>184.17</v>
       </c>
       <c r="J14" s="26">
         <f>F14-H14</f>
@@ -5654,16 +5646,16 @@
         <v>9.43</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G15" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H15" s="25" t="n">
-        <v>184.07</v>
+        <v>184.17</v>
       </c>
       <c r="I15" s="25" t="n">
-        <v>184.022</v>
+        <v>184.122</v>
       </c>
       <c r="J15" s="26">
         <f>F15-H15</f>
@@ -5721,16 +5713,16 @@
         <v>3.78</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G16" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H16" s="25" t="n">
-        <v>184.022</v>
+        <v>184.122</v>
       </c>
       <c r="I16" s="25" t="n">
-        <v>184.003</v>
+        <v>184.103</v>
       </c>
       <c r="J16" s="26">
         <f>F16-H16</f>
@@ -5788,16 +5780,16 @@
         <v>15.97</v>
       </c>
       <c r="F17" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G17" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H17" s="25" t="n">
-        <v>184.003</v>
+        <v>184.103</v>
       </c>
       <c r="I17" s="25" t="n">
-        <v>183.924</v>
+        <v>184.024</v>
       </c>
       <c r="J17" s="26">
         <f>F17-H17</f>
@@ -5855,16 +5847,16 @@
         <v>6.79</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G18" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H18" s="25" t="n">
-        <v>183.924</v>
+        <v>184.024</v>
       </c>
       <c r="I18" s="25" t="n">
-        <v>183.89</v>
+        <v>183.99</v>
       </c>
       <c r="J18" s="26">
         <f>F18-H18</f>
@@ -5922,16 +5914,16 @@
         <v>32.81</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G19" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H19" s="25" t="n">
-        <v>183.89</v>
+        <v>183.99</v>
       </c>
       <c r="I19" s="25" t="n">
-        <v>183.726</v>
+        <v>183.826</v>
       </c>
       <c r="J19" s="26">
         <f>F19-H19</f>
@@ -5989,16 +5981,16 @@
         <v>21.32</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G20" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H20" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I20" s="25" t="n">
-        <v>184.093</v>
+        <v>184.193</v>
       </c>
       <c r="J20" s="26">
         <f>F20-H20</f>
@@ -6056,16 +6048,16 @@
         <v>5.89</v>
       </c>
       <c r="F21" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G21" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H21" s="25" t="n">
-        <v>184.093</v>
+        <v>184.193</v>
       </c>
       <c r="I21" s="25" t="n">
-        <v>184.064</v>
+        <v>184.164</v>
       </c>
       <c r="J21" s="26">
         <f>F21-H21</f>
@@ -6123,16 +6115,16 @@
         <v>17.83</v>
       </c>
       <c r="F22" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G22" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H22" s="25" t="n">
-        <v>184.064</v>
+        <v>184.164</v>
       </c>
       <c r="I22" s="25" t="n">
-        <v>183.975</v>
+        <v>184.075</v>
       </c>
       <c r="J22" s="26">
         <f>F22-H22</f>
@@ -6190,16 +6182,16 @@
         <v>5.77</v>
       </c>
       <c r="F23" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G23" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>183.975</v>
+        <v>184.075</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>183.946</v>
+        <v>184.046</v>
       </c>
       <c r="J23" s="26">
         <f>F23-H23</f>
@@ -6257,16 +6249,16 @@
         <v>39.15</v>
       </c>
       <c r="F24" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G24" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H24" s="25" t="n">
-        <v>183.946</v>
+        <v>184.046</v>
       </c>
       <c r="I24" s="25" t="n">
-        <v>183.75</v>
+        <v>183.85</v>
       </c>
       <c r="J24" s="26">
         <f>F24-H24</f>
@@ -6324,16 +6316,16 @@
         <v>11.74</v>
       </c>
       <c r="F25" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G25" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H25" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I25" s="25" t="n">
-        <v>184.141</v>
+        <v>184.241</v>
       </c>
       <c r="J25" s="26">
         <f>F25-H25</f>
@@ -6391,16 +6383,16 @@
         <v>11.51</v>
       </c>
       <c r="F26" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G26" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H26" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I26" s="25" t="n">
-        <v>184.002</v>
+        <v>184.102</v>
       </c>
       <c r="J26" s="26">
         <f>F26-H26</f>
@@ -6458,16 +6450,16 @@
         <v>17.85</v>
       </c>
       <c r="F27" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G27" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H27" s="25" t="n">
-        <v>184.002</v>
+        <v>184.102</v>
       </c>
       <c r="I27" s="25" t="n">
-        <v>183.912</v>
+        <v>184.012</v>
       </c>
       <c r="J27" s="26">
         <f>F27-H27</f>
@@ -6525,16 +6517,16 @@
         <v>6.12</v>
       </c>
       <c r="F28" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G28" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H28" s="25" t="n">
-        <v>183.912</v>
+        <v>184.012</v>
       </c>
       <c r="I28" s="25" t="n">
-        <v>183.882</v>
+        <v>183.982</v>
       </c>
       <c r="J28" s="26">
         <f>F28-H28</f>
@@ -6592,16 +6584,16 @@
         <v>22.77</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G29" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H29" s="25" t="n">
-        <v>183.882</v>
+        <v>183.982</v>
       </c>
       <c r="I29" s="25" t="n">
-        <v>183.768</v>
+        <v>183.868</v>
       </c>
       <c r="J29" s="26">
         <f>F29-H29</f>
@@ -6659,16 +6651,16 @@
         <v>11.77</v>
       </c>
       <c r="F30" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G30" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H30" s="25" t="n">
-        <v>183.768</v>
+        <v>183.868</v>
       </c>
       <c r="I30" s="25" t="n">
-        <v>183.709</v>
+        <v>183.809</v>
       </c>
       <c r="J30" s="26">
         <f>F30-H30</f>
@@ -6726,16 +6718,16 @@
         <v>3.07</v>
       </c>
       <c r="F31" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G31" s="24" t="n">
-        <v>184.412</v>
+        <v>184.6</v>
       </c>
       <c r="H31" s="25" t="n">
-        <v>183.709</v>
+        <v>183.809</v>
       </c>
       <c r="I31" s="25" t="n">
-        <v>183.694</v>
+        <v>183.794</v>
       </c>
       <c r="J31" s="26">
         <f>F31-H31</f>
@@ -6793,16 +6785,16 @@
         <v>7.96</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>184.412</v>
+        <v>184.6</v>
       </c>
       <c r="G32" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H32" s="25" t="n">
-        <v>183.694</v>
+        <v>183.794</v>
       </c>
       <c r="I32" s="25" t="n">
-        <v>183.654</v>
+        <v>183.754</v>
       </c>
       <c r="J32" s="26">
         <f>F32-H32</f>
@@ -6860,16 +6852,16 @@
         <v>6.69</v>
       </c>
       <c r="F33" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G33" s="24" t="n">
-        <v>183.852</v>
+        <v>184.6</v>
       </c>
       <c r="H33" s="25" t="n">
-        <v>183.654</v>
+        <v>183.754</v>
       </c>
       <c r="I33" s="25" t="n">
-        <v>183.578</v>
+        <v>183.72</v>
       </c>
       <c r="J33" s="26">
         <f>F33-H33</f>
@@ -6927,16 +6919,16 @@
         <v>8.210000000000001</v>
       </c>
       <c r="F34" s="24" t="n">
-        <v>183.852</v>
+        <v>184.6</v>
       </c>
       <c r="G34" s="24" t="n">
-        <v>184.023</v>
+        <v>184.6</v>
       </c>
       <c r="H34" s="25" t="n">
-        <v>183.578</v>
+        <v>183.72</v>
       </c>
       <c r="I34" s="25" t="n">
-        <v>183.485</v>
+        <v>183.679</v>
       </c>
       <c r="J34" s="26">
         <f>F34-H34</f>
@@ -6994,16 +6986,16 @@
         <v>0.6</v>
       </c>
       <c r="F35" s="24" t="n">
-        <v>184.023</v>
+        <v>184.6</v>
       </c>
       <c r="G35" s="24" t="n">
         <v>183.826</v>
       </c>
       <c r="H35" s="25" t="n">
-        <v>183.485</v>
+        <v>183.679</v>
       </c>
       <c r="I35" s="25" t="n">
-        <v>183.482</v>
+        <v>183.576</v>
       </c>
       <c r="J35" s="26">
         <f>F35-H35</f>
@@ -7061,16 +7053,16 @@
         <v>3.88</v>
       </c>
       <c r="F36" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G36" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H36" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I36" s="25" t="n">
-        <v>184.181</v>
+        <v>184.281</v>
       </c>
       <c r="J36" s="26">
         <f>F36-H36</f>
@@ -7128,16 +7120,16 @@
         <v>35.8</v>
       </c>
       <c r="F37" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G37" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H37" s="25" t="n">
-        <v>184.181</v>
+        <v>184.281</v>
       </c>
       <c r="I37" s="25" t="n">
-        <v>184.002</v>
+        <v>184.102</v>
       </c>
       <c r="J37" s="26">
         <f>F37-H37</f>
@@ -7195,16 +7187,16 @@
         <v>35.8</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G38" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H38" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I38" s="25" t="n">
-        <v>184.021</v>
+        <v>184.121</v>
       </c>
       <c r="J38" s="26">
         <f>F38-H38</f>
@@ -7262,16 +7254,16 @@
         <v>17.85</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G39" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H39" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I39" s="25" t="n">
-        <v>184.111</v>
+        <v>184.211</v>
       </c>
       <c r="J39" s="26">
         <f>F39-H39</f>
@@ -7329,16 +7321,16 @@
         <v>6.12</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G40" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H40" s="25" t="n">
-        <v>184.111</v>
+        <v>184.211</v>
       </c>
       <c r="I40" s="25" t="n">
-        <v>184.08</v>
+        <v>184.18</v>
       </c>
       <c r="J40" s="26">
         <f>F40-H40</f>
@@ -7396,16 +7388,16 @@
         <v>13.03</v>
       </c>
       <c r="F41" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G41" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H41" s="25" t="n">
-        <v>184.08</v>
+        <v>184.18</v>
       </c>
       <c r="I41" s="25" t="n">
-        <v>184.015</v>
+        <v>184.115</v>
       </c>
       <c r="J41" s="26">
         <f>F41-H41</f>
@@ -7463,16 +7455,16 @@
         <v>30.36</v>
       </c>
       <c r="F42" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G42" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H42" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I42" s="25" t="n">
-        <v>184.048</v>
+        <v>184.148</v>
       </c>
       <c r="J42" s="26">
         <f>F42-H42</f>
@@ -7530,16 +7522,16 @@
         <v>15.66</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G43" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H43" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I43" s="25" t="n">
-        <v>184.122</v>
+        <v>184.222</v>
       </c>
       <c r="J43" s="26">
         <f>F43-H43</f>
@@ -7597,16 +7589,16 @@
         <v>23.7</v>
       </c>
       <c r="F44" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G44" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H44" s="25" t="n">
-        <v>184.122</v>
+        <v>184.222</v>
       </c>
       <c r="I44" s="25" t="n">
-        <v>184.003</v>
+        <v>184.103</v>
       </c>
       <c r="J44" s="26">
         <f>F44-H44</f>
@@ -7664,16 +7656,16 @@
         <v>35.28</v>
       </c>
       <c r="F45" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G45" s="24" t="n">
         <v>184.5</v>
       </c>
       <c r="H45" s="25" t="n">
-        <v>184.003</v>
+        <v>184.103</v>
       </c>
       <c r="I45" s="25" t="n">
-        <v>183.827</v>
+        <v>183.927</v>
       </c>
       <c r="J45" s="26">
         <f>F45-H45</f>
@@ -7737,10 +7729,10 @@
         <v>184.5</v>
       </c>
       <c r="H46" s="25" t="n">
-        <v>183.827</v>
+        <v>183.927</v>
       </c>
       <c r="I46" s="25" t="n">
-        <v>183.783</v>
+        <v>183.883</v>
       </c>
       <c r="J46" s="26">
         <f>F46-H46</f>
@@ -7801,13 +7793,13 @@
         <v>184.5</v>
       </c>
       <c r="G47" s="24" t="n">
-        <v>181.8</v>
+        <v>184.5</v>
       </c>
       <c r="H47" s="25" t="n">
-        <v>183.783</v>
+        <v>183.883</v>
       </c>
       <c r="I47" s="25" t="n">
-        <v>181.55</v>
+        <v>183.824</v>
       </c>
       <c r="J47" s="26">
         <f>F47-H47</f>
@@ -7865,16 +7857,16 @@
         <v>8.630000000000001</v>
       </c>
       <c r="F48" s="24" t="n">
-        <v>181.8</v>
+        <v>184.5</v>
       </c>
       <c r="G48" s="24" t="n">
-        <v>181.418</v>
+        <v>184.5</v>
       </c>
       <c r="H48" s="25" t="n">
-        <v>181.55</v>
+        <v>183.824</v>
       </c>
       <c r="I48" s="25" t="n">
-        <v>181.117</v>
+        <v>183.781</v>
       </c>
       <c r="J48" s="26">
         <f>F48-H48</f>
@@ -7932,16 +7924,16 @@
         <v>12.29</v>
       </c>
       <c r="F49" s="24" t="n">
-        <v>181.418</v>
+        <v>184.5</v>
       </c>
       <c r="G49" s="24" t="n">
-        <v>180.523</v>
+        <v>184.5</v>
       </c>
       <c r="H49" s="25" t="n">
-        <v>181.117</v>
+        <v>183.781</v>
       </c>
       <c r="I49" s="25" t="n">
-        <v>180.266</v>
+        <v>183.719</v>
       </c>
       <c r="J49" s="26">
         <f>F49-H49</f>
@@ -7999,16 +7991,16 @@
         <v>2.5</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>180.523</v>
+        <v>184.5</v>
       </c>
       <c r="G50" s="24" t="n">
-        <v>180.623</v>
+        <v>184.5</v>
       </c>
       <c r="H50" s="25" t="n">
-        <v>180.266</v>
+        <v>183.719</v>
       </c>
       <c r="I50" s="25" t="n">
-        <v>180.224</v>
+        <v>183.707</v>
       </c>
       <c r="J50" s="26">
         <f>F50-H50</f>
@@ -8066,16 +8058,16 @@
         <v>0.6</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>180.623</v>
+        <v>184.5</v>
       </c>
       <c r="G51" s="24" t="n">
-        <v>180.553</v>
+        <v>184.5</v>
       </c>
       <c r="H51" s="25" t="n">
-        <v>180.224</v>
+        <v>183.707</v>
       </c>
       <c r="I51" s="25" t="n">
-        <v>180.154</v>
+        <v>183.704</v>
       </c>
       <c r="J51" s="26">
         <f>F51-H51</f>
@@ -8200,16 +8192,16 @@
         <v>17.06</v>
       </c>
       <c r="F53" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G53" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H53" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I53" s="25" t="n">
-        <v>184.115</v>
+        <v>184.215</v>
       </c>
       <c r="J53" s="26">
         <f>F53-H53</f>
@@ -8267,16 +8259,16 @@
         <v>22.85</v>
       </c>
       <c r="F54" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G54" s="24" t="n">
         <v>184.5</v>
       </c>
       <c r="H54" s="25" t="n">
-        <v>184.115</v>
+        <v>184.215</v>
       </c>
       <c r="I54" s="25" t="n">
-        <v>184</v>
+        <v>184.1</v>
       </c>
       <c r="J54" s="26">
         <f>F54-H54</f>
@@ -8340,10 +8332,10 @@
         <v>184.5</v>
       </c>
       <c r="H55" s="25" t="n">
-        <v>184</v>
+        <v>184.1</v>
       </c>
       <c r="I55" s="25" t="n">
-        <v>183.995</v>
+        <v>184.095</v>
       </c>
       <c r="J55" s="26">
         <f>F55-H55</f>
@@ -8407,10 +8399,10 @@
         <v>184.5</v>
       </c>
       <c r="H56" s="25" t="n">
-        <v>183.995</v>
+        <v>184.095</v>
       </c>
       <c r="I56" s="25" t="n">
-        <v>183.898</v>
+        <v>183.998</v>
       </c>
       <c r="J56" s="26">
         <f>F56-H56</f>
@@ -8474,10 +8466,10 @@
         <v>184.5</v>
       </c>
       <c r="H57" s="25" t="n">
-        <v>183.898</v>
+        <v>183.998</v>
       </c>
       <c r="I57" s="25" t="n">
-        <v>183.872</v>
+        <v>183.972</v>
       </c>
       <c r="J57" s="26">
         <f>F57-H57</f>
@@ -8535,16 +8527,16 @@
         <v>13.05</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G58" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H58" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I58" s="25" t="n">
-        <v>184.135</v>
+        <v>184.235</v>
       </c>
       <c r="J58" s="26">
         <f>F58-H58</f>
@@ -8602,16 +8594,16 @@
         <v>23.58</v>
       </c>
       <c r="F59" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G59" s="24" t="n">
         <v>184.5</v>
       </c>
       <c r="H59" s="25" t="n">
-        <v>184.135</v>
+        <v>184.235</v>
       </c>
       <c r="I59" s="25" t="n">
-        <v>184.017</v>
+        <v>184.117</v>
       </c>
       <c r="J59" s="26">
         <f>F59-H59</f>
@@ -8672,13 +8664,13 @@
         <v>184.5</v>
       </c>
       <c r="G60" s="24" t="n">
-        <v>181.8</v>
+        <v>184.5</v>
       </c>
       <c r="H60" s="25" t="n">
-        <v>184.017</v>
+        <v>184.117</v>
       </c>
       <c r="I60" s="25" t="n">
-        <v>181.55</v>
+        <v>184.091</v>
       </c>
       <c r="J60" s="26">
         <f>F60-H60</f>
@@ -8736,16 +8728,16 @@
         <v>31.2</v>
       </c>
       <c r="F61" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G61" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H61" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I61" s="25" t="n">
-        <v>184.044</v>
+        <v>184.144</v>
       </c>
       <c r="J61" s="26">
         <f>F61-H61</f>
@@ -8803,16 +8795,16 @@
         <v>3.93</v>
       </c>
       <c r="F62" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G62" s="24" t="n">
-        <v>183.86</v>
+        <v>184.6</v>
       </c>
       <c r="H62" s="25" t="n">
-        <v>184.044</v>
+        <v>184.144</v>
       </c>
       <c r="I62" s="25" t="n">
-        <v>183.61</v>
+        <v>184.124</v>
       </c>
       <c r="J62" s="26">
         <f>F62-H62</f>
@@ -8870,16 +8862,16 @@
         <v>14.9</v>
       </c>
       <c r="F63" s="24" t="n">
-        <v>183.86</v>
+        <v>184.6</v>
       </c>
       <c r="G63" s="24" t="n">
-        <v>180.623</v>
+        <v>184.5</v>
       </c>
       <c r="H63" s="25" t="n">
-        <v>183.61</v>
+        <v>184.124</v>
       </c>
       <c r="I63" s="25" t="n">
-        <v>180.373</v>
+        <v>184.05</v>
       </c>
       <c r="J63" s="26">
         <f>F63-H63</f>
@@ -8937,16 +8929,16 @@
         <v>39.03</v>
       </c>
       <c r="F64" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G64" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H64" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I64" s="25" t="n">
-        <v>184.004</v>
+        <v>184.104</v>
       </c>
       <c r="J64" s="26">
         <f>F64-H64</f>
@@ -9004,16 +8996,16 @@
         <v>0.5</v>
       </c>
       <c r="F65" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G65" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H65" s="25" t="n">
-        <v>184.004</v>
+        <v>184.104</v>
       </c>
       <c r="I65" s="25" t="n">
-        <v>184.002</v>
+        <v>184.102</v>
       </c>
       <c r="J65" s="26">
         <f>F65-H65</f>
@@ -9071,16 +9063,16 @@
         <v>0.6</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G66" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H66" s="25" t="n">
-        <v>184.002</v>
+        <v>184.102</v>
       </c>
       <c r="I66" s="25" t="n">
-        <v>183.999</v>
+        <v>184.099</v>
       </c>
       <c r="J66" s="26">
         <f>F66-H66</f>
@@ -9138,16 +9130,16 @@
         <v>11.75</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G67" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H67" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I67" s="25" t="n">
-        <v>184.141</v>
+        <v>184.241</v>
       </c>
       <c r="J67" s="26">
         <f>F67-H67</f>
@@ -9205,16 +9197,16 @@
         <v>25.47</v>
       </c>
       <c r="F68" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G68" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H68" s="25" t="n">
-        <v>184.141</v>
+        <v>184.241</v>
       </c>
       <c r="I68" s="25" t="n">
-        <v>184.014</v>
+        <v>184.114</v>
       </c>
       <c r="J68" s="26">
         <f>F68-H68</f>
@@ -9272,16 +9264,16 @@
         <v>1.91</v>
       </c>
       <c r="F69" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G69" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H69" s="25" t="n">
-        <v>184.014</v>
+        <v>184.114</v>
       </c>
       <c r="I69" s="25" t="n">
-        <v>184.004</v>
+        <v>184.104</v>
       </c>
       <c r="J69" s="26">
         <f>F69-H69</f>
@@ -9339,16 +9331,16 @@
         <v>13.84</v>
       </c>
       <c r="F70" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="G70" s="24" t="n">
-        <v>184.5</v>
+        <v>184.6</v>
       </c>
       <c r="H70" s="25" t="n">
-        <v>184.2</v>
+        <v>184.3</v>
       </c>
       <c r="I70" s="25" t="n">
-        <v>184.131</v>
+        <v>184.231</v>
       </c>
       <c r="J70" s="26">
         <f>F70-H70</f>
@@ -10689,7 +10681,7 @@
       </c>
       <c r="E68" s="30" t="inlineStr">
         <is>
-          <t>Cerco norte (x = 965.5): poza de salida que rebalsa a nivel del fondo de la hondonada natural (baja a la quebrada del norte)</t>
+          <t>Cerco norte (x = 965.5): pase en el cimiento del cerco al terreno exterior que baja a la quebrada del norte</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Barranquita: avisos de seccion por linea y vistas previas de las 21 laminas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -10946,7 +10946,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Llega EJE-02</t>
+          <t>Inicio de tapado; Llega EJE-02</t>
         </is>
       </c>
     </row>
@@ -12175,7 +12175,11 @@
           <t>TAPADA</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Inicio de tapado</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -13043,7 +13047,7 @@
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>Llega EJE-13</t>
+          <t>Llega EJE-13; Cambio de borde</t>
         </is>
       </c>
     </row>
@@ -13164,7 +13168,11 @@
           <t>TAPADA</t>
         </is>
       </c>
-      <c r="J63" s="4" t="inlineStr"/>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>Inicio de tapado</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -14354,7 +14362,11 @@
           <t>TAPADA</t>
         </is>
       </c>
-      <c r="J93" s="4" t="inlineStr"/>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>Inicio de tapado</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Barranquita: todo a escala real, planta con rejilla/tapado del usuario y tapas de inspeccion
- planta_cunetas_b (nuevo): bordes 0.60/0.40 a escala real, rejilla celeste con platinas,
  tapado en verde, flechas rojas y tapas de inspeccion 0.60 x 0.60 (inicio, fin, empalmes, max 10 m).
- descargas_b: planta e isometrico a escala real (lamina 1/25) con el mismo estilo de planta.
- Se quitan los isometricos de toda la red; laminas renumeradas DC-15 a DC-19.
- Perfiles: titulo sin coordenadas con progresivas; longitud y pendiente completas entre secciones.
- Excel: hoja TAPAS INSPECCION.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRAMOS" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NUDOS" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SECCIONES" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAPAS INSPECCION" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -791,7 +792,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>7. Ver planos PLANTEAMIENTO_CUNETAS_IE0590_BARRANQUITA.dxf: DC-01 planta general de cunetas - planteamiento preliminar; DC-02 cuadro de tramos y secciones tipicas de cuneta; DC-03 a DC-11 perfiles longitudinales de cunetas por eje; DC-12 a DC-14 secciones transversales de cunetas; DC-15 isometrico de la red - vista desde el sur; DC-16 isometrico de la red - vista desde el norte; DC-17 cortes generales del terreno y la red; DC-18 detalle de la descarga d1 por el cerco; DC-19 detalle de la descarga d2 por el cerco; DC-20 detalle de la descarga d3 por el cerco; DC-21 detalle de la descarga d4 por el cerco.</t>
+          <t>7. Ver planos PLANTEAMIENTO_CUNETAS_IE0590_BARRANQUITA.dxf: DC-01 planta general de cunetas - planteamiento preliminar; DC-02 cuadro de tramos y secciones tipicas de cuneta; DC-03 a DC-11 perfiles longitudinales de cunetas por eje; DC-12 a DC-14 secciones transversales de cunetas; DC-15 cortes generales del terreno y la red; DC-16 detalle de la descarga d1 por el cerco; DC-17 detalle de la descarga d2 por el cerco; DC-18 detalle de la descarga d3 por el cerco; DC-19 detalle de la descarga d4 por el cerco.</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6234,7 @@
       </c>
       <c r="Q5" s="27" t="inlineStr">
         <is>
-          <t>Pabellon oeste A: lado nor-oeste; entrega al EJE-02 junto al cerco (caida)</t>
+          <t>Pabellon oeste A: lado nor-oeste; entrega al EJE-02 junto al cerco</t>
         </is>
       </c>
     </row>
@@ -6300,7 +6301,7 @@
       </c>
       <c r="Q6" s="27" t="inlineStr">
         <is>
-          <t>Pabellon oeste A: lado nor-oeste; entrega al EJE-02 junto al cerco (caida)</t>
+          <t>Pabellon oeste A: lado nor-oeste; entrega al EJE-02 junto al cerco</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7038,7 @@
       </c>
       <c r="Q17" s="27" t="inlineStr">
         <is>
-          <t>Bloque x=884.9 (lado oeste), bloque D (lado norte) y pabellon C (lado nor-este)</t>
+          <t>Bloque D (lado norte) y pabellon C (lado nor-este)</t>
         </is>
       </c>
     </row>
@@ -7104,7 +7105,7 @@
       </c>
       <c r="Q18" s="27" t="inlineStr">
         <is>
-          <t>Bloque x=884.9 (lado oeste), bloque D (lado norte) y pabellon C (lado nor-este)</t>
+          <t>Bloque D (lado norte) y pabellon C (lado nor-este)</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7172,7 @@
       </c>
       <c r="Q19" s="27" t="inlineStr">
         <is>
-          <t>Bloque x=884.9 (lado oeste), bloque D (lado norte) y pabellon C (lado nor-este)</t>
+          <t>Bloque D (lado norte) y pabellon C (lado nor-este)</t>
         </is>
       </c>
     </row>
@@ -7238,7 +7239,7 @@
       </c>
       <c r="Q20" s="27" t="inlineStr">
         <is>
-          <t>Bloque x=884.9 (lado oeste), bloque D (lado norte) y pabellon C (lado nor-este)</t>
+          <t>Bloque D (lado norte) y pabellon C (lado nor-este)</t>
         </is>
       </c>
     </row>
@@ -7305,7 +7306,7 @@
       </c>
       <c r="Q21" s="27" t="inlineStr">
         <is>
-          <t>Bloque x=884.9 (lado oeste), bloque D (lado norte) y pabellon C (lado nor-este)</t>
+          <t>Bloque D (lado norte) y pabellon C (lado nor-este)</t>
         </is>
       </c>
     </row>
@@ -7372,7 +7373,7 @@
       </c>
       <c r="Q22" s="27" t="inlineStr">
         <is>
-          <t>Bloque x=884.9 (lado oeste), bloque D (lado norte) y pabellon C (lado nor-este)</t>
+          <t>Bloque D (lado norte) y pabellon C (lado nor-este)</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7440,7 @@
       </c>
       <c r="Q23" s="27" t="inlineStr">
         <is>
-          <t>Bloque x=884.9 (lado oeste), bloque D (lado norte) y pabellon C (lado nor-este)</t>
+          <t>Bloque D (lado norte) y pabellon C (lado nor-este)</t>
         </is>
       </c>
     </row>
@@ -7841,7 +7842,7 @@
       </c>
       <c r="Q29" s="27" t="inlineStr">
         <is>
-          <t>Bloque del ingreso: lado norte (y=815.97) al oeste de x=896.8</t>
+          <t>Bloque del ingreso: lado norte, tramo oeste</t>
         </is>
       </c>
     </row>
@@ -7908,7 +7909,7 @@
       </c>
       <c r="Q30" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -7975,7 +7976,7 @@
       </c>
       <c r="Q31" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8042,7 +8043,7 @@
       </c>
       <c r="Q32" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8109,7 +8110,7 @@
       </c>
       <c r="Q33" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8176,7 +8177,7 @@
       </c>
       <c r="Q34" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8243,7 +8244,7 @@
       </c>
       <c r="Q35" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8311,7 @@
       </c>
       <c r="Q36" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8377,7 +8378,7 @@
       </c>
       <c r="Q37" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8444,7 +8445,7 @@
       </c>
       <c r="Q38" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8511,7 +8512,7 @@
       </c>
       <c r="Q39" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8578,7 +8579,7 @@
       </c>
       <c r="Q40" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8645,7 +8646,7 @@
       </c>
       <c r="Q41" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8712,7 +8713,7 @@
       </c>
       <c r="Q42" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8779,7 +8780,7 @@
       </c>
       <c r="Q43" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8846,7 +8847,7 @@
       </c>
       <c r="Q44" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8913,7 +8914,7 @@
       </c>
       <c r="Q45" s="27" t="inlineStr">
         <is>
-          <t>Patio central (x=896.8), y=815.97, bajada x=919.6 y atrio de ingreso a D3</t>
+          <t>Patio central, bajada al atrio de ingreso y salida D3</t>
         </is>
       </c>
     </row>
@@ -8980,7 +8981,7 @@
       </c>
       <c r="Q46" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado sur (y=839.94)</t>
+          <t>Bloque del centro: lado sur</t>
         </is>
       </c>
     </row>
@@ -9047,7 +9048,7 @@
       </c>
       <c r="Q47" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado sur (y=839.94)</t>
+          <t>Bloque del centro: lado sur</t>
         </is>
       </c>
     </row>
@@ -9114,7 +9115,7 @@
       </c>
       <c r="Q48" s="27" t="inlineStr">
         <is>
-          <t>Patio central: y=822.09</t>
+          <t>Patio central</t>
         </is>
       </c>
     </row>
@@ -9181,7 +9182,7 @@
       </c>
       <c r="Q49" s="27" t="inlineStr">
         <is>
-          <t>x=932.6 y bloque del frente: lado norte (y=815.97)</t>
+          <t>Bloque del frente: lado norte</t>
         </is>
       </c>
     </row>
@@ -9248,7 +9249,7 @@
       </c>
       <c r="Q50" s="27" t="inlineStr">
         <is>
-          <t>x=932.6 y bloque del frente: lado norte (y=815.97)</t>
+          <t>Bloque del frente: lado norte</t>
         </is>
       </c>
     </row>
@@ -9315,7 +9316,7 @@
       </c>
       <c r="Q51" s="27" t="inlineStr">
         <is>
-          <t>x=932.6 y bloque del frente: lado norte (y=815.97)</t>
+          <t>Bloque del frente: lado norte</t>
         </is>
       </c>
     </row>
@@ -9382,7 +9383,7 @@
       </c>
       <c r="Q52" s="27" t="inlineStr">
         <is>
-          <t>x=932.6 y bloque del frente: lado norte (y=815.97)</t>
+          <t>Bloque del frente: lado norte</t>
         </is>
       </c>
     </row>
@@ -9449,7 +9450,7 @@
       </c>
       <c r="Q53" s="27" t="inlineStr">
         <is>
-          <t>x=932.6 y bloque del frente: lado norte (y=815.97)</t>
+          <t>Bloque del frente: lado norte</t>
         </is>
       </c>
     </row>
@@ -9516,7 +9517,7 @@
       </c>
       <c r="Q54" s="27" t="inlineStr">
         <is>
-          <t>Bloque del frente: lado sur (y=804.1)</t>
+          <t>Bloque del frente: lado sur</t>
         </is>
       </c>
     </row>
@@ -10387,7 +10388,7 @@
       </c>
       <c r="Q67" s="27" t="inlineStr">
         <is>
-          <t>Losa: lado norte (y=831.3)</t>
+          <t>Losa: lado norte</t>
         </is>
       </c>
     </row>
@@ -10454,7 +10455,7 @@
       </c>
       <c r="Q68" s="27" t="inlineStr">
         <is>
-          <t>y=815.97, x=952.3 y bloque nor-este: lado sur (y=839.9)</t>
+          <t>Bloque nor-este: lado sur</t>
         </is>
       </c>
     </row>
@@ -10521,7 +10522,7 @@
       </c>
       <c r="Q69" s="27" t="inlineStr">
         <is>
-          <t>y=815.97, x=952.3 y bloque nor-este: lado sur (y=839.9)</t>
+          <t>Bloque nor-este: lado sur</t>
         </is>
       </c>
     </row>
@@ -10588,7 +10589,7 @@
       </c>
       <c r="Q70" s="27" t="inlineStr">
         <is>
-          <t>y=815.97, x=952.3 y bloque nor-este: lado sur (y=839.9)</t>
+          <t>Bloque nor-este: lado sur</t>
         </is>
       </c>
     </row>
@@ -10655,7 +10656,7 @@
       </c>
       <c r="Q71" s="27" t="inlineStr">
         <is>
-          <t>y=815.97, x=952.3 y bloque nor-este: lado sur (y=839.9)</t>
+          <t>Bloque nor-este: lado sur</t>
         </is>
       </c>
     </row>
@@ -10722,7 +10723,7 @@
       </c>
       <c r="Q72" s="27" t="inlineStr">
         <is>
-          <t>y=815.97, x=952.3 y bloque nor-este: lado sur (y=839.9)</t>
+          <t>Bloque nor-este: lado sur</t>
         </is>
       </c>
     </row>
@@ -10789,7 +10790,7 @@
       </c>
       <c r="Q73" s="27" t="inlineStr">
         <is>
-          <t>y=815.97, x=952.3 y bloque nor-este: lado sur (y=839.9)</t>
+          <t>Bloque nor-este: lado sur</t>
         </is>
       </c>
     </row>
@@ -10856,7 +10857,7 @@
       </c>
       <c r="Q74" s="27" t="inlineStr">
         <is>
-          <t>y=815.97, x=952.3 y bloque nor-este: lado sur (y=839.9)</t>
+          <t>Bloque nor-este: lado sur</t>
         </is>
       </c>
     </row>
@@ -10923,7 +10924,7 @@
       </c>
       <c r="Q75" s="27" t="inlineStr">
         <is>
-          <t>Bloque nor-este: lado oeste (x=948.1) y lado norte (y=851.9)</t>
+          <t>Bloque nor-este: lados oeste y norte</t>
         </is>
       </c>
     </row>
@@ -10990,7 +10991,7 @@
       </c>
       <c r="Q76" s="27" t="inlineStr">
         <is>
-          <t>Bloque nor-este: lado oeste (x=948.1) y lado norte (y=851.9)</t>
+          <t>Bloque nor-este: lados oeste y norte</t>
         </is>
       </c>
     </row>
@@ -11057,7 +11058,7 @@
       </c>
       <c r="Q77" s="27" t="inlineStr">
         <is>
-          <t>Bloque nor-este: lado oeste (x=948.1) y lado norte (y=851.9)</t>
+          <t>Bloque nor-este: lados oeste y norte</t>
         </is>
       </c>
     </row>
@@ -11124,7 +11125,7 @@
       </c>
       <c r="Q78" s="27" t="inlineStr">
         <is>
-          <t>Bloque nor-este: lado oeste (x=948.1) y lado norte (y=851.9)</t>
+          <t>Bloque nor-este: lados oeste y norte</t>
         </is>
       </c>
     </row>
@@ -11191,7 +11192,7 @@
       </c>
       <c r="Q79" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado norte (y=865.1) y union a D2 por el norte de la planta de tratamiento</t>
+          <t>Bloque norte: lado norte y union a D2 por el norte de la planta de tratamiento</t>
         </is>
       </c>
     </row>
@@ -11258,7 +11259,7 @@
       </c>
       <c r="Q80" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado norte (y=865.1) y union a D2 por el norte de la planta de tratamiento</t>
+          <t>Bloque norte: lado norte y union a D2 por el norte de la planta de tratamiento</t>
         </is>
       </c>
     </row>
@@ -11325,7 +11326,7 @@
       </c>
       <c r="Q81" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado norte (y=865.1) y union a D2 por el norte de la planta de tratamiento</t>
+          <t>Bloque norte: lado norte y union a D2 por el norte de la planta de tratamiento</t>
         </is>
       </c>
     </row>
@@ -11392,7 +11393,7 @@
       </c>
       <c r="Q82" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado norte (y=865.1) y union a D2 por el norte de la planta de tratamiento</t>
+          <t>Bloque norte: lado norte y union a D2 por el norte de la planta de tratamiento</t>
         </is>
       </c>
     </row>
@@ -11459,7 +11460,7 @@
       </c>
       <c r="Q83" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado norte (y=865.1) y union a D2 por el norte de la planta de tratamiento</t>
+          <t>Bloque norte: lado norte y union a D2 por el norte de la planta de tratamiento</t>
         </is>
       </c>
     </row>
@@ -11526,7 +11527,7 @@
       </c>
       <c r="Q84" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado norte (y=865.1) y union a D2 por el norte de la planta de tratamiento</t>
+          <t>Bloque norte: lado norte y union a D2 por el norte de la planta de tratamiento</t>
         </is>
       </c>
     </row>
@@ -11593,7 +11594,7 @@
       </c>
       <c r="Q85" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado sur (y=853.5) y salida D4</t>
+          <t>Bloque norte: lado sur y salida D4</t>
         </is>
       </c>
     </row>
@@ -11660,7 +11661,7 @@
       </c>
       <c r="Q86" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado sur (y=853.5) y salida D4</t>
+          <t>Bloque norte: lado sur y salida D4</t>
         </is>
       </c>
     </row>
@@ -11727,7 +11728,7 @@
       </c>
       <c r="Q87" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado sur (y=853.5) y salida D4</t>
+          <t>Bloque norte: lado sur y salida D4</t>
         </is>
       </c>
     </row>
@@ -11794,7 +11795,7 @@
       </c>
       <c r="Q88" s="27" t="inlineStr">
         <is>
-          <t>Bloque norte: lado sur (y=853.5) y salida D4</t>
+          <t>Bloque norte: lado sur y salida D4</t>
         </is>
       </c>
     </row>
@@ -11861,7 +11862,7 @@
       </c>
       <c r="Q89" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado este (x=936.5) y lado norte (y=851.7), tramo este</t>
+          <t>Bloque del centro: lados este y norte, tramo este</t>
         </is>
       </c>
     </row>
@@ -11928,7 +11929,7 @@
       </c>
       <c r="Q90" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado este (x=936.5) y lado norte (y=851.7), tramo este</t>
+          <t>Bloque del centro: lados este y norte, tramo este</t>
         </is>
       </c>
     </row>
@@ -11995,7 +11996,7 @@
       </c>
       <c r="Q91" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado este (x=936.5) y lado norte (y=851.7), tramo este</t>
+          <t>Bloque del centro: lados este y norte, tramo este</t>
         </is>
       </c>
     </row>
@@ -12062,7 +12063,7 @@
       </c>
       <c r="Q92" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado este (x=936.5) y lado norte (y=851.7), tramo este</t>
+          <t>Bloque del centro: lados este y norte, tramo este</t>
         </is>
       </c>
     </row>
@@ -12129,7 +12130,7 @@
       </c>
       <c r="Q93" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado este (x=936.5) y lado norte (y=851.7), tramo este</t>
+          <t>Bloque del centro: lados este y norte, tramo este</t>
         </is>
       </c>
     </row>
@@ -12196,7 +12197,7 @@
       </c>
       <c r="Q94" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado norte (y=851.7), tramo oeste</t>
+          <t>Bloque del centro: lado norte, tramo oeste</t>
         </is>
       </c>
     </row>
@@ -12263,7 +12264,7 @@
       </c>
       <c r="Q95" s="27" t="inlineStr">
         <is>
-          <t>Bloque del centro: lado norte (y=851.7), tramo oeste</t>
+          <t>Bloque del centro: lado norte, tramo oeste</t>
         </is>
       </c>
     </row>
@@ -17046,4 +17047,347 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TAPAS DE INSPECCION EN TRAMOS TAPADOS (0.60 x 0.60, CONCRETO REMOVIBLE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>MEJORAMIENTO Y AMPLIACION DEL SERVICIO DE EDUCACION PRIMARIA EN LA I.E. N.° 0590, DISTRITO DE BARRANQUITA, PROVINCIA DE LAMAS, DEPARTAMENTO DE SAN MARTIN - C.I. N.° 468901</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>N.</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>EJE</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>PROGRESIVA (m)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>ESTE (m)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>NORTE (m)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>UBICACION</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>T-01</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>EJE-02</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="n">
+        <v>75.73999999999999</v>
+      </c>
+      <c r="D5" s="28" t="n">
+        <v>354820.328</v>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>9249849.642999999</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>T-02</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>EJE-07</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="n">
+        <v>72.19</v>
+      </c>
+      <c r="D6" s="28" t="n">
+        <v>354919.895</v>
+      </c>
+      <c r="E6" s="28" t="n">
+        <v>9249801.445</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>T-03</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>EJE-07</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="n">
+        <v>79.41</v>
+      </c>
+      <c r="D7" s="28" t="n">
+        <v>354926.978</v>
+      </c>
+      <c r="E7" s="28" t="n">
+        <v>9249801.122</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>T-04</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>EJE-07</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="n">
+        <v>86.62</v>
+      </c>
+      <c r="D8" s="28" t="n">
+        <v>354928.135</v>
+      </c>
+      <c r="E8" s="28" t="n">
+        <v>9249794.353</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>T-05</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>EJE-07</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="n">
+        <v>93.84</v>
+      </c>
+      <c r="D9" s="28" t="n">
+        <v>354935.2</v>
+      </c>
+      <c r="E9" s="28" t="n">
+        <v>9249792.92</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>T-06</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>EJE-12</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="n">
+        <v>103.56</v>
+      </c>
+      <c r="D10" s="28" t="n">
+        <v>354976.611</v>
+      </c>
+      <c r="E10" s="28" t="n">
+        <v>9249860.776000001</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>T-07</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>EJE-12</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="n">
+        <v>110.54</v>
+      </c>
+      <c r="D11" s="28" t="n">
+        <v>354971.554</v>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>9249865.593</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>T-08</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>EJE-12</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="n">
+        <v>117.53</v>
+      </c>
+      <c r="D12" s="28" t="n">
+        <v>354965.926</v>
+      </c>
+      <c r="E12" s="28" t="n">
+        <v>9249868.98</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>T-09</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>EJE-17</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="D13" s="28" t="n">
+        <v>354940.68</v>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>9249853.501</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>T-10</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>EJE-17</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="n">
+        <v>12.53</v>
+      </c>
+      <c r="D14" s="28" t="n">
+        <v>354937.5</v>
+      </c>
+      <c r="E14" s="28" t="n">
+        <v>9249853.512</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Inicio / fin de tramo tapado, empalme o a 10 m como maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C15" s="29">
+        <f>COUNTA(B5:B14)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Barranquita: hidrologia transpuesta de Tarapoto, cantidades y metrado de drenaje pluvial
- hidrologia_b: serie Pmax24 CO Tarapoto, transposicion por precipitacion anual (factor 1.90),
  Log-Normal T = 25 anos, Dick y Peschke, IDF; I = 401 mm/h con tc = 10 min.
- verifica_b: caudales con C por superficie (techos, pavimentos, areas verdes); cunetas 0.40/0.60 cumplen.
- cantidades_b y metrado_b: metrado con formulas (RESUMEN, PLANILLA GENERAL, METRADO ACERO, PARAMETROS).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>I = 211 mm/h, C = 0.80, area total 9393 m2; menor borde libre 0.135 m en EJE-11 P-48-P-33 (Q 16.3 l/s, y 0.065, h 0.20)</t>
+          <t>I = 401 mm/h, C ponderado = 0.57, area total 9393 m2; menor borde libre 0.119 m en EJE-11 P-48-P-33 (Q 22.7 l/s, y 0.081, h 0.20)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>V max 1.84 m/s</t>
+          <t>V max 1.73 m/s</t>
         </is>
       </c>
     </row>
@@ -1462,31 +1462,31 @@
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>C (escorrentia)</t>
+          <t>C ponderado (escorrentia)</t>
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>0.8</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>I (mm/h)</t>
+          <t>I (mm/h), T = 25 anos, tc = 10 min</t>
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>211</v>
+        <v>400.96</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Factor de seguridad</t>
+          <t>P max 24 h transpuesta (mm)</t>
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1.15</v>
+        <v>231.49</v>
       </c>
     </row>
     <row r="7">
@@ -1502,7 +1502,7 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>I: tc = 10 min, TR = 25 anos, P10 = 35.16 mm (estacion usada en el Hogar de Refugio - Morales); reemplazar por la del proyecto. Area tributaria: cada m2 dentro del cerco a la cuneta mas cercana.</t>
+          <t>I: tc = 10 min, TR = 25 anos, P10 = 66.83 mm (estacion usada en el Hogar de Refugio - Morales); reemplazar por la del proyecto. Area tributaria: cada m2 dentro del cerco a la cuneta mas cercana.</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
         <v>0.5</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>0.095</v>
+        <v>0.083</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>0.3</v>
@@ -1610,7 +1610,7 @@
         <v/>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0.84</v>
+        <v>0.79</v>
       </c>
       <c r="K11" s="20">
         <f>IF(I11&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1649,7 +1649,7 @@
         <v>0.5</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>0.098</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>0.46</v>
@@ -1659,7 +1659,7 @@
         <v/>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="K12" s="20">
         <f>IF(I12&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1698,7 +1698,7 @@
         <v>0.5</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>0.3</v>
@@ -1708,7 +1708,7 @@
         <v/>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.77</v>
+        <v>0.72</v>
       </c>
       <c r="K13" s="20">
         <f>IF(I13&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1747,7 +1747,7 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>0.083</v>
+        <v>0.073</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>0.46</v>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0.79</v>
+        <v>0.74</v>
       </c>
       <c r="K14" s="20">
         <f>IF(I14&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1796,7 +1796,7 @@
         <v>0.5</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.094</v>
+        <v>0.083</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>0.46</v>
@@ -1806,7 +1806,7 @@
         <v/>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.83</v>
+        <v>0.78</v>
       </c>
       <c r="K15" s="20">
         <f>IF(I15&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1845,7 +1845,7 @@
         <v>2.92</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>0.078</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>0.52</v>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="J16" s="6" t="n">
-        <v>1.84</v>
+        <v>1.73</v>
       </c>
       <c r="K16" s="20">
         <f>IF(I16&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1894,7 +1894,7 @@
         <v>0.5</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>0.269</v>
+        <v>0.253</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>0.77</v>
@@ -1904,7 +1904,7 @@
         <v/>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1.24</v>
+        <v>1.22</v>
       </c>
       <c r="K17" s="20">
         <f>IF(I17&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1943,7 +1943,7 @@
         <v>0.5</v>
       </c>
       <c r="G18" s="18" t="n">
-        <v>0.269</v>
+        <v>0.253</v>
       </c>
       <c r="H18" s="17" t="n">
         <v>0.83</v>
@@ -1953,7 +1953,7 @@
         <v/>
       </c>
       <c r="J18" s="6" t="n">
-        <v>1.24</v>
+        <v>1.22</v>
       </c>
       <c r="K18" s="20">
         <f>IF(I18&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1992,7 +1992,7 @@
         <v>0.5</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>0.339</v>
+        <v>0.327</v>
       </c>
       <c r="H19" s="17" t="n">
         <v>0.83</v>
@@ -2002,7 +2002,7 @@
         <v/>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1.33</v>
+        <v>1.31</v>
       </c>
       <c r="K19" s="20">
         <f>IF(I19&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2041,7 +2041,7 @@
         <v>0.5</v>
       </c>
       <c r="G20" s="18" t="n">
-        <v>0.339</v>
+        <v>0.327</v>
       </c>
       <c r="H20" s="17" t="n">
         <v>0.79</v>
@@ -2051,7 +2051,7 @@
         <v/>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.33</v>
+        <v>1.31</v>
       </c>
       <c r="K20" s="20">
         <f>IF(I20&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2090,7 +2090,7 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>0.39</v>
+        <v>0.369</v>
       </c>
       <c r="H21" s="17" t="n">
         <v>0.79</v>
@@ -2100,7 +2100,7 @@
         <v/>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1.37</v>
+        <v>1.36</v>
       </c>
       <c r="K21" s="20">
         <f>IF(I21&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2139,7 +2139,7 @@
         <v>0.5</v>
       </c>
       <c r="G22" s="18" t="n">
-        <v>0.074</v>
+        <v>0.065</v>
       </c>
       <c r="H22" s="17" t="n">
         <v>0.3</v>
@@ -2149,7 +2149,7 @@
         <v/>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="K22" s="20">
         <f>IF(I22&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2188,7 +2188,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0.076</v>
+        <v>0.083</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>0.3</v>
@@ -2198,7 +2198,7 @@
         <v/>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.75</v>
+        <v>0.78</v>
       </c>
       <c r="K23" s="20">
         <f>IF(I23&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2237,7 +2237,7 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="18" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.089</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>0.43</v>
@@ -2247,7 +2247,7 @@
         <v/>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K24" s="20">
         <f>IF(I24&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2286,7 +2286,7 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="H25" s="17" t="n">
         <v>0.47</v>
@@ -2296,7 +2296,7 @@
         <v/>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K25" s="20">
         <f>IF(I25&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2335,7 +2335,7 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="18" t="n">
-        <v>0.101</v>
+        <v>0.112</v>
       </c>
       <c r="H26" s="17" t="n">
         <v>0.48</v>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="K26" s="20">
         <f>IF(I26&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2384,7 +2384,7 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0.124</v>
+        <v>0.132</v>
       </c>
       <c r="H27" s="17" t="n">
         <v>0.49</v>
@@ -2394,7 +2394,7 @@
         <v/>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.96</v>
       </c>
       <c r="K27" s="20">
         <f>IF(I27&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2433,7 +2433,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="18" t="n">
-        <v>0.132</v>
+        <v>0.139</v>
       </c>
       <c r="H28" s="17" t="n">
         <v>0.57</v>
@@ -2443,7 +2443,7 @@
         <v/>
       </c>
       <c r="J28" s="6" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="K28" s="20">
         <f>IF(I28&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2482,7 +2482,7 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0.166</v>
+        <v>0.167</v>
       </c>
       <c r="H29" s="17" t="n">
         <v>0.61</v>
@@ -2531,7 +2531,7 @@
         <v>0.5</v>
       </c>
       <c r="G30" s="18" t="n">
-        <v>0.047</v>
+        <v>0.067</v>
       </c>
       <c r="H30" s="17" t="n">
         <v>0.3</v>
@@ -2541,7 +2541,7 @@
         <v/>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.59</v>
+        <v>0.7</v>
       </c>
       <c r="K30" s="20">
         <f>IF(I30&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2580,7 +2580,7 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0.054</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H31" s="17" t="n">
         <v>0.41</v>
@@ -2590,7 +2590,7 @@
         <v/>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.63</v>
+        <v>0.73</v>
       </c>
       <c r="K31" s="20">
         <f>IF(I31&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2629,7 +2629,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="18" t="n">
-        <v>0.074</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H32" s="17" t="n">
         <v>0.44</v>
@@ -2639,7 +2639,7 @@
         <v/>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.74</v>
+        <v>0.8</v>
       </c>
       <c r="K32" s="20">
         <f>IF(I32&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2678,7 +2678,7 @@
         <v>0.5</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0.079</v>
+        <v>0.092</v>
       </c>
       <c r="H33" s="17" t="n">
         <v>0.53</v>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
       <c r="J33" s="6" t="n">
-        <v>0.77</v>
+        <v>0.82</v>
       </c>
       <c r="K33" s="20">
         <f>IF(I33&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2727,7 +2727,7 @@
         <v>0.5</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>0.115</v>
+        <v>0.12</v>
       </c>
       <c r="H34" s="17" t="n">
         <v>0.55</v>
@@ -2737,7 +2737,7 @@
         <v/>
       </c>
       <c r="J34" s="6" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="K34" s="20">
         <f>IF(I34&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2776,7 +2776,7 @@
         <v>0.5</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0.034</v>
+        <v>0.043</v>
       </c>
       <c r="H35" s="17" t="n">
         <v>0.3</v>
@@ -2786,7 +2786,7 @@
         <v/>
       </c>
       <c r="J35" s="6" t="n">
-        <v>0.49</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K35" s="20">
         <f>IF(I35&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2825,7 +2825,7 @@
         <v>1.72</v>
       </c>
       <c r="G36" s="18" t="n">
-        <v>0.023</v>
+        <v>0.03</v>
       </c>
       <c r="H36" s="17" t="n">
         <v>0.3</v>
@@ -2835,7 +2835,7 @@
         <v/>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0.73</v>
+        <v>0.84</v>
       </c>
       <c r="K36" s="20">
         <f>IF(I36&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2874,7 +2874,7 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0.124</v>
+        <v>0.134</v>
       </c>
       <c r="H37" s="17" t="n">
         <v>0.5</v>
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="J37" s="6" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="K37" s="20">
         <f>IF(I37&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2923,7 +2923,7 @@
         <v>0.5</v>
       </c>
       <c r="G38" s="18" t="n">
-        <v>0.164</v>
+        <v>0.175</v>
       </c>
       <c r="H38" s="17" t="n">
         <v>0.59</v>
@@ -2933,7 +2933,7 @@
         <v/>
       </c>
       <c r="J38" s="6" t="n">
-        <v>1.05</v>
+        <v>1.08</v>
       </c>
       <c r="K38" s="20">
         <f>IF(I38&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2972,7 +2972,7 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0.164</v>
+        <v>0.175</v>
       </c>
       <c r="H39" s="17" t="n">
         <v>0.61</v>
@@ -2982,7 +2982,7 @@
         <v/>
       </c>
       <c r="J39" s="6" t="n">
-        <v>1.05</v>
+        <v>1.08</v>
       </c>
       <c r="K39" s="20">
         <f>IF(I39&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3021,7 +3021,7 @@
         <v>0.5</v>
       </c>
       <c r="G40" s="18" t="n">
-        <v>0.183</v>
+        <v>0.207</v>
       </c>
       <c r="H40" s="17" t="n">
         <v>0.62</v>
@@ -3031,7 +3031,7 @@
         <v/>
       </c>
       <c r="J40" s="6" t="n">
-        <v>1.1</v>
+        <v>1.14</v>
       </c>
       <c r="K40" s="20">
         <f>IF(I40&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3070,7 +3070,7 @@
         <v>0.5</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0.183</v>
+        <v>0.207</v>
       </c>
       <c r="H41" s="17" t="n">
         <v>0.73</v>
@@ -3080,7 +3080,7 @@
         <v/>
       </c>
       <c r="J41" s="6" t="n">
-        <v>1.1</v>
+        <v>1.14</v>
       </c>
       <c r="K41" s="20">
         <f>IF(I41&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3119,7 +3119,7 @@
         <v>0.5</v>
       </c>
       <c r="G42" s="18" t="n">
-        <v>0.226</v>
+        <v>0.271</v>
       </c>
       <c r="H42" s="17" t="n">
         <v>0.73</v>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
       <c r="J42" s="6" t="n">
-        <v>1.18</v>
+        <v>1.25</v>
       </c>
       <c r="K42" s="20">
         <f>IF(I42&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3168,7 +3168,7 @@
         <v>0.5</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0.256</v>
+        <v>0.312</v>
       </c>
       <c r="H43" s="17" t="n">
         <v>0.79</v>
@@ -3178,7 +3178,7 @@
         <v/>
       </c>
       <c r="J43" s="6" t="n">
-        <v>1.22</v>
+        <v>1.3</v>
       </c>
       <c r="K43" s="20">
         <f>IF(I43&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3217,7 +3217,7 @@
         <v>0.5</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>0.256</v>
+        <v>0.312</v>
       </c>
       <c r="H44" s="17" t="n">
         <v>0.7</v>
@@ -3227,7 +3227,7 @@
         <v/>
       </c>
       <c r="J44" s="6" t="n">
-        <v>1.22</v>
+        <v>1.3</v>
       </c>
       <c r="K44" s="20">
         <f>IF(I44&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3266,7 +3266,7 @@
         <v>0.5</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>0.257</v>
+        <v>0.313</v>
       </c>
       <c r="H45" s="17" t="n">
         <v>0.7</v>
@@ -3276,7 +3276,7 @@
         <v/>
       </c>
       <c r="J45" s="6" t="n">
-        <v>1.23</v>
+        <v>1.3</v>
       </c>
       <c r="K45" s="20">
         <f>IF(I45&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3315,7 +3315,7 @@
         <v>0.5</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>0.258</v>
+        <v>0.314</v>
       </c>
       <c r="H46" s="17" t="n">
         <v>0.74</v>
@@ -3325,7 +3325,7 @@
         <v/>
       </c>
       <c r="J46" s="6" t="n">
-        <v>1.23</v>
+        <v>1.3</v>
       </c>
       <c r="K46" s="20">
         <f>IF(I46&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3364,7 +3364,7 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>0.26</v>
+        <v>0.315</v>
       </c>
       <c r="H47" s="17" t="n">
         <v>0.74</v>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="J47" s="6" t="n">
-        <v>1.23</v>
+        <v>1.3</v>
       </c>
       <c r="K47" s="20">
         <f>IF(I47&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3413,7 +3413,7 @@
         <v>0.5</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>0.26</v>
+        <v>0.315</v>
       </c>
       <c r="H48" s="17" t="n">
         <v>0.77</v>
@@ -3423,7 +3423,7 @@
         <v/>
       </c>
       <c r="J48" s="6" t="n">
-        <v>1.23</v>
+        <v>1.3</v>
       </c>
       <c r="K48" s="20">
         <f>IF(I48&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3462,7 +3462,7 @@
         <v>0.5</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>0.265</v>
+        <v>0.319</v>
       </c>
       <c r="H49" s="17" t="n">
         <v>0.77</v>
@@ -3472,7 +3472,7 @@
         <v/>
       </c>
       <c r="J49" s="6" t="n">
-        <v>1.24</v>
+        <v>1.31</v>
       </c>
       <c r="K49" s="20">
         <f>IF(I49&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3511,7 +3511,7 @@
         <v>0.5</v>
       </c>
       <c r="G50" s="18" t="n">
-        <v>0.266</v>
+        <v>0.32</v>
       </c>
       <c r="H50" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3521,7 +3521,7 @@
         <v/>
       </c>
       <c r="J50" s="6" t="n">
-        <v>1.24</v>
+        <v>1.31</v>
       </c>
       <c r="K50" s="20">
         <f>IF(I50&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3560,7 +3560,7 @@
         <v>0.5</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>0.266</v>
+        <v>0.32</v>
       </c>
       <c r="H51" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3570,7 +3570,7 @@
         <v/>
       </c>
       <c r="J51" s="6" t="n">
-        <v>1.24</v>
+        <v>1.31</v>
       </c>
       <c r="K51" s="20">
         <f>IF(I51&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3609,7 +3609,7 @@
         <v>0.5</v>
       </c>
       <c r="G52" s="18" t="n">
-        <v>0.02</v>
+        <v>0.027</v>
       </c>
       <c r="H52" s="17" t="n">
         <v>0.3</v>
@@ -3619,7 +3619,7 @@
         <v/>
       </c>
       <c r="J52" s="6" t="n">
-        <v>0.35</v>
+        <v>0.43</v>
       </c>
       <c r="K52" s="20">
         <f>IF(I52&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3658,7 +3658,7 @@
         <v>0.5</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>0.089</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H53" s="17" t="n">
         <v>0.32</v>
@@ -3668,7 +3668,7 @@
         <v/>
       </c>
       <c r="J53" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="K53" s="20">
         <f>IF(I53&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3707,7 +3707,7 @@
         <v>0.5</v>
       </c>
       <c r="G54" s="18" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.073</v>
       </c>
       <c r="H54" s="17" t="n">
         <v>0.3</v>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J54" s="6" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="K54" s="20">
         <f>IF(I54&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3756,7 +3756,7 @@
         <v>0.5</v>
       </c>
       <c r="G55" s="18" t="n">
-        <v>0.05</v>
+        <v>0.062</v>
       </c>
       <c r="H55" s="17" t="n">
         <v>0.3</v>
@@ -3766,7 +3766,7 @@
         <v/>
       </c>
       <c r="J55" s="6" t="n">
-        <v>0.61</v>
+        <v>0.68</v>
       </c>
       <c r="K55" s="20">
         <f>IF(I55&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3805,7 +3805,7 @@
         <v>0.5</v>
       </c>
       <c r="G56" s="18" t="n">
-        <v>0.054</v>
+        <v>0.068</v>
       </c>
       <c r="H56" s="17" t="n">
         <v>0.39</v>
@@ -3815,7 +3815,7 @@
         <v/>
       </c>
       <c r="J56" s="6" t="n">
-        <v>0.63</v>
+        <v>0.71</v>
       </c>
       <c r="K56" s="20">
         <f>IF(I56&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3854,7 +3854,7 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="18" t="n">
-        <v>0.056</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H57" s="17" t="n">
         <v>0.42</v>
@@ -3864,7 +3864,7 @@
         <v/>
       </c>
       <c r="J57" s="6" t="n">
-        <v>0.64</v>
+        <v>0.73</v>
       </c>
       <c r="K57" s="20">
         <f>IF(I57&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3903,7 +3903,7 @@
         <v>0.5</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.091</v>
       </c>
       <c r="H58" s="17" t="n">
         <v>0.42</v>
@@ -3913,7 +3913,7 @@
         <v/>
       </c>
       <c r="J58" s="6" t="n">
-        <v>0.72</v>
+        <v>0.82</v>
       </c>
       <c r="K58" s="20">
         <f>IF(I58&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3952,7 +3952,7 @@
         <v>0.5</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.091</v>
       </c>
       <c r="H59" s="17" t="n">
         <v>0.48</v>
@@ -3962,7 +3962,7 @@
         <v/>
       </c>
       <c r="J59" s="6" t="n">
-        <v>0.72</v>
+        <v>0.82</v>
       </c>
       <c r="K59" s="20">
         <f>IF(I59&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4001,7 +4001,7 @@
         <v>0.5</v>
       </c>
       <c r="G60" s="18" t="n">
-        <v>0.065</v>
+        <v>0.081</v>
       </c>
       <c r="H60" s="17" t="n">
         <v>0.2</v>
@@ -4011,7 +4011,7 @@
         <v/>
       </c>
       <c r="J60" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.77</v>
       </c>
       <c r="K60" s="20">
         <f>IF(I60&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4050,7 +4050,7 @@
         <v>0.5</v>
       </c>
       <c r="G61" s="18" t="n">
-        <v>0.055</v>
+        <v>0.057</v>
       </c>
       <c r="H61" s="17" t="n">
         <v>0.3</v>
@@ -4060,7 +4060,7 @@
         <v/>
       </c>
       <c r="J61" s="6" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="K61" s="20">
         <f>IF(I61&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4099,7 +4099,7 @@
         <v>0.5</v>
       </c>
       <c r="G62" s="18" t="n">
-        <v>0.057</v>
+        <v>0.06</v>
       </c>
       <c r="H62" s="17" t="n">
         <v>0.38</v>
@@ -4109,7 +4109,7 @@
         <v/>
       </c>
       <c r="J62" s="6" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="K62" s="20">
         <f>IF(I62&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4148,7 +4148,7 @@
         <v>0.5</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>0.095</v>
+        <v>0.092</v>
       </c>
       <c r="H63" s="17" t="n">
         <v>0.38</v>
@@ -4158,7 +4158,7 @@
         <v/>
       </c>
       <c r="J63" s="6" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="K63" s="20">
         <f>IF(I63&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4197,7 +4197,7 @@
         <v>0.5</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>0.095</v>
+        <v>0.093</v>
       </c>
       <c r="H64" s="17" t="n">
         <v>0.49</v>
@@ -4207,7 +4207,7 @@
         <v/>
       </c>
       <c r="J64" s="6" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="K64" s="20">
         <f>IF(I64&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4246,7 +4246,7 @@
         <v>0.5</v>
       </c>
       <c r="G65" s="18" t="n">
-        <v>0.132</v>
+        <v>0.124</v>
       </c>
       <c r="H65" s="17" t="n">
         <v>0.5</v>
@@ -4256,7 +4256,7 @@
         <v/>
       </c>
       <c r="J65" s="6" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K65" s="20">
         <f>IF(I65&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4295,7 +4295,7 @@
         <v>0.5</v>
       </c>
       <c r="G66" s="18" t="n">
-        <v>0.162</v>
+        <v>0.161</v>
       </c>
       <c r="H66" s="17" t="n">
         <v>0.52</v>
@@ -4305,7 +4305,7 @@
         <v/>
       </c>
       <c r="J66" s="6" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="K66" s="20">
         <f>IF(I66&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4344,7 +4344,7 @@
         <v>0.5</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>0.235</v>
+        <v>0.279</v>
       </c>
       <c r="H67" s="17" t="n">
         <v>0.5600000000000001</v>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="J67" s="6" t="n">
-        <v>1.19</v>
+        <v>1.26</v>
       </c>
       <c r="K67" s="20">
         <f>IF(I67&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4393,7 +4393,7 @@
         <v>0.5</v>
       </c>
       <c r="G68" s="18" t="n">
-        <v>0.282</v>
+        <v>0.36</v>
       </c>
       <c r="H68" s="17" t="n">
         <v>0.62</v>
@@ -4403,7 +4403,7 @@
         <v/>
       </c>
       <c r="J68" s="6" t="n">
-        <v>1.26</v>
+        <v>1.35</v>
       </c>
       <c r="K68" s="20">
         <f>IF(I68&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4442,7 +4442,7 @@
         <v>0.5</v>
       </c>
       <c r="G69" s="18" t="n">
-        <v>0.294</v>
+        <v>0.38</v>
       </c>
       <c r="H69" s="17" t="n">
         <v>0.57</v>
@@ -4452,7 +4452,7 @@
         <v/>
       </c>
       <c r="J69" s="6" t="n">
-        <v>1.28</v>
+        <v>1.36</v>
       </c>
       <c r="K69" s="20">
         <f>IF(I69&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4491,7 +4491,7 @@
         <v>0.5</v>
       </c>
       <c r="G70" s="18" t="n">
-        <v>0.295</v>
+        <v>0.382</v>
       </c>
       <c r="H70" s="17" t="n">
         <v>0.63</v>
@@ -4501,7 +4501,7 @@
         <v/>
       </c>
       <c r="J70" s="6" t="n">
-        <v>1.28</v>
+        <v>1.37</v>
       </c>
       <c r="K70" s="20">
         <f>IF(I70&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4540,7 +4540,7 @@
         <v>0.5</v>
       </c>
       <c r="G71" s="18" t="n">
-        <v>0.295</v>
+        <v>0.382</v>
       </c>
       <c r="H71" s="17" t="n">
         <v>0.64</v>
@@ -4550,7 +4550,7 @@
         <v/>
       </c>
       <c r="J71" s="6" t="n">
-        <v>1.28</v>
+        <v>1.37</v>
       </c>
       <c r="K71" s="20">
         <f>IF(I71&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4589,7 +4589,7 @@
         <v>0.5</v>
       </c>
       <c r="G72" s="18" t="n">
-        <v>0.344</v>
+        <v>0.45</v>
       </c>
       <c r="H72" s="17" t="n">
         <v>0.64</v>
@@ -4599,7 +4599,7 @@
         <v/>
       </c>
       <c r="J72" s="6" t="n">
-        <v>1.33</v>
+        <v>1.42</v>
       </c>
       <c r="K72" s="20">
         <f>IF(I72&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4638,7 +4638,7 @@
         <v>0.5</v>
       </c>
       <c r="G73" s="18" t="n">
-        <v>0.056</v>
+        <v>0.064</v>
       </c>
       <c r="H73" s="17" t="n">
         <v>0.3</v>
@@ -4648,7 +4648,7 @@
         <v/>
       </c>
       <c r="J73" s="6" t="n">
-        <v>0.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K73" s="20">
         <f>IF(I73&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4687,7 +4687,7 @@
         <v>0.5</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>0.049</v>
+        <v>0.073</v>
       </c>
       <c r="H74" s="17" t="n">
         <v>0.3</v>
@@ -4697,7 +4697,7 @@
         <v/>
       </c>
       <c r="J74" s="6" t="n">
-        <v>0.6</v>
+        <v>0.73</v>
       </c>
       <c r="K74" s="20">
         <f>IF(I74&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4736,7 +4736,7 @@
         <v>0.5</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>0.053</v>
+        <v>0.075</v>
       </c>
       <c r="H75" s="17" t="n">
         <v>0.38</v>
@@ -4746,7 +4746,7 @@
         <v/>
       </c>
       <c r="J75" s="6" t="n">
-        <v>0.62</v>
+        <v>0.75</v>
       </c>
       <c r="K75" s="20">
         <f>IF(I75&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4785,7 +4785,7 @@
         <v>0.5</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.12</v>
       </c>
       <c r="H76" s="17" t="n">
         <v>0.35</v>
@@ -4795,7 +4795,7 @@
         <v/>
       </c>
       <c r="J76" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.93</v>
       </c>
       <c r="K76" s="20">
         <f>IF(I76&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4834,7 +4834,7 @@
         <v>0.5</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.12</v>
       </c>
       <c r="H77" s="17" t="n">
         <v>0.35</v>
@@ -4844,7 +4844,7 @@
         <v/>
       </c>
       <c r="J77" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.93</v>
       </c>
       <c r="K77" s="20">
         <f>IF(I77&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4883,7 +4883,7 @@
         <v>0.5</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>0.089</v>
+        <v>0.122</v>
       </c>
       <c r="H78" s="17" t="n">
         <v>0.35</v>
@@ -4893,7 +4893,7 @@
         <v/>
       </c>
       <c r="J78" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.93</v>
       </c>
       <c r="K78" s="20">
         <f>IF(I78&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4932,7 +4932,7 @@
         <v>0.5</v>
       </c>
       <c r="G79" s="18" t="n">
-        <v>0.111</v>
+        <v>0.158</v>
       </c>
       <c r="H79" s="17" t="n">
         <v>0.35</v>
@@ -4942,7 +4942,7 @@
         <v/>
       </c>
       <c r="J79" s="6" t="n">
-        <v>0.9</v>
+        <v>1.04</v>
       </c>
       <c r="K79" s="20">
         <f>IF(I79&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4981,7 +4981,7 @@
         <v>0.5</v>
       </c>
       <c r="G80" s="18" t="n">
-        <v>0.114</v>
+        <v>0.161</v>
       </c>
       <c r="H80" s="17" t="n">
         <v>0.45</v>
@@ -4991,7 +4991,7 @@
         <v/>
       </c>
       <c r="J80" s="6" t="n">
-        <v>0.91</v>
+        <v>1.05</v>
       </c>
       <c r="K80" s="20">
         <f>IF(I80&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5030,7 +5030,7 @@
         <v>0.5</v>
       </c>
       <c r="G81" s="18" t="n">
-        <v>0.042</v>
+        <v>0.061</v>
       </c>
       <c r="H81" s="17" t="n">
         <v>0.3</v>
@@ -5040,7 +5040,7 @@
         <v/>
       </c>
       <c r="J81" s="6" t="n">
-        <v>0.55</v>
+        <v>0.67</v>
       </c>
       <c r="K81" s="20">
         <f>IF(I81&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5079,7 +5079,7 @@
         <v>0.5</v>
       </c>
       <c r="G82" s="18" t="n">
-        <v>0.042</v>
+        <v>0.062</v>
       </c>
       <c r="H82" s="17" t="n">
         <v>0.36</v>
@@ -5089,7 +5089,7 @@
         <v/>
       </c>
       <c r="J82" s="6" t="n">
-        <v>0.55</v>
+        <v>0.68</v>
       </c>
       <c r="K82" s="20">
         <f>IF(I82&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5128,7 +5128,7 @@
         <v>0.58</v>
       </c>
       <c r="G83" s="18" t="n">
-        <v>0.078</v>
+        <v>0.117</v>
       </c>
       <c r="H83" s="17" t="n">
         <v>0.35</v>
@@ -5138,7 +5138,7 @@
         <v/>
       </c>
       <c r="J83" s="6" t="n">
-        <v>0.82</v>
+        <v>0.99</v>
       </c>
       <c r="K83" s="20">
         <f>IF(I83&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5177,7 +5177,7 @@
         <v>0.5</v>
       </c>
       <c r="G84" s="18" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.128</v>
       </c>
       <c r="H84" s="17" t="n">
         <v>0.35</v>
@@ -5187,7 +5187,7 @@
         <v/>
       </c>
       <c r="J84" s="6" t="n">
-        <v>0.79</v>
+        <v>0.95</v>
       </c>
       <c r="K84" s="20">
         <f>IF(I84&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5226,7 +5226,7 @@
         <v>0.5</v>
       </c>
       <c r="G85" s="18" t="n">
-        <v>0.075</v>
+        <v>0.092</v>
       </c>
       <c r="H85" s="17" t="n">
         <v>0.3</v>
@@ -5236,7 +5236,7 @@
         <v/>
       </c>
       <c r="J85" s="6" t="n">
-        <v>0.75</v>
+        <v>0.82</v>
       </c>
       <c r="K85" s="20">
         <f>IF(I85&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5275,7 +5275,7 @@
         <v>0.5</v>
       </c>
       <c r="G86" s="18" t="n">
-        <v>0.078</v>
+        <v>0.097</v>
       </c>
       <c r="H86" s="17" t="n">
         <v>0.45</v>
@@ -5285,7 +5285,7 @@
         <v/>
       </c>
       <c r="J86" s="6" t="n">
-        <v>0.76</v>
+        <v>0.84</v>
       </c>
       <c r="K86" s="20">
         <f>IF(I86&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5324,7 +5324,7 @@
         <v>0.5</v>
       </c>
       <c r="G87" s="18" t="n">
-        <v>0.08</v>
+        <v>0.099</v>
       </c>
       <c r="H87" s="17" t="n">
         <v>0.46</v>
@@ -5334,7 +5334,7 @@
         <v/>
       </c>
       <c r="J87" s="6" t="n">
-        <v>0.77</v>
+        <v>0.85</v>
       </c>
       <c r="K87" s="20">
         <f>IF(I87&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5373,7 +5373,7 @@
         <v>0.5</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>0.08</v>
+        <v>0.099</v>
       </c>
       <c r="H88" s="17" t="n">
         <v>0.47</v>
@@ -5383,7 +5383,7 @@
         <v/>
       </c>
       <c r="J88" s="6" t="n">
-        <v>0.77</v>
+        <v>0.85</v>
       </c>
       <c r="K88" s="20">
         <f>IF(I88&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5422,7 +5422,7 @@
         <v>0.5</v>
       </c>
       <c r="G89" s="18" t="n">
-        <v>0.094</v>
+        <v>0.122</v>
       </c>
       <c r="H89" s="17" t="n">
         <v>0.4</v>
@@ -5432,7 +5432,7 @@
         <v/>
       </c>
       <c r="J89" s="6" t="n">
-        <v>0.83</v>
+        <v>0.93</v>
       </c>
       <c r="K89" s="20">
         <f>IF(I89&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5471,7 +5471,7 @@
         <v>0.5</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>0.094</v>
+        <v>0.122</v>
       </c>
       <c r="H90" s="17" t="n">
         <v>0.4</v>
@@ -5481,7 +5481,7 @@
         <v/>
       </c>
       <c r="J90" s="6" t="n">
-        <v>0.83</v>
+        <v>0.93</v>
       </c>
       <c r="K90" s="20">
         <f>IF(I90&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5520,7 +5520,7 @@
         <v>0.51</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>0.059</v>
+        <v>0.08</v>
       </c>
       <c r="H91" s="17" t="n">
         <v>0.2</v>
@@ -5530,7 +5530,7 @@
         <v/>
       </c>
       <c r="J91" s="6" t="n">
-        <v>0.67</v>
+        <v>0.78</v>
       </c>
       <c r="K91" s="20">
         <f>IF(I91&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5569,7 +5569,7 @@
         <v>0.5</v>
       </c>
       <c r="G92" s="18" t="n">
-        <v>0.059</v>
+        <v>0.08</v>
       </c>
       <c r="H92" s="17" t="n">
         <v>0.5</v>
@@ -5579,7 +5579,7 @@
         <v/>
       </c>
       <c r="J92" s="6" t="n">
-        <v>0.66</v>
+        <v>0.77</v>
       </c>
       <c r="K92" s="20">
         <f>IF(I92&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5618,7 +5618,7 @@
         <v>0.5</v>
       </c>
       <c r="G93" s="18" t="n">
-        <v>0.106</v>
+        <v>0.122</v>
       </c>
       <c r="H93" s="17" t="n">
         <v>0.5</v>
@@ -5628,7 +5628,7 @@
         <v/>
       </c>
       <c r="J93" s="6" t="n">
-        <v>0.88</v>
+        <v>0.93</v>
       </c>
       <c r="K93" s="20">
         <f>IF(I93&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5667,7 +5667,7 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="18" t="n">
-        <v>0.107</v>
+        <v>0.123</v>
       </c>
       <c r="H94" s="17" t="n">
         <v>0.4</v>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="J94" s="6" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K94" s="20">
         <f>IF(I94&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5716,7 +5716,7 @@
         <v>0.5</v>
       </c>
       <c r="G95" s="18" t="n">
-        <v>0.03</v>
+        <v>0.036</v>
       </c>
       <c r="H95" s="17" t="n">
         <v>0.3</v>
@@ -5726,7 +5726,7 @@
         <v/>
       </c>
       <c r="J95" s="6" t="n">
-        <v>0.45</v>
+        <v>0.51</v>
       </c>
       <c r="K95" s="20">
         <f>IF(I95&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5765,7 +5765,7 @@
         <v>0.5</v>
       </c>
       <c r="G96" s="18" t="n">
-        <v>0.03</v>
+        <v>0.036</v>
       </c>
       <c r="H96" s="17" t="n">
         <v>0.36</v>
@@ -5775,7 +5775,7 @@
         <v/>
       </c>
       <c r="J96" s="6" t="n">
-        <v>0.45</v>
+        <v>0.51</v>
       </c>
       <c r="K96" s="20">
         <f>IF(I96&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5814,7 +5814,7 @@
         <v>0.5</v>
       </c>
       <c r="G97" s="18" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
       <c r="H97" s="17" t="n">
         <v>0.36</v>
@@ -5824,7 +5824,7 @@
         <v/>
       </c>
       <c r="J97" s="6" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="K97" s="20">
         <f>IF(I97&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5863,7 +5863,7 @@
         <v>0.5</v>
       </c>
       <c r="G98" s="18" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
       <c r="H98" s="17" t="n">
         <v>0.48</v>
@@ -5873,7 +5873,7 @@
         <v/>
       </c>
       <c r="J98" s="6" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="K98" s="20">
         <f>IF(I98&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5912,7 +5912,7 @@
         <v>0.5</v>
       </c>
       <c r="G99" s="18" t="n">
-        <v>0.073</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H99" s="17" t="n">
         <v>0.49</v>
@@ -5922,7 +5922,7 @@
         <v/>
       </c>
       <c r="J99" s="6" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="K99" s="20">
         <f>IF(I99&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5961,7 +5961,7 @@
         <v>0.5</v>
       </c>
       <c r="G100" s="18" t="n">
-        <v>0.033</v>
+        <v>0.03</v>
       </c>
       <c r="H100" s="17" t="n">
         <v>0.3</v>
@@ -5971,7 +5971,7 @@
         <v/>
       </c>
       <c r="J100" s="6" t="n">
-        <v>0.48</v>
+        <v>0.45</v>
       </c>
       <c r="K100" s="20">
         <f>IF(I100&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -6010,7 +6010,7 @@
         <v>0.5</v>
       </c>
       <c r="G101" s="18" t="n">
-        <v>0.033</v>
+        <v>0.03</v>
       </c>
       <c r="H101" s="17" t="n">
         <v>0.37</v>
@@ -6020,7 +6020,7 @@
         <v/>
       </c>
       <c r="J101" s="6" t="n">
-        <v>0.48</v>
+        <v>0.45</v>
       </c>
       <c r="K101" s="20">
         <f>IF(I101&gt;=0.05,"CUMPLE","NO CUMPLE")</f>

</xml_diff>

<commit_message>
Barranquita: lluvia anual de las estaciones de llanura (Navarro, Pelejo, Shanusi) en la transposicion
Factor 2.21 (2,375.6 / 1,073.1 mm); P24 T25 = 269.6 mm; I = 467 mm/h. Las cunetas 0.40/0.60 cumplen en todos los tramos.
Memorias hidrologica, descriptiva y de calculo actualizadas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>I = 401 mm/h, C ponderado = 0.57, area total 9393 m2; menor borde libre 0.119 m en EJE-11 P-48-P-33 (Q 22.7 l/s, y 0.081, h 0.20)</t>
+          <t>I = 467 mm/h, C ponderado = 0.57, area total 9393 m2; menor borde libre 0.110 m en EJE-11 P-48-P-33 (Q 26.4 l/s, y 0.090, h 0.20)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>V max 1.73 m/s</t>
+          <t>V max 1.82 m/s</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>400.96</v>
+        <v>467</v>
       </c>
     </row>
     <row r="6">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>231.49</v>
+        <v>269.62</v>
       </c>
     </row>
     <row r="7">
@@ -1502,7 +1502,7 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>I: tc = 10 min, TR = 25 anos, P10 = 66.83 mm (estacion usada en el Hogar de Refugio - Morales); reemplazar por la del proyecto. Area tributaria: cada m2 dentro del cerco a la cuneta mas cercana.</t>
+          <t>I: tc = 10 min, TR = 25 anos, P10 = 77.83 mm (estacion usada en el Hogar de Refugio - Morales); reemplazar por la del proyecto. Area tributaria: cada m2 dentro del cerco a la cuneta mas cercana.</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
         <v>0.5</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>0.083</v>
+        <v>0.092</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>0.3</v>
@@ -1610,7 +1610,7 @@
         <v/>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0.79</v>
+        <v>0.82</v>
       </c>
       <c r="K11" s="20">
         <f>IF(I11&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1649,7 +1649,7 @@
         <v>0.5</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.096</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>0.46</v>
@@ -1659,7 +1659,7 @@
         <v/>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="K12" s="20">
         <f>IF(I12&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1698,7 +1698,7 @@
         <v>0.5</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.078</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>0.3</v>
@@ -1708,7 +1708,7 @@
         <v/>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
       <c r="K13" s="20">
         <f>IF(I13&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1747,7 +1747,7 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>0.073</v>
+        <v>0.081</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>0.46</v>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0.74</v>
+        <v>0.78</v>
       </c>
       <c r="K14" s="20">
         <f>IF(I14&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1796,7 +1796,7 @@
         <v>0.5</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.083</v>
+        <v>0.092</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>0.46</v>
@@ -1806,7 +1806,7 @@
         <v/>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.78</v>
+        <v>0.82</v>
       </c>
       <c r="K15" s="20">
         <f>IF(I15&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1845,7 +1845,7 @@
         <v>2.92</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.076</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>0.52</v>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="J16" s="6" t="n">
-        <v>1.73</v>
+        <v>1.82</v>
       </c>
       <c r="K16" s="20">
         <f>IF(I16&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1894,7 +1894,7 @@
         <v>0.5</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>0.253</v>
+        <v>0.285</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>0.77</v>
@@ -1904,7 +1904,7 @@
         <v/>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1.22</v>
+        <v>1.26</v>
       </c>
       <c r="K17" s="20">
         <f>IF(I17&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1943,7 +1943,7 @@
         <v>0.5</v>
       </c>
       <c r="G18" s="18" t="n">
-        <v>0.253</v>
+        <v>0.285</v>
       </c>
       <c r="H18" s="17" t="n">
         <v>0.83</v>
@@ -1953,7 +1953,7 @@
         <v/>
       </c>
       <c r="J18" s="6" t="n">
-        <v>1.22</v>
+        <v>1.26</v>
       </c>
       <c r="K18" s="20">
         <f>IF(I18&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1992,7 +1992,7 @@
         <v>0.5</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>0.327</v>
+        <v>0.37</v>
       </c>
       <c r="H19" s="17" t="n">
         <v>0.83</v>
@@ -2002,7 +2002,7 @@
         <v/>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1.31</v>
+        <v>1.36</v>
       </c>
       <c r="K19" s="20">
         <f>IF(I19&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2041,7 +2041,7 @@
         <v>0.5</v>
       </c>
       <c r="G20" s="18" t="n">
-        <v>0.327</v>
+        <v>0.37</v>
       </c>
       <c r="H20" s="17" t="n">
         <v>0.79</v>
@@ -2051,7 +2051,7 @@
         <v/>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.31</v>
+        <v>1.36</v>
       </c>
       <c r="K20" s="20">
         <f>IF(I20&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2090,7 +2090,7 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>0.369</v>
+        <v>0.418</v>
       </c>
       <c r="H21" s="17" t="n">
         <v>0.79</v>
@@ -2100,7 +2100,7 @@
         <v/>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1.36</v>
+        <v>1.4</v>
       </c>
       <c r="K21" s="20">
         <f>IF(I21&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2139,7 +2139,7 @@
         <v>0.5</v>
       </c>
       <c r="G22" s="18" t="n">
-        <v>0.065</v>
+        <v>0.073</v>
       </c>
       <c r="H22" s="17" t="n">
         <v>0.3</v>
@@ -2149,7 +2149,7 @@
         <v/>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="K22" s="20">
         <f>IF(I22&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2188,7 +2188,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0.083</v>
+        <v>0.092</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>0.3</v>
@@ -2198,7 +2198,7 @@
         <v/>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.78</v>
+        <v>0.82</v>
       </c>
       <c r="K23" s="20">
         <f>IF(I23&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2237,7 +2237,7 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="18" t="n">
-        <v>0.089</v>
+        <v>0.099</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>0.43</v>
@@ -2247,7 +2247,7 @@
         <v/>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="K24" s="20">
         <f>IF(I24&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2286,7 +2286,7 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="H25" s="17" t="n">
         <v>0.47</v>
@@ -2296,7 +2296,7 @@
         <v/>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="K25" s="20">
         <f>IF(I25&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2335,7 +2335,7 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="18" t="n">
-        <v>0.112</v>
+        <v>0.124</v>
       </c>
       <c r="H26" s="17" t="n">
         <v>0.48</v>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.9</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K26" s="20">
         <f>IF(I26&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2384,7 +2384,7 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0.132</v>
+        <v>0.147</v>
       </c>
       <c r="H27" s="17" t="n">
         <v>0.49</v>
@@ -2394,7 +2394,7 @@
         <v/>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0.96</v>
+        <v>1.01</v>
       </c>
       <c r="K27" s="20">
         <f>IF(I27&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2433,7 +2433,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="18" t="n">
-        <v>0.139</v>
+        <v>0.156</v>
       </c>
       <c r="H28" s="17" t="n">
         <v>0.57</v>
@@ -2443,7 +2443,7 @@
         <v/>
       </c>
       <c r="J28" s="6" t="n">
-        <v>0.99</v>
+        <v>1.03</v>
       </c>
       <c r="K28" s="20">
         <f>IF(I28&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2482,7 +2482,7 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0.167</v>
+        <v>0.187</v>
       </c>
       <c r="H29" s="17" t="n">
         <v>0.61</v>
@@ -2492,7 +2492,7 @@
         <v/>
       </c>
       <c r="J29" s="6" t="n">
-        <v>1.06</v>
+        <v>1.1</v>
       </c>
       <c r="K29" s="20">
         <f>IF(I29&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2531,7 +2531,7 @@
         <v>0.5</v>
       </c>
       <c r="G30" s="18" t="n">
-        <v>0.067</v>
+        <v>0.074</v>
       </c>
       <c r="H30" s="17" t="n">
         <v>0.3</v>
@@ -2541,7 +2541,7 @@
         <v/>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="K30" s="20">
         <f>IF(I30&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2580,7 +2580,7 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.08</v>
       </c>
       <c r="H31" s="17" t="n">
         <v>0.41</v>
@@ -2590,7 +2590,7 @@
         <v/>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
       <c r="K31" s="20">
         <f>IF(I31&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2629,7 +2629,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.097</v>
       </c>
       <c r="H32" s="17" t="n">
         <v>0.44</v>
@@ -2639,7 +2639,7 @@
         <v/>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="K32" s="20">
         <f>IF(I32&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2678,7 +2678,7 @@
         <v>0.5</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0.092</v>
+        <v>0.102</v>
       </c>
       <c r="H33" s="17" t="n">
         <v>0.53</v>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
       <c r="J33" s="6" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="K33" s="20">
         <f>IF(I33&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2727,7 +2727,7 @@
         <v>0.5</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>0.12</v>
+        <v>0.133</v>
       </c>
       <c r="H34" s="17" t="n">
         <v>0.55</v>
@@ -2737,7 +2737,7 @@
         <v/>
       </c>
       <c r="J34" s="6" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="K34" s="20">
         <f>IF(I34&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2776,7 +2776,7 @@
         <v>0.5</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0.043</v>
+        <v>0.048</v>
       </c>
       <c r="H35" s="17" t="n">
         <v>0.3</v>
@@ -2786,7 +2786,7 @@
         <v/>
       </c>
       <c r="J35" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="K35" s="20">
         <f>IF(I35&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2825,7 +2825,7 @@
         <v>1.72</v>
       </c>
       <c r="G36" s="18" t="n">
-        <v>0.03</v>
+        <v>0.033</v>
       </c>
       <c r="H36" s="17" t="n">
         <v>0.3</v>
@@ -2835,7 +2835,7 @@
         <v/>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="K36" s="20">
         <f>IF(I36&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2874,7 +2874,7 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0.134</v>
+        <v>0.15</v>
       </c>
       <c r="H37" s="17" t="n">
         <v>0.5</v>
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="J37" s="6" t="n">
-        <v>0.97</v>
+        <v>1.02</v>
       </c>
       <c r="K37" s="20">
         <f>IF(I37&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2923,7 +2923,7 @@
         <v>0.5</v>
       </c>
       <c r="G38" s="18" t="n">
-        <v>0.175</v>
+        <v>0.196</v>
       </c>
       <c r="H38" s="17" t="n">
         <v>0.59</v>
@@ -2933,7 +2933,7 @@
         <v/>
       </c>
       <c r="J38" s="6" t="n">
-        <v>1.08</v>
+        <v>1.12</v>
       </c>
       <c r="K38" s="20">
         <f>IF(I38&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2972,7 +2972,7 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0.175</v>
+        <v>0.196</v>
       </c>
       <c r="H39" s="17" t="n">
         <v>0.61</v>
@@ -2982,7 +2982,7 @@
         <v/>
       </c>
       <c r="J39" s="6" t="n">
-        <v>1.08</v>
+        <v>1.12</v>
       </c>
       <c r="K39" s="20">
         <f>IF(I39&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3021,7 +3021,7 @@
         <v>0.5</v>
       </c>
       <c r="G40" s="18" t="n">
-        <v>0.207</v>
+        <v>0.233</v>
       </c>
       <c r="H40" s="17" t="n">
         <v>0.62</v>
@@ -3031,7 +3031,7 @@
         <v/>
       </c>
       <c r="J40" s="6" t="n">
-        <v>1.14</v>
+        <v>1.19</v>
       </c>
       <c r="K40" s="20">
         <f>IF(I40&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3070,7 +3070,7 @@
         <v>0.5</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0.207</v>
+        <v>0.233</v>
       </c>
       <c r="H41" s="17" t="n">
         <v>0.73</v>
@@ -3080,7 +3080,7 @@
         <v/>
       </c>
       <c r="J41" s="6" t="n">
-        <v>1.14</v>
+        <v>1.19</v>
       </c>
       <c r="K41" s="20">
         <f>IF(I41&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3119,7 +3119,7 @@
         <v>0.5</v>
       </c>
       <c r="G42" s="18" t="n">
-        <v>0.271</v>
+        <v>0.305</v>
       </c>
       <c r="H42" s="17" t="n">
         <v>0.73</v>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
       <c r="J42" s="6" t="n">
-        <v>1.25</v>
+        <v>1.29</v>
       </c>
       <c r="K42" s="20">
         <f>IF(I42&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3168,7 +3168,7 @@
         <v>0.5</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0.312</v>
+        <v>0.353</v>
       </c>
       <c r="H43" s="17" t="n">
         <v>0.79</v>
@@ -3178,7 +3178,7 @@
         <v/>
       </c>
       <c r="J43" s="6" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="K43" s="20">
         <f>IF(I43&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3217,7 +3217,7 @@
         <v>0.5</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>0.312</v>
+        <v>0.353</v>
       </c>
       <c r="H44" s="17" t="n">
         <v>0.7</v>
@@ -3227,7 +3227,7 @@
         <v/>
       </c>
       <c r="J44" s="6" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="K44" s="20">
         <f>IF(I44&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3266,7 +3266,7 @@
         <v>0.5</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>0.313</v>
+        <v>0.354</v>
       </c>
       <c r="H45" s="17" t="n">
         <v>0.7</v>
@@ -3276,7 +3276,7 @@
         <v/>
       </c>
       <c r="J45" s="6" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="K45" s="20">
         <f>IF(I45&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3315,7 +3315,7 @@
         <v>0.5</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>0.314</v>
+        <v>0.354</v>
       </c>
       <c r="H46" s="17" t="n">
         <v>0.74</v>
@@ -3325,7 +3325,7 @@
         <v/>
       </c>
       <c r="J46" s="6" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="K46" s="20">
         <f>IF(I46&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3364,7 +3364,7 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>0.315</v>
+        <v>0.356</v>
       </c>
       <c r="H47" s="17" t="n">
         <v>0.74</v>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="J47" s="6" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="K47" s="20">
         <f>IF(I47&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3413,7 +3413,7 @@
         <v>0.5</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>0.315</v>
+        <v>0.356</v>
       </c>
       <c r="H48" s="17" t="n">
         <v>0.77</v>
@@ -3423,7 +3423,7 @@
         <v/>
       </c>
       <c r="J48" s="6" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="K48" s="20">
         <f>IF(I48&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3462,7 +3462,7 @@
         <v>0.5</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>0.319</v>
+        <v>0.361</v>
       </c>
       <c r="H49" s="17" t="n">
         <v>0.77</v>
@@ -3472,7 +3472,7 @@
         <v/>
       </c>
       <c r="J49" s="6" t="n">
-        <v>1.31</v>
+        <v>1.35</v>
       </c>
       <c r="K49" s="20">
         <f>IF(I49&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3511,7 +3511,7 @@
         <v>0.5</v>
       </c>
       <c r="G50" s="18" t="n">
-        <v>0.32</v>
+        <v>0.362</v>
       </c>
       <c r="H50" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3521,7 +3521,7 @@
         <v/>
       </c>
       <c r="J50" s="6" t="n">
-        <v>1.31</v>
+        <v>1.35</v>
       </c>
       <c r="K50" s="20">
         <f>IF(I50&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3560,7 +3560,7 @@
         <v>0.5</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>0.32</v>
+        <v>0.362</v>
       </c>
       <c r="H51" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3570,7 +3570,7 @@
         <v/>
       </c>
       <c r="J51" s="6" t="n">
-        <v>1.31</v>
+        <v>1.35</v>
       </c>
       <c r="K51" s="20">
         <f>IF(I51&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3609,7 +3609,7 @@
         <v>0.5</v>
       </c>
       <c r="G52" s="18" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="H52" s="17" t="n">
         <v>0.3</v>
@@ -3619,7 +3619,7 @@
         <v/>
       </c>
       <c r="J52" s="6" t="n">
-        <v>0.43</v>
+        <v>0.45</v>
       </c>
       <c r="K52" s="20">
         <f>IF(I52&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3658,7 +3658,7 @@
         <v>0.5</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.095</v>
       </c>
       <c r="H53" s="17" t="n">
         <v>0.32</v>
@@ -3668,7 +3668,7 @@
         <v/>
       </c>
       <c r="J53" s="6" t="n">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="K53" s="20">
         <f>IF(I53&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3707,7 +3707,7 @@
         <v>0.5</v>
       </c>
       <c r="G54" s="18" t="n">
-        <v>0.073</v>
+        <v>0.081</v>
       </c>
       <c r="H54" s="17" t="n">
         <v>0.3</v>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J54" s="6" t="n">
-        <v>0.74</v>
+        <v>0.77</v>
       </c>
       <c r="K54" s="20">
         <f>IF(I54&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3756,7 +3756,7 @@
         <v>0.5</v>
       </c>
       <c r="G55" s="18" t="n">
-        <v>0.062</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H55" s="17" t="n">
         <v>0.3</v>
@@ -3766,7 +3766,7 @@
         <v/>
       </c>
       <c r="J55" s="6" t="n">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
       <c r="K55" s="20">
         <f>IF(I55&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3805,7 +3805,7 @@
         <v>0.5</v>
       </c>
       <c r="G56" s="18" t="n">
-        <v>0.068</v>
+        <v>0.075</v>
       </c>
       <c r="H56" s="17" t="n">
         <v>0.39</v>
@@ -3815,7 +3815,7 @@
         <v/>
       </c>
       <c r="J56" s="6" t="n">
-        <v>0.71</v>
+        <v>0.75</v>
       </c>
       <c r="K56" s="20">
         <f>IF(I56&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3854,7 +3854,7 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.078</v>
       </c>
       <c r="H57" s="17" t="n">
         <v>0.42</v>
@@ -3864,7 +3864,7 @@
         <v/>
       </c>
       <c r="J57" s="6" t="n">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="K57" s="20">
         <f>IF(I57&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3903,7 +3903,7 @@
         <v>0.5</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>0.091</v>
+        <v>0.101</v>
       </c>
       <c r="H58" s="17" t="n">
         <v>0.42</v>
@@ -3913,7 +3913,7 @@
         <v/>
       </c>
       <c r="J58" s="6" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="K58" s="20">
         <f>IF(I58&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3952,7 +3952,7 @@
         <v>0.5</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>0.091</v>
+        <v>0.101</v>
       </c>
       <c r="H59" s="17" t="n">
         <v>0.48</v>
@@ -3962,7 +3962,7 @@
         <v/>
       </c>
       <c r="J59" s="6" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="K59" s="20">
         <f>IF(I59&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4001,7 +4001,7 @@
         <v>0.5</v>
       </c>
       <c r="G60" s="18" t="n">
-        <v>0.081</v>
+        <v>0.09</v>
       </c>
       <c r="H60" s="17" t="n">
         <v>0.2</v>
@@ -4011,7 +4011,7 @@
         <v/>
       </c>
       <c r="J60" s="6" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K60" s="20">
         <f>IF(I60&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4050,7 +4050,7 @@
         <v>0.5</v>
       </c>
       <c r="G61" s="18" t="n">
-        <v>0.057</v>
+        <v>0.063</v>
       </c>
       <c r="H61" s="17" t="n">
         <v>0.3</v>
@@ -4060,7 +4060,7 @@
         <v/>
       </c>
       <c r="J61" s="6" t="n">
-        <v>0.65</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K61" s="20">
         <f>IF(I61&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4099,7 +4099,7 @@
         <v>0.5</v>
       </c>
       <c r="G62" s="18" t="n">
-        <v>0.06</v>
+        <v>0.066</v>
       </c>
       <c r="H62" s="17" t="n">
         <v>0.38</v>
@@ -4109,7 +4109,7 @@
         <v/>
       </c>
       <c r="J62" s="6" t="n">
-        <v>0.66</v>
+        <v>0.7</v>
       </c>
       <c r="K62" s="20">
         <f>IF(I62&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4148,7 +4148,7 @@
         <v>0.5</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>0.092</v>
+        <v>0.103</v>
       </c>
       <c r="H63" s="17" t="n">
         <v>0.38</v>
@@ -4158,7 +4158,7 @@
         <v/>
       </c>
       <c r="J63" s="6" t="n">
-        <v>0.82</v>
+        <v>0.87</v>
       </c>
       <c r="K63" s="20">
         <f>IF(I63&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4197,7 +4197,7 @@
         <v>0.5</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>0.093</v>
+        <v>0.103</v>
       </c>
       <c r="H64" s="17" t="n">
         <v>0.49</v>
@@ -4207,7 +4207,7 @@
         <v/>
       </c>
       <c r="J64" s="6" t="n">
-        <v>0.83</v>
+        <v>0.87</v>
       </c>
       <c r="K64" s="20">
         <f>IF(I64&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4246,7 +4246,7 @@
         <v>0.5</v>
       </c>
       <c r="G65" s="18" t="n">
-        <v>0.124</v>
+        <v>0.138</v>
       </c>
       <c r="H65" s="17" t="n">
         <v>0.5</v>
@@ -4256,7 +4256,7 @@
         <v/>
       </c>
       <c r="J65" s="6" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="K65" s="20">
         <f>IF(I65&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4295,7 +4295,7 @@
         <v>0.5</v>
       </c>
       <c r="G66" s="18" t="n">
-        <v>0.161</v>
+        <v>0.18</v>
       </c>
       <c r="H66" s="17" t="n">
         <v>0.52</v>
@@ -4305,7 +4305,7 @@
         <v/>
       </c>
       <c r="J66" s="6" t="n">
-        <v>1.04</v>
+        <v>1.09</v>
       </c>
       <c r="K66" s="20">
         <f>IF(I66&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4344,7 +4344,7 @@
         <v>0.5</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>0.279</v>
+        <v>0.315</v>
       </c>
       <c r="H67" s="17" t="n">
         <v>0.5600000000000001</v>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="J67" s="6" t="n">
-        <v>1.26</v>
+        <v>1.3</v>
       </c>
       <c r="K67" s="20">
         <f>IF(I67&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4393,7 +4393,7 @@
         <v>0.5</v>
       </c>
       <c r="G68" s="18" t="n">
-        <v>0.36</v>
+        <v>0.407</v>
       </c>
       <c r="H68" s="17" t="n">
         <v>0.62</v>
@@ -4403,7 +4403,7 @@
         <v/>
       </c>
       <c r="J68" s="6" t="n">
-        <v>1.35</v>
+        <v>1.39</v>
       </c>
       <c r="K68" s="20">
         <f>IF(I68&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4442,7 +4442,7 @@
         <v>0.5</v>
       </c>
       <c r="G69" s="18" t="n">
-        <v>0.38</v>
+        <v>0.43</v>
       </c>
       <c r="H69" s="17" t="n">
         <v>0.57</v>
@@ -4452,7 +4452,7 @@
         <v/>
       </c>
       <c r="J69" s="6" t="n">
-        <v>1.36</v>
+        <v>1.41</v>
       </c>
       <c r="K69" s="20">
         <f>IF(I69&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4491,7 +4491,7 @@
         <v>0.5</v>
       </c>
       <c r="G70" s="18" t="n">
-        <v>0.382</v>
+        <v>0.433</v>
       </c>
       <c r="H70" s="17" t="n">
         <v>0.63</v>
@@ -4501,7 +4501,7 @@
         <v/>
       </c>
       <c r="J70" s="6" t="n">
-        <v>1.37</v>
+        <v>1.41</v>
       </c>
       <c r="K70" s="20">
         <f>IF(I70&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4540,7 +4540,7 @@
         <v>0.5</v>
       </c>
       <c r="G71" s="18" t="n">
-        <v>0.382</v>
+        <v>0.433</v>
       </c>
       <c r="H71" s="17" t="n">
         <v>0.64</v>
@@ -4550,7 +4550,7 @@
         <v/>
       </c>
       <c r="J71" s="6" t="n">
-        <v>1.37</v>
+        <v>1.41</v>
       </c>
       <c r="K71" s="20">
         <f>IF(I71&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4589,7 +4589,7 @@
         <v>0.5</v>
       </c>
       <c r="G72" s="18" t="n">
-        <v>0.45</v>
+        <v>0.512</v>
       </c>
       <c r="H72" s="17" t="n">
         <v>0.64</v>
@@ -4599,7 +4599,7 @@
         <v/>
       </c>
       <c r="J72" s="6" t="n">
-        <v>1.42</v>
+        <v>1.46</v>
       </c>
       <c r="K72" s="20">
         <f>IF(I72&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4638,7 +4638,7 @@
         <v>0.5</v>
       </c>
       <c r="G73" s="18" t="n">
-        <v>0.064</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H73" s="17" t="n">
         <v>0.3</v>
@@ -4648,7 +4648,7 @@
         <v/>
       </c>
       <c r="J73" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.73</v>
       </c>
       <c r="K73" s="20">
         <f>IF(I73&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4687,7 +4687,7 @@
         <v>0.5</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>0.073</v>
+        <v>0.081</v>
       </c>
       <c r="H74" s="17" t="n">
         <v>0.3</v>
@@ -4697,7 +4697,7 @@
         <v/>
       </c>
       <c r="J74" s="6" t="n">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
       <c r="K74" s="20">
         <f>IF(I74&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4736,7 +4736,7 @@
         <v>0.5</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>0.075</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H75" s="17" t="n">
         <v>0.38</v>
@@ -4746,7 +4746,7 @@
         <v/>
       </c>
       <c r="J75" s="6" t="n">
-        <v>0.75</v>
+        <v>0.79</v>
       </c>
       <c r="K75" s="20">
         <f>IF(I75&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4785,7 +4785,7 @@
         <v>0.5</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>0.12</v>
+        <v>0.133</v>
       </c>
       <c r="H76" s="17" t="n">
         <v>0.35</v>
@@ -4795,7 +4795,7 @@
         <v/>
       </c>
       <c r="J76" s="6" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="K76" s="20">
         <f>IF(I76&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4834,7 +4834,7 @@
         <v>0.5</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>0.12</v>
+        <v>0.134</v>
       </c>
       <c r="H77" s="17" t="n">
         <v>0.35</v>
@@ -4844,7 +4844,7 @@
         <v/>
       </c>
       <c r="J77" s="6" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="K77" s="20">
         <f>IF(I77&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4883,7 +4883,7 @@
         <v>0.5</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>0.122</v>
+        <v>0.136</v>
       </c>
       <c r="H78" s="17" t="n">
         <v>0.35</v>
@@ -4893,7 +4893,7 @@
         <v/>
       </c>
       <c r="J78" s="6" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="K78" s="20">
         <f>IF(I78&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4932,7 +4932,7 @@
         <v>0.5</v>
       </c>
       <c r="G79" s="18" t="n">
-        <v>0.158</v>
+        <v>0.176</v>
       </c>
       <c r="H79" s="17" t="n">
         <v>0.35</v>
@@ -4942,7 +4942,7 @@
         <v/>
       </c>
       <c r="J79" s="6" t="n">
-        <v>1.04</v>
+        <v>1.08</v>
       </c>
       <c r="K79" s="20">
         <f>IF(I79&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4981,7 +4981,7 @@
         <v>0.5</v>
       </c>
       <c r="G80" s="18" t="n">
-        <v>0.161</v>
+        <v>0.181</v>
       </c>
       <c r="H80" s="17" t="n">
         <v>0.45</v>
@@ -4991,7 +4991,7 @@
         <v/>
       </c>
       <c r="J80" s="6" t="n">
-        <v>1.05</v>
+        <v>1.09</v>
       </c>
       <c r="K80" s="20">
         <f>IF(I80&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5030,7 +5030,7 @@
         <v>0.5</v>
       </c>
       <c r="G81" s="18" t="n">
-        <v>0.061</v>
+        <v>0.068</v>
       </c>
       <c r="H81" s="17" t="n">
         <v>0.3</v>
@@ -5040,7 +5040,7 @@
         <v/>
       </c>
       <c r="J81" s="6" t="n">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="K81" s="20">
         <f>IF(I81&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5079,7 +5079,7 @@
         <v>0.5</v>
       </c>
       <c r="G82" s="18" t="n">
-        <v>0.062</v>
+        <v>0.068</v>
       </c>
       <c r="H82" s="17" t="n">
         <v>0.36</v>
@@ -5089,7 +5089,7 @@
         <v/>
       </c>
       <c r="J82" s="6" t="n">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
       <c r="K82" s="20">
         <f>IF(I82&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5128,7 +5128,7 @@
         <v>0.58</v>
       </c>
       <c r="G83" s="18" t="n">
-        <v>0.117</v>
+        <v>0.13</v>
       </c>
       <c r="H83" s="17" t="n">
         <v>0.35</v>
@@ -5138,7 +5138,7 @@
         <v/>
       </c>
       <c r="J83" s="6" t="n">
-        <v>0.99</v>
+        <v>1.03</v>
       </c>
       <c r="K83" s="20">
         <f>IF(I83&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5177,7 +5177,7 @@
         <v>0.5</v>
       </c>
       <c r="G84" s="18" t="n">
-        <v>0.128</v>
+        <v>0.143</v>
       </c>
       <c r="H84" s="17" t="n">
         <v>0.35</v>
@@ -5187,7 +5187,7 @@
         <v/>
       </c>
       <c r="J84" s="6" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="K84" s="20">
         <f>IF(I84&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5226,7 +5226,7 @@
         <v>0.5</v>
       </c>
       <c r="G85" s="18" t="n">
-        <v>0.092</v>
+        <v>0.102</v>
       </c>
       <c r="H85" s="17" t="n">
         <v>0.3</v>
@@ -5236,7 +5236,7 @@
         <v/>
       </c>
       <c r="J85" s="6" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="K85" s="20">
         <f>IF(I85&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5275,7 +5275,7 @@
         <v>0.5</v>
       </c>
       <c r="G86" s="18" t="n">
-        <v>0.097</v>
+        <v>0.107</v>
       </c>
       <c r="H86" s="17" t="n">
         <v>0.45</v>
@@ -5285,7 +5285,7 @@
         <v/>
       </c>
       <c r="J86" s="6" t="n">
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="K86" s="20">
         <f>IF(I86&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5324,7 +5324,7 @@
         <v>0.5</v>
       </c>
       <c r="G87" s="18" t="n">
-        <v>0.099</v>
+        <v>0.11</v>
       </c>
       <c r="H87" s="17" t="n">
         <v>0.46</v>
@@ -5334,7 +5334,7 @@
         <v/>
       </c>
       <c r="J87" s="6" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="K87" s="20">
         <f>IF(I87&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5373,7 +5373,7 @@
         <v>0.5</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>0.099</v>
+        <v>0.11</v>
       </c>
       <c r="H88" s="17" t="n">
         <v>0.47</v>
@@ -5383,7 +5383,7 @@
         <v/>
       </c>
       <c r="J88" s="6" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="K88" s="20">
         <f>IF(I88&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5422,7 +5422,7 @@
         <v>0.5</v>
       </c>
       <c r="G89" s="18" t="n">
-        <v>0.122</v>
+        <v>0.136</v>
       </c>
       <c r="H89" s="17" t="n">
         <v>0.4</v>
@@ -5432,7 +5432,7 @@
         <v/>
       </c>
       <c r="J89" s="6" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="K89" s="20">
         <f>IF(I89&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5471,7 +5471,7 @@
         <v>0.5</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>0.122</v>
+        <v>0.136</v>
       </c>
       <c r="H90" s="17" t="n">
         <v>0.4</v>
@@ -5481,7 +5481,7 @@
         <v/>
       </c>
       <c r="J90" s="6" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="K90" s="20">
         <f>IF(I90&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5520,7 +5520,7 @@
         <v>0.51</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>0.08</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H91" s="17" t="n">
         <v>0.2</v>
@@ -5530,7 +5530,7 @@
         <v/>
       </c>
       <c r="J91" s="6" t="n">
-        <v>0.78</v>
+        <v>0.82</v>
       </c>
       <c r="K91" s="20">
         <f>IF(I91&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5569,7 +5569,7 @@
         <v>0.5</v>
       </c>
       <c r="G92" s="18" t="n">
-        <v>0.08</v>
+        <v>0.089</v>
       </c>
       <c r="H92" s="17" t="n">
         <v>0.5</v>
@@ -5579,7 +5579,7 @@
         <v/>
       </c>
       <c r="J92" s="6" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K92" s="20">
         <f>IF(I92&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5618,7 +5618,7 @@
         <v>0.5</v>
       </c>
       <c r="G93" s="18" t="n">
-        <v>0.122</v>
+        <v>0.136</v>
       </c>
       <c r="H93" s="17" t="n">
         <v>0.5</v>
@@ -5628,7 +5628,7 @@
         <v/>
       </c>
       <c r="J93" s="6" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="K93" s="20">
         <f>IF(I93&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5667,7 +5667,7 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="18" t="n">
-        <v>0.123</v>
+        <v>0.137</v>
       </c>
       <c r="H94" s="17" t="n">
         <v>0.4</v>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="J94" s="6" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="K94" s="20">
         <f>IF(I94&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5716,7 +5716,7 @@
         <v>0.5</v>
       </c>
       <c r="G95" s="18" t="n">
-        <v>0.036</v>
+        <v>0.04</v>
       </c>
       <c r="H95" s="17" t="n">
         <v>0.3</v>
@@ -5726,7 +5726,7 @@
         <v/>
       </c>
       <c r="J95" s="6" t="n">
-        <v>0.51</v>
+        <v>0.54</v>
       </c>
       <c r="K95" s="20">
         <f>IF(I95&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5765,7 +5765,7 @@
         <v>0.5</v>
       </c>
       <c r="G96" s="18" t="n">
-        <v>0.036</v>
+        <v>0.04</v>
       </c>
       <c r="H96" s="17" t="n">
         <v>0.36</v>
@@ -5775,7 +5775,7 @@
         <v/>
       </c>
       <c r="J96" s="6" t="n">
-        <v>0.51</v>
+        <v>0.54</v>
       </c>
       <c r="K96" s="20">
         <f>IF(I96&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5814,7 +5814,7 @@
         <v>0.5</v>
       </c>
       <c r="G97" s="18" t="n">
-        <v>0.058</v>
+        <v>0.064</v>
       </c>
       <c r="H97" s="17" t="n">
         <v>0.36</v>
@@ -5824,7 +5824,7 @@
         <v/>
       </c>
       <c r="J97" s="6" t="n">
-        <v>0.66</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K97" s="20">
         <f>IF(I97&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5863,7 +5863,7 @@
         <v>0.5</v>
       </c>
       <c r="G98" s="18" t="n">
-        <v>0.058</v>
+        <v>0.064</v>
       </c>
       <c r="H98" s="17" t="n">
         <v>0.48</v>
@@ -5873,7 +5873,7 @@
         <v/>
       </c>
       <c r="J98" s="6" t="n">
-        <v>0.66</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K98" s="20">
         <f>IF(I98&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5912,7 +5912,7 @@
         <v>0.5</v>
       </c>
       <c r="G99" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.079</v>
       </c>
       <c r="H99" s="17" t="n">
         <v>0.49</v>
@@ -5922,7 +5922,7 @@
         <v/>
       </c>
       <c r="J99" s="6" t="n">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
       <c r="K99" s="20">
         <f>IF(I99&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5961,7 +5961,7 @@
         <v>0.5</v>
       </c>
       <c r="G100" s="18" t="n">
-        <v>0.03</v>
+        <v>0.033</v>
       </c>
       <c r="H100" s="17" t="n">
         <v>0.3</v>
@@ -5971,7 +5971,7 @@
         <v/>
       </c>
       <c r="J100" s="6" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="K100" s="20">
         <f>IF(I100&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -6010,7 +6010,7 @@
         <v>0.5</v>
       </c>
       <c r="G101" s="18" t="n">
-        <v>0.03</v>
+        <v>0.033</v>
       </c>
       <c r="H101" s="17" t="n">
         <v>0.37</v>
@@ -6020,7 +6020,7 @@
         <v/>
       </c>
       <c r="J101" s="6" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="K101" s="20">
         <f>IF(I101&gt;=0.05,"CUMPLE","NO CUMPLE")</f>

</xml_diff>

<commit_message>
Barranquita: memoria hidrologica completa (estructura de los CAR), FS 1.15 y norma CE.040
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>I = 467 mm/h, C ponderado = 0.57, area total 9393 m2; menor borde libre 0.110 m en EJE-11 P-48-P-33 (Q 26.4 l/s, y 0.090, h 0.20)</t>
+          <t>I = 467 mm/h, C ponderado = 0.57, area total 9393 m2; menor borde libre 0.064 m en EJE-12 P-60-D2 (Q 304.4 l/s, y 0.576, h 0.64)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>V max 1.82 m/s</t>
+          <t>V max 1.90 m/s</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
         <v>0.5</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>0.092</v>
+        <v>0.102</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>0.3</v>
@@ -1610,7 +1610,7 @@
         <v/>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="K11" s="20">
         <f>IF(I11&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1649,7 +1649,7 @@
         <v>0.5</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>0.096</v>
+        <v>0.105</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>0.46</v>
@@ -1659,7 +1659,7 @@
         <v/>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="K12" s="20">
         <f>IF(I12&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1698,7 +1698,7 @@
         <v>0.5</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0.078</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>0.3</v>
@@ -1708,7 +1708,7 @@
         <v/>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.76</v>
+        <v>0.79</v>
       </c>
       <c r="K13" s="20">
         <f>IF(I13&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1747,7 +1747,7 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>0.081</v>
+        <v>0.089</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>0.46</v>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0.78</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K14" s="20">
         <f>IF(I14&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1796,7 +1796,7 @@
         <v>0.5</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.092</v>
+        <v>0.101</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>0.46</v>
@@ -1806,7 +1806,7 @@
         <v/>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="K15" s="20">
         <f>IF(I15&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1845,7 +1845,7 @@
         <v>2.92</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>0.076</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>0.52</v>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="J16" s="6" t="n">
-        <v>1.82</v>
+        <v>1.9</v>
       </c>
       <c r="K16" s="20">
         <f>IF(I16&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1894,7 +1894,7 @@
         <v>0.5</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>0.285</v>
+        <v>0.319</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>0.77</v>
@@ -1904,7 +1904,7 @@
         <v/>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1.26</v>
+        <v>1.3</v>
       </c>
       <c r="K17" s="20">
         <f>IF(I17&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1943,7 +1943,7 @@
         <v>0.5</v>
       </c>
       <c r="G18" s="18" t="n">
-        <v>0.285</v>
+        <v>0.319</v>
       </c>
       <c r="H18" s="17" t="n">
         <v>0.83</v>
@@ -1953,7 +1953,7 @@
         <v/>
       </c>
       <c r="J18" s="6" t="n">
-        <v>1.26</v>
+        <v>1.3</v>
       </c>
       <c r="K18" s="20">
         <f>IF(I18&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1992,7 +1992,7 @@
         <v>0.5</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>0.37</v>
+        <v>0.414</v>
       </c>
       <c r="H19" s="17" t="n">
         <v>0.83</v>
@@ -2002,7 +2002,7 @@
         <v/>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1.36</v>
+        <v>1.39</v>
       </c>
       <c r="K19" s="20">
         <f>IF(I19&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2041,7 +2041,7 @@
         <v>0.5</v>
       </c>
       <c r="G20" s="18" t="n">
-        <v>0.37</v>
+        <v>0.414</v>
       </c>
       <c r="H20" s="17" t="n">
         <v>0.79</v>
@@ -2051,7 +2051,7 @@
         <v/>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.36</v>
+        <v>1.39</v>
       </c>
       <c r="K20" s="20">
         <f>IF(I20&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2090,7 +2090,7 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>0.418</v>
+        <v>0.469</v>
       </c>
       <c r="H21" s="17" t="n">
         <v>0.79</v>
@@ -2100,7 +2100,7 @@
         <v/>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1.4</v>
+        <v>1.43</v>
       </c>
       <c r="K21" s="20">
         <f>IF(I21&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2139,7 +2139,7 @@
         <v>0.5</v>
       </c>
       <c r="G22" s="18" t="n">
-        <v>0.073</v>
+        <v>0.08</v>
       </c>
       <c r="H22" s="17" t="n">
         <v>0.3</v>
@@ -2149,7 +2149,7 @@
         <v/>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
       <c r="K22" s="20">
         <f>IF(I22&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2188,7 +2188,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0.092</v>
+        <v>0.101</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>0.3</v>
@@ -2198,7 +2198,7 @@
         <v/>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="K23" s="20">
         <f>IF(I23&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2237,7 +2237,7 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="18" t="n">
-        <v>0.099</v>
+        <v>0.109</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>0.43</v>
@@ -2247,7 +2247,7 @@
         <v/>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="K24" s="20">
         <f>IF(I24&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2286,7 +2286,7 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="H25" s="17" t="n">
         <v>0.47</v>
@@ -2296,7 +2296,7 @@
         <v/>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="K25" s="20">
         <f>IF(I25&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2335,7 +2335,7 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="18" t="n">
-        <v>0.124</v>
+        <v>0.138</v>
       </c>
       <c r="H26" s="17" t="n">
         <v>0.48</v>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="K26" s="20">
         <f>IF(I26&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2384,7 +2384,7 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0.147</v>
+        <v>0.162</v>
       </c>
       <c r="H27" s="17" t="n">
         <v>0.49</v>
@@ -2394,7 +2394,7 @@
         <v/>
       </c>
       <c r="J27" s="6" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="K27" s="20">
         <f>IF(I27&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2433,7 +2433,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="18" t="n">
-        <v>0.156</v>
+        <v>0.172</v>
       </c>
       <c r="H28" s="17" t="n">
         <v>0.57</v>
@@ -2443,7 +2443,7 @@
         <v/>
       </c>
       <c r="J28" s="6" t="n">
-        <v>1.03</v>
+        <v>1.07</v>
       </c>
       <c r="K28" s="20">
         <f>IF(I28&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2482,7 +2482,7 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0.187</v>
+        <v>0.207</v>
       </c>
       <c r="H29" s="17" t="n">
         <v>0.61</v>
@@ -2492,7 +2492,7 @@
         <v/>
       </c>
       <c r="J29" s="6" t="n">
-        <v>1.1</v>
+        <v>1.14</v>
       </c>
       <c r="K29" s="20">
         <f>IF(I29&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2531,7 +2531,7 @@
         <v>0.5</v>
       </c>
       <c r="G30" s="18" t="n">
-        <v>0.074</v>
+        <v>0.081</v>
       </c>
       <c r="H30" s="17" t="n">
         <v>0.3</v>
@@ -2541,7 +2541,7 @@
         <v/>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.74</v>
+        <v>0.78</v>
       </c>
       <c r="K30" s="20">
         <f>IF(I30&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2580,7 +2580,7 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0.08</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H31" s="17" t="n">
         <v>0.41</v>
@@ -2590,7 +2590,7 @@
         <v/>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K31" s="20">
         <f>IF(I31&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2629,7 +2629,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="18" t="n">
-        <v>0.097</v>
+        <v>0.106</v>
       </c>
       <c r="H32" s="17" t="n">
         <v>0.44</v>
@@ -2639,7 +2639,7 @@
         <v/>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="K32" s="20">
         <f>IF(I32&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2678,7 +2678,7 @@
         <v>0.5</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0.102</v>
+        <v>0.112</v>
       </c>
       <c r="H33" s="17" t="n">
         <v>0.53</v>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
       <c r="J33" s="6" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="K33" s="20">
         <f>IF(I33&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2727,7 +2727,7 @@
         <v>0.5</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>0.133</v>
+        <v>0.148</v>
       </c>
       <c r="H34" s="17" t="n">
         <v>0.55</v>
@@ -2737,7 +2737,7 @@
         <v/>
       </c>
       <c r="J34" s="6" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="K34" s="20">
         <f>IF(I34&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2776,7 +2776,7 @@
         <v>0.5</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0.048</v>
+        <v>0.052</v>
       </c>
       <c r="H35" s="17" t="n">
         <v>0.3</v>
@@ -2786,7 +2786,7 @@
         <v/>
       </c>
       <c r="J35" s="6" t="n">
-        <v>0.59</v>
+        <v>0.62</v>
       </c>
       <c r="K35" s="20">
         <f>IF(I35&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2825,7 +2825,7 @@
         <v>1.72</v>
       </c>
       <c r="G36" s="18" t="n">
-        <v>0.033</v>
+        <v>0.036</v>
       </c>
       <c r="H36" s="17" t="n">
         <v>0.3</v>
@@ -2835,7 +2835,7 @@
         <v/>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0.88</v>
+        <v>0.93</v>
       </c>
       <c r="K36" s="20">
         <f>IF(I36&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2874,7 +2874,7 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0.15</v>
+        <v>0.166</v>
       </c>
       <c r="H37" s="17" t="n">
         <v>0.5</v>
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="J37" s="6" t="n">
-        <v>1.02</v>
+        <v>1.06</v>
       </c>
       <c r="K37" s="20">
         <f>IF(I37&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2923,7 +2923,7 @@
         <v>0.5</v>
       </c>
       <c r="G38" s="18" t="n">
-        <v>0.196</v>
+        <v>0.218</v>
       </c>
       <c r="H38" s="17" t="n">
         <v>0.59</v>
@@ -2933,7 +2933,7 @@
         <v/>
       </c>
       <c r="J38" s="6" t="n">
-        <v>1.12</v>
+        <v>1.16</v>
       </c>
       <c r="K38" s="20">
         <f>IF(I38&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2972,7 +2972,7 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0.196</v>
+        <v>0.218</v>
       </c>
       <c r="H39" s="17" t="n">
         <v>0.61</v>
@@ -2982,7 +2982,7 @@
         <v/>
       </c>
       <c r="J39" s="6" t="n">
-        <v>1.12</v>
+        <v>1.16</v>
       </c>
       <c r="K39" s="20">
         <f>IF(I39&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3021,7 +3021,7 @@
         <v>0.5</v>
       </c>
       <c r="G40" s="18" t="n">
-        <v>0.233</v>
+        <v>0.259</v>
       </c>
       <c r="H40" s="17" t="n">
         <v>0.62</v>
@@ -3031,7 +3031,7 @@
         <v/>
       </c>
       <c r="J40" s="6" t="n">
-        <v>1.19</v>
+        <v>1.23</v>
       </c>
       <c r="K40" s="20">
         <f>IF(I40&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3070,7 +3070,7 @@
         <v>0.5</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0.233</v>
+        <v>0.259</v>
       </c>
       <c r="H41" s="17" t="n">
         <v>0.73</v>
@@ -3080,7 +3080,7 @@
         <v/>
       </c>
       <c r="J41" s="6" t="n">
-        <v>1.19</v>
+        <v>1.23</v>
       </c>
       <c r="K41" s="20">
         <f>IF(I41&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3119,7 +3119,7 @@
         <v>0.5</v>
       </c>
       <c r="G42" s="18" t="n">
-        <v>0.305</v>
+        <v>0.341</v>
       </c>
       <c r="H42" s="17" t="n">
         <v>0.73</v>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
       <c r="J42" s="6" t="n">
-        <v>1.29</v>
+        <v>1.33</v>
       </c>
       <c r="K42" s="20">
         <f>IF(I42&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3168,7 +3168,7 @@
         <v>0.5</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0.353</v>
+        <v>0.395</v>
       </c>
       <c r="H43" s="17" t="n">
         <v>0.79</v>
@@ -3178,7 +3178,7 @@
         <v/>
       </c>
       <c r="J43" s="6" t="n">
-        <v>1.34</v>
+        <v>1.38</v>
       </c>
       <c r="K43" s="20">
         <f>IF(I43&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3217,7 +3217,7 @@
         <v>0.5</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>0.353</v>
+        <v>0.395</v>
       </c>
       <c r="H44" s="17" t="n">
         <v>0.7</v>
@@ -3227,7 +3227,7 @@
         <v/>
       </c>
       <c r="J44" s="6" t="n">
-        <v>1.34</v>
+        <v>1.38</v>
       </c>
       <c r="K44" s="20">
         <f>IF(I44&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3266,7 +3266,7 @@
         <v>0.5</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>0.354</v>
+        <v>0.396</v>
       </c>
       <c r="H45" s="17" t="n">
         <v>0.7</v>
@@ -3276,7 +3276,7 @@
         <v/>
       </c>
       <c r="J45" s="6" t="n">
-        <v>1.34</v>
+        <v>1.38</v>
       </c>
       <c r="K45" s="20">
         <f>IF(I45&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3315,7 +3315,7 @@
         <v>0.5</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>0.354</v>
+        <v>0.397</v>
       </c>
       <c r="H46" s="17" t="n">
         <v>0.74</v>
@@ -3325,7 +3325,7 @@
         <v/>
       </c>
       <c r="J46" s="6" t="n">
-        <v>1.34</v>
+        <v>1.38</v>
       </c>
       <c r="K46" s="20">
         <f>IF(I46&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3364,7 +3364,7 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>0.356</v>
+        <v>0.399</v>
       </c>
       <c r="H47" s="17" t="n">
         <v>0.74</v>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="J47" s="6" t="n">
-        <v>1.34</v>
+        <v>1.38</v>
       </c>
       <c r="K47" s="20">
         <f>IF(I47&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3413,7 +3413,7 @@
         <v>0.5</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>0.356</v>
+        <v>0.399</v>
       </c>
       <c r="H48" s="17" t="n">
         <v>0.77</v>
@@ -3423,7 +3423,7 @@
         <v/>
       </c>
       <c r="J48" s="6" t="n">
-        <v>1.34</v>
+        <v>1.38</v>
       </c>
       <c r="K48" s="20">
         <f>IF(I48&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3462,7 +3462,7 @@
         <v>0.5</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>0.361</v>
+        <v>0.404</v>
       </c>
       <c r="H49" s="17" t="n">
         <v>0.77</v>
@@ -3472,7 +3472,7 @@
         <v/>
       </c>
       <c r="J49" s="6" t="n">
-        <v>1.35</v>
+        <v>1.39</v>
       </c>
       <c r="K49" s="20">
         <f>IF(I49&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3511,7 +3511,7 @@
         <v>0.5</v>
       </c>
       <c r="G50" s="18" t="n">
-        <v>0.362</v>
+        <v>0.406</v>
       </c>
       <c r="H50" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3521,7 +3521,7 @@
         <v/>
       </c>
       <c r="J50" s="6" t="n">
-        <v>1.35</v>
+        <v>1.39</v>
       </c>
       <c r="K50" s="20">
         <f>IF(I50&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3560,7 +3560,7 @@
         <v>0.5</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>0.362</v>
+        <v>0.406</v>
       </c>
       <c r="H51" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3570,7 +3570,7 @@
         <v/>
       </c>
       <c r="J51" s="6" t="n">
-        <v>1.35</v>
+        <v>1.39</v>
       </c>
       <c r="K51" s="20">
         <f>IF(I51&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3609,7 +3609,7 @@
         <v>0.5</v>
       </c>
       <c r="G52" s="18" t="n">
-        <v>0.03</v>
+        <v>0.033</v>
       </c>
       <c r="H52" s="17" t="n">
         <v>0.3</v>
@@ -3619,7 +3619,7 @@
         <v/>
       </c>
       <c r="J52" s="6" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="K52" s="20">
         <f>IF(I52&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3658,7 +3658,7 @@
         <v>0.5</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>0.095</v>
+        <v>0.105</v>
       </c>
       <c r="H53" s="17" t="n">
         <v>0.32</v>
@@ -3668,7 +3668,7 @@
         <v/>
       </c>
       <c r="J53" s="6" t="n">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="K53" s="20">
         <f>IF(I53&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3707,7 +3707,7 @@
         <v>0.5</v>
       </c>
       <c r="G54" s="18" t="n">
-        <v>0.081</v>
+        <v>0.089</v>
       </c>
       <c r="H54" s="17" t="n">
         <v>0.3</v>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J54" s="6" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K54" s="20">
         <f>IF(I54&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3756,7 +3756,7 @@
         <v>0.5</v>
       </c>
       <c r="G55" s="18" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.075</v>
       </c>
       <c r="H55" s="17" t="n">
         <v>0.3</v>
@@ -3766,7 +3766,7 @@
         <v/>
       </c>
       <c r="J55" s="6" t="n">
-        <v>0.71</v>
+        <v>0.75</v>
       </c>
       <c r="K55" s="20">
         <f>IF(I55&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3805,7 +3805,7 @@
         <v>0.5</v>
       </c>
       <c r="G56" s="18" t="n">
-        <v>0.075</v>
+        <v>0.082</v>
       </c>
       <c r="H56" s="17" t="n">
         <v>0.39</v>
@@ -3815,7 +3815,7 @@
         <v/>
       </c>
       <c r="J56" s="6" t="n">
-        <v>0.75</v>
+        <v>0.78</v>
       </c>
       <c r="K56" s="20">
         <f>IF(I56&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3854,7 +3854,7 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="18" t="n">
-        <v>0.078</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H57" s="17" t="n">
         <v>0.42</v>
@@ -3864,7 +3864,7 @@
         <v/>
       </c>
       <c r="J57" s="6" t="n">
-        <v>0.76</v>
+        <v>0.8</v>
       </c>
       <c r="K57" s="20">
         <f>IF(I57&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3903,7 +3903,7 @@
         <v>0.5</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>0.101</v>
+        <v>0.111</v>
       </c>
       <c r="H58" s="17" t="n">
         <v>0.42</v>
@@ -3913,7 +3913,7 @@
         <v/>
       </c>
       <c r="J58" s="6" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="K58" s="20">
         <f>IF(I58&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3952,7 +3952,7 @@
         <v>0.5</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>0.101</v>
+        <v>0.111</v>
       </c>
       <c r="H59" s="17" t="n">
         <v>0.48</v>
@@ -3962,7 +3962,7 @@
         <v/>
       </c>
       <c r="J59" s="6" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="K59" s="20">
         <f>IF(I59&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4001,7 +4001,7 @@
         <v>0.5</v>
       </c>
       <c r="G60" s="18" t="n">
-        <v>0.09</v>
+        <v>0.099</v>
       </c>
       <c r="H60" s="17" t="n">
         <v>0.2</v>
@@ -4011,7 +4011,7 @@
         <v/>
       </c>
       <c r="J60" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="K60" s="20">
         <f>IF(I60&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4050,7 +4050,7 @@
         <v>0.5</v>
       </c>
       <c r="G61" s="18" t="n">
-        <v>0.063</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H61" s="17" t="n">
         <v>0.3</v>
@@ -4060,7 +4060,7 @@
         <v/>
       </c>
       <c r="J61" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.72</v>
       </c>
       <c r="K61" s="20">
         <f>IF(I61&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4099,7 +4099,7 @@
         <v>0.5</v>
       </c>
       <c r="G62" s="18" t="n">
-        <v>0.066</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H62" s="17" t="n">
         <v>0.38</v>
@@ -4109,7 +4109,7 @@
         <v/>
       </c>
       <c r="J62" s="6" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="K62" s="20">
         <f>IF(I62&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4148,7 +4148,7 @@
         <v>0.5</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>0.103</v>
+        <v>0.113</v>
       </c>
       <c r="H63" s="17" t="n">
         <v>0.38</v>
@@ -4158,7 +4158,7 @@
         <v/>
       </c>
       <c r="J63" s="6" t="n">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="K63" s="20">
         <f>IF(I63&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4197,7 +4197,7 @@
         <v>0.5</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>0.103</v>
+        <v>0.113</v>
       </c>
       <c r="H64" s="17" t="n">
         <v>0.49</v>
@@ -4207,7 +4207,7 @@
         <v/>
       </c>
       <c r="J64" s="6" t="n">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="K64" s="20">
         <f>IF(I64&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4246,7 +4246,7 @@
         <v>0.5</v>
       </c>
       <c r="G65" s="18" t="n">
-        <v>0.138</v>
+        <v>0.153</v>
       </c>
       <c r="H65" s="17" t="n">
         <v>0.5</v>
@@ -4256,7 +4256,7 @@
         <v/>
       </c>
       <c r="J65" s="6" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="K65" s="20">
         <f>IF(I65&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4295,7 +4295,7 @@
         <v>0.5</v>
       </c>
       <c r="G66" s="18" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="H66" s="17" t="n">
         <v>0.52</v>
@@ -4305,7 +4305,7 @@
         <v/>
       </c>
       <c r="J66" s="6" t="n">
-        <v>1.09</v>
+        <v>1.13</v>
       </c>
       <c r="K66" s="20">
         <f>IF(I66&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4344,7 +4344,7 @@
         <v>0.5</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>0.315</v>
+        <v>0.352</v>
       </c>
       <c r="H67" s="17" t="n">
         <v>0.5600000000000001</v>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="J67" s="6" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="K67" s="20">
         <f>IF(I67&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4393,7 +4393,7 @@
         <v>0.5</v>
       </c>
       <c r="G68" s="18" t="n">
-        <v>0.407</v>
+        <v>0.457</v>
       </c>
       <c r="H68" s="17" t="n">
         <v>0.62</v>
@@ -4403,7 +4403,7 @@
         <v/>
       </c>
       <c r="J68" s="6" t="n">
-        <v>1.39</v>
+        <v>1.42</v>
       </c>
       <c r="K68" s="20">
         <f>IF(I68&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4442,7 +4442,7 @@
         <v>0.5</v>
       </c>
       <c r="G69" s="18" t="n">
-        <v>0.43</v>
+        <v>0.483</v>
       </c>
       <c r="H69" s="17" t="n">
         <v>0.57</v>
@@ -4452,7 +4452,7 @@
         <v/>
       </c>
       <c r="J69" s="6" t="n">
-        <v>1.41</v>
+        <v>1.44</v>
       </c>
       <c r="K69" s="20">
         <f>IF(I69&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4491,7 +4491,7 @@
         <v>0.5</v>
       </c>
       <c r="G70" s="18" t="n">
-        <v>0.433</v>
+        <v>0.486</v>
       </c>
       <c r="H70" s="17" t="n">
         <v>0.63</v>
@@ -4501,7 +4501,7 @@
         <v/>
       </c>
       <c r="J70" s="6" t="n">
-        <v>1.41</v>
+        <v>1.44</v>
       </c>
       <c r="K70" s="20">
         <f>IF(I70&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4540,7 +4540,7 @@
         <v>0.5</v>
       </c>
       <c r="G71" s="18" t="n">
-        <v>0.433</v>
+        <v>0.486</v>
       </c>
       <c r="H71" s="17" t="n">
         <v>0.64</v>
@@ -4550,7 +4550,7 @@
         <v/>
       </c>
       <c r="J71" s="6" t="n">
-        <v>1.41</v>
+        <v>1.44</v>
       </c>
       <c r="K71" s="20">
         <f>IF(I71&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4589,7 +4589,7 @@
         <v>0.5</v>
       </c>
       <c r="G72" s="18" t="n">
-        <v>0.512</v>
+        <v>0.576</v>
       </c>
       <c r="H72" s="17" t="n">
         <v>0.64</v>
@@ -4599,7 +4599,7 @@
         <v/>
       </c>
       <c r="J72" s="6" t="n">
-        <v>1.46</v>
+        <v>1.49</v>
       </c>
       <c r="K72" s="20">
         <f>IF(I72&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4638,7 +4638,7 @@
         <v>0.5</v>
       </c>
       <c r="G73" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.078</v>
       </c>
       <c r="H73" s="17" t="n">
         <v>0.3</v>
@@ -4648,7 +4648,7 @@
         <v/>
       </c>
       <c r="J73" s="6" t="n">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="K73" s="20">
         <f>IF(I73&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4687,7 +4687,7 @@
         <v>0.5</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>0.081</v>
+        <v>0.089</v>
       </c>
       <c r="H74" s="17" t="n">
         <v>0.3</v>
@@ -4697,7 +4697,7 @@
         <v/>
       </c>
       <c r="J74" s="6" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K74" s="20">
         <f>IF(I74&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4736,7 +4736,7 @@
         <v>0.5</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.092</v>
       </c>
       <c r="H75" s="17" t="n">
         <v>0.38</v>
@@ -4746,7 +4746,7 @@
         <v/>
       </c>
       <c r="J75" s="6" t="n">
-        <v>0.79</v>
+        <v>0.82</v>
       </c>
       <c r="K75" s="20">
         <f>IF(I75&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4785,7 +4785,7 @@
         <v>0.5</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>0.133</v>
+        <v>0.147</v>
       </c>
       <c r="H76" s="17" t="n">
         <v>0.35</v>
@@ -4795,7 +4795,7 @@
         <v/>
       </c>
       <c r="J76" s="6" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="K76" s="20">
         <f>IF(I76&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4834,7 +4834,7 @@
         <v>0.5</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>0.134</v>
+        <v>0.148</v>
       </c>
       <c r="H77" s="17" t="n">
         <v>0.35</v>
@@ -4844,7 +4844,7 @@
         <v/>
       </c>
       <c r="J77" s="6" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="K77" s="20">
         <f>IF(I77&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4883,7 +4883,7 @@
         <v>0.5</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>0.136</v>
+        <v>0.15</v>
       </c>
       <c r="H78" s="17" t="n">
         <v>0.35</v>
@@ -4893,7 +4893,7 @@
         <v/>
       </c>
       <c r="J78" s="6" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="K78" s="20">
         <f>IF(I78&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4932,7 +4932,7 @@
         <v>0.5</v>
       </c>
       <c r="G79" s="18" t="n">
-        <v>0.176</v>
+        <v>0.196</v>
       </c>
       <c r="H79" s="17" t="n">
         <v>0.35</v>
@@ -4942,7 +4942,7 @@
         <v/>
       </c>
       <c r="J79" s="6" t="n">
-        <v>1.08</v>
+        <v>1.12</v>
       </c>
       <c r="K79" s="20">
         <f>IF(I79&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4981,7 +4981,7 @@
         <v>0.5</v>
       </c>
       <c r="G80" s="18" t="n">
-        <v>0.181</v>
+        <v>0.2</v>
       </c>
       <c r="H80" s="17" t="n">
         <v>0.45</v>
@@ -4991,7 +4991,7 @@
         <v/>
       </c>
       <c r="J80" s="6" t="n">
-        <v>1.09</v>
+        <v>1.13</v>
       </c>
       <c r="K80" s="20">
         <f>IF(I80&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5030,7 +5030,7 @@
         <v>0.5</v>
       </c>
       <c r="G81" s="18" t="n">
-        <v>0.068</v>
+        <v>0.075</v>
       </c>
       <c r="H81" s="17" t="n">
         <v>0.3</v>
@@ -5040,7 +5040,7 @@
         <v/>
       </c>
       <c r="J81" s="6" t="n">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
       <c r="K81" s="20">
         <f>IF(I81&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5079,7 +5079,7 @@
         <v>0.5</v>
       </c>
       <c r="G82" s="18" t="n">
-        <v>0.068</v>
+        <v>0.075</v>
       </c>
       <c r="H82" s="17" t="n">
         <v>0.36</v>
@@ -5089,7 +5089,7 @@
         <v/>
       </c>
       <c r="J82" s="6" t="n">
-        <v>0.71</v>
+        <v>0.75</v>
       </c>
       <c r="K82" s="20">
         <f>IF(I82&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5128,7 +5128,7 @@
         <v>0.58</v>
       </c>
       <c r="G83" s="18" t="n">
-        <v>0.13</v>
+        <v>0.144</v>
       </c>
       <c r="H83" s="17" t="n">
         <v>0.35</v>
@@ -5138,7 +5138,7 @@
         <v/>
       </c>
       <c r="J83" s="6" t="n">
-        <v>1.03</v>
+        <v>1.08</v>
       </c>
       <c r="K83" s="20">
         <f>IF(I83&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5177,7 +5177,7 @@
         <v>0.5</v>
       </c>
       <c r="G84" s="18" t="n">
-        <v>0.143</v>
+        <v>0.158</v>
       </c>
       <c r="H84" s="17" t="n">
         <v>0.35</v>
@@ -5187,7 +5187,7 @@
         <v/>
       </c>
       <c r="J84" s="6" t="n">
-        <v>1</v>
+        <v>1.04</v>
       </c>
       <c r="K84" s="20">
         <f>IF(I84&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5226,7 +5226,7 @@
         <v>0.5</v>
       </c>
       <c r="G85" s="18" t="n">
-        <v>0.102</v>
+        <v>0.113</v>
       </c>
       <c r="H85" s="17" t="n">
         <v>0.3</v>
@@ -5236,7 +5236,7 @@
         <v/>
       </c>
       <c r="J85" s="6" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="K85" s="20">
         <f>IF(I85&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5275,7 +5275,7 @@
         <v>0.5</v>
       </c>
       <c r="G86" s="18" t="n">
-        <v>0.107</v>
+        <v>0.119</v>
       </c>
       <c r="H86" s="17" t="n">
         <v>0.45</v>
@@ -5285,7 +5285,7 @@
         <v/>
       </c>
       <c r="J86" s="6" t="n">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="K86" s="20">
         <f>IF(I86&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5324,7 +5324,7 @@
         <v>0.5</v>
       </c>
       <c r="G87" s="18" t="n">
-        <v>0.11</v>
+        <v>0.121</v>
       </c>
       <c r="H87" s="17" t="n">
         <v>0.46</v>
@@ -5334,7 +5334,7 @@
         <v/>
       </c>
       <c r="J87" s="6" t="n">
-        <v>0.89</v>
+        <v>0.93</v>
       </c>
       <c r="K87" s="20">
         <f>IF(I87&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5373,7 +5373,7 @@
         <v>0.5</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>0.11</v>
+        <v>0.121</v>
       </c>
       <c r="H88" s="17" t="n">
         <v>0.47</v>
@@ -5383,7 +5383,7 @@
         <v/>
       </c>
       <c r="J88" s="6" t="n">
-        <v>0.89</v>
+        <v>0.93</v>
       </c>
       <c r="K88" s="20">
         <f>IF(I88&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5422,7 +5422,7 @@
         <v>0.5</v>
       </c>
       <c r="G89" s="18" t="n">
-        <v>0.136</v>
+        <v>0.15</v>
       </c>
       <c r="H89" s="17" t="n">
         <v>0.4</v>
@@ -5432,7 +5432,7 @@
         <v/>
       </c>
       <c r="J89" s="6" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="K89" s="20">
         <f>IF(I89&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5471,7 +5471,7 @@
         <v>0.5</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>0.136</v>
+        <v>0.15</v>
       </c>
       <c r="H90" s="17" t="n">
         <v>0.4</v>
@@ -5481,7 +5481,7 @@
         <v/>
       </c>
       <c r="J90" s="6" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="K90" s="20">
         <f>IF(I90&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5520,7 +5520,7 @@
         <v>0.51</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.097</v>
       </c>
       <c r="H91" s="17" t="n">
         <v>0.2</v>
@@ -5530,7 +5530,7 @@
         <v/>
       </c>
       <c r="J91" s="6" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="K91" s="20">
         <f>IF(I91&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5569,7 +5569,7 @@
         <v>0.5</v>
       </c>
       <c r="G92" s="18" t="n">
-        <v>0.089</v>
+        <v>0.098</v>
       </c>
       <c r="H92" s="17" t="n">
         <v>0.5</v>
@@ -5579,7 +5579,7 @@
         <v/>
       </c>
       <c r="J92" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="K92" s="20">
         <f>IF(I92&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5618,7 +5618,7 @@
         <v>0.5</v>
       </c>
       <c r="G93" s="18" t="n">
-        <v>0.136</v>
+        <v>0.151</v>
       </c>
       <c r="H93" s="17" t="n">
         <v>0.5</v>
@@ -5628,7 +5628,7 @@
         <v/>
       </c>
       <c r="J93" s="6" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="K93" s="20">
         <f>IF(I93&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5667,7 +5667,7 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="18" t="n">
-        <v>0.137</v>
+        <v>0.151</v>
       </c>
       <c r="H94" s="17" t="n">
         <v>0.4</v>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="J94" s="6" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="K94" s="20">
         <f>IF(I94&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5716,7 +5716,7 @@
         <v>0.5</v>
       </c>
       <c r="G95" s="18" t="n">
-        <v>0.04</v>
+        <v>0.044</v>
       </c>
       <c r="H95" s="17" t="n">
         <v>0.3</v>
@@ -5726,7 +5726,7 @@
         <v/>
       </c>
       <c r="J95" s="6" t="n">
-        <v>0.54</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K95" s="20">
         <f>IF(I95&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5765,7 +5765,7 @@
         <v>0.5</v>
       </c>
       <c r="G96" s="18" t="n">
-        <v>0.04</v>
+        <v>0.044</v>
       </c>
       <c r="H96" s="17" t="n">
         <v>0.36</v>
@@ -5775,7 +5775,7 @@
         <v/>
       </c>
       <c r="J96" s="6" t="n">
-        <v>0.54</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K96" s="20">
         <f>IF(I96&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5814,7 +5814,7 @@
         <v>0.5</v>
       </c>
       <c r="G97" s="18" t="n">
-        <v>0.064</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H97" s="17" t="n">
         <v>0.36</v>
@@ -5824,7 +5824,7 @@
         <v/>
       </c>
       <c r="J97" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.72</v>
       </c>
       <c r="K97" s="20">
         <f>IF(I97&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5863,7 +5863,7 @@
         <v>0.5</v>
       </c>
       <c r="G98" s="18" t="n">
-        <v>0.064</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H98" s="17" t="n">
         <v>0.48</v>
@@ -5873,7 +5873,7 @@
         <v/>
       </c>
       <c r="J98" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.72</v>
       </c>
       <c r="K98" s="20">
         <f>IF(I98&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5912,7 +5912,7 @@
         <v>0.5</v>
       </c>
       <c r="G99" s="18" t="n">
-        <v>0.079</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H99" s="17" t="n">
         <v>0.49</v>
@@ -5922,7 +5922,7 @@
         <v/>
       </c>
       <c r="J99" s="6" t="n">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="K99" s="20">
         <f>IF(I99&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5961,7 +5961,7 @@
         <v>0.5</v>
       </c>
       <c r="G100" s="18" t="n">
-        <v>0.033</v>
+        <v>0.036</v>
       </c>
       <c r="H100" s="17" t="n">
         <v>0.3</v>
@@ -5971,7 +5971,7 @@
         <v/>
       </c>
       <c r="J100" s="6" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="K100" s="20">
         <f>IF(I100&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -6010,7 +6010,7 @@
         <v>0.5</v>
       </c>
       <c r="G101" s="18" t="n">
-        <v>0.033</v>
+        <v>0.036</v>
       </c>
       <c r="H101" s="17" t="n">
         <v>0.37</v>
@@ -6020,7 +6020,7 @@
         <v/>
       </c>
       <c r="J101" s="6" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="K101" s="20">
         <f>IF(I101&gt;=0.05,"CUMPLE","NO CUMPLE")</f>

</xml_diff>

<commit_message>
Barranquita: lluvia de diseno con la serie medida de Pongo de Caynarachi 1989-2013 (25 anios)
Gumbel T 25: P24 166.64 mm, I 288.63 mm/h (antes Tarapoto transpuesta 269.62 mm, 467 mm/h).
Cunetas 0.40/0.60 cumplen en 91 tramos; Q max 188.1 l/s, borde libre min 0.129 m.
Metrado y especificaciones sin cambios. Memorias, memoria de calculo y cuadro de tramos actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015PDqx6f7E7zQjSSBqaUPou
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>I = 467 mm/h, C ponderado = 0.57, area total 9393 m2; menor borde libre 0.064 m en EJE-12 P-60-D2 (Q 304.4 l/s, y 0.576, h 0.64)</t>
+          <t>I = 289 mm/h, C ponderado = 0.57, area total 9393 m2; menor borde libre 0.129 m en EJE-11 P-48-P-33 (Q 18.8 l/s, y 0.071, h 0.20)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>V max 1.90 m/s</t>
+          <t>V max 1.62 m/s</t>
         </is>
       </c>
     </row>
@@ -1476,17 +1476,17 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>467</v>
+        <v>288.63</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>P max 24 h transpuesta (mm)</t>
+          <t>P max 24 h, T = 25 anos, Pongo de Caynarachi (mm)</t>
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>269.62</v>
+        <v>166.64</v>
       </c>
     </row>
     <row r="7">
@@ -1502,7 +1502,7 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>I: tc = 10 min, TR = 25 anos, P10 = 77.83 mm (estacion usada en el Hogar de Refugio - Morales); reemplazar por la del proyecto. Area tributaria: cada m2 dentro del cerco a la cuneta mas cercana.</t>
+          <t>I: tc = 10 min, TR = 25 anos, P10 = 48.11 mm (estacion Pongo de Caynarachi, SENAMHI 003317, 1989-2013; Dick y Peschke). Area tributaria: cada m2 dentro del cerco a la cuneta mas cercana.</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
         <v>0.5</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>0.102</v>
+        <v>0.073</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>0.3</v>
@@ -1610,7 +1610,7 @@
         <v/>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0.86</v>
+        <v>0.74</v>
       </c>
       <c r="K11" s="20">
         <f>IF(I11&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1649,7 +1649,7 @@
         <v>0.5</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>0.105</v>
+        <v>0.076</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>0.46</v>
@@ -1659,7 +1659,7 @@
         <v/>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.88</v>
+        <v>0.75</v>
       </c>
       <c r="K12" s="20">
         <f>IF(I12&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1698,7 +1698,7 @@
         <v>0.5</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.062</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>0.3</v>
@@ -1708,7 +1708,7 @@
         <v/>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.79</v>
+        <v>0.68</v>
       </c>
       <c r="K13" s="20">
         <f>IF(I13&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1747,7 +1747,7 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>0.089</v>
+        <v>0.065</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>0.46</v>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K14" s="20">
         <f>IF(I14&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1796,7 +1796,7 @@
         <v>0.5</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.101</v>
+        <v>0.073</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>0.46</v>
@@ -1806,7 +1806,7 @@
         <v/>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.86</v>
+        <v>0.74</v>
       </c>
       <c r="K15" s="20">
         <f>IF(I15&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1845,7 +1845,7 @@
         <v>2.92</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.061</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>0.52</v>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="J16" s="6" t="n">
-        <v>1.9</v>
+        <v>1.62</v>
       </c>
       <c r="K16" s="20">
         <f>IF(I16&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1894,7 +1894,7 @@
         <v>0.5</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>0.319</v>
+        <v>0.219</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>0.77</v>
@@ -1904,7 +1904,7 @@
         <v/>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1.3</v>
+        <v>1.17</v>
       </c>
       <c r="K17" s="20">
         <f>IF(I17&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1943,7 +1943,7 @@
         <v>0.5</v>
       </c>
       <c r="G18" s="18" t="n">
-        <v>0.319</v>
+        <v>0.219</v>
       </c>
       <c r="H18" s="17" t="n">
         <v>0.83</v>
@@ -1953,7 +1953,7 @@
         <v/>
       </c>
       <c r="J18" s="6" t="n">
-        <v>1.3</v>
+        <v>1.17</v>
       </c>
       <c r="K18" s="20">
         <f>IF(I18&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1992,7 +1992,7 @@
         <v>0.5</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>0.414</v>
+        <v>0.282</v>
       </c>
       <c r="H19" s="17" t="n">
         <v>0.83</v>
@@ -2002,7 +2002,7 @@
         <v/>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1.39</v>
+        <v>1.26</v>
       </c>
       <c r="K19" s="20">
         <f>IF(I19&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2041,7 +2041,7 @@
         <v>0.5</v>
       </c>
       <c r="G20" s="18" t="n">
-        <v>0.414</v>
+        <v>0.282</v>
       </c>
       <c r="H20" s="17" t="n">
         <v>0.79</v>
@@ -2051,7 +2051,7 @@
         <v/>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.39</v>
+        <v>1.26</v>
       </c>
       <c r="K20" s="20">
         <f>IF(I20&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2090,7 +2090,7 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>0.469</v>
+        <v>0.317</v>
       </c>
       <c r="H21" s="17" t="n">
         <v>0.79</v>
@@ -2100,7 +2100,7 @@
         <v/>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1.43</v>
+        <v>1.3</v>
       </c>
       <c r="K21" s="20">
         <f>IF(I21&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2139,7 +2139,7 @@
         <v>0.5</v>
       </c>
       <c r="G22" s="18" t="n">
-        <v>0.08</v>
+        <v>0.058</v>
       </c>
       <c r="H22" s="17" t="n">
         <v>0.3</v>
@@ -2149,7 +2149,7 @@
         <v/>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.77</v>
+        <v>0.65</v>
       </c>
       <c r="K22" s="20">
         <f>IF(I22&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2188,7 +2188,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0.101</v>
+        <v>0.073</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>0.3</v>
@@ -2198,7 +2198,7 @@
         <v/>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.86</v>
+        <v>0.73</v>
       </c>
       <c r="K23" s="20">
         <f>IF(I23&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2237,7 +2237,7 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="18" t="n">
-        <v>0.109</v>
+        <v>0.078</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>0.43</v>
@@ -2247,7 +2247,7 @@
         <v/>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.89</v>
+        <v>0.76</v>
       </c>
       <c r="K24" s="20">
         <f>IF(I24&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2286,7 +2286,7 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>0.11</v>
+        <v>0.079</v>
       </c>
       <c r="H25" s="17" t="n">
         <v>0.47</v>
@@ -2296,7 +2296,7 @@
         <v/>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.89</v>
+        <v>0.77</v>
       </c>
       <c r="K25" s="20">
         <f>IF(I25&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2335,7 +2335,7 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="18" t="n">
-        <v>0.138</v>
+        <v>0.098</v>
       </c>
       <c r="H26" s="17" t="n">
         <v>0.48</v>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.98</v>
+        <v>0.85</v>
       </c>
       <c r="K26" s="20">
         <f>IF(I26&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2384,7 +2384,7 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0.162</v>
+        <v>0.115</v>
       </c>
       <c r="H27" s="17" t="n">
         <v>0.49</v>
@@ -2394,7 +2394,7 @@
         <v/>
       </c>
       <c r="J27" s="6" t="n">
-        <v>1.05</v>
+        <v>0.91</v>
       </c>
       <c r="K27" s="20">
         <f>IF(I27&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2433,7 +2433,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="18" t="n">
-        <v>0.172</v>
+        <v>0.122</v>
       </c>
       <c r="H28" s="17" t="n">
         <v>0.57</v>
@@ -2443,7 +2443,7 @@
         <v/>
       </c>
       <c r="J28" s="6" t="n">
-        <v>1.07</v>
+        <v>0.93</v>
       </c>
       <c r="K28" s="20">
         <f>IF(I28&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2482,7 +2482,7 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0.207</v>
+        <v>0.145</v>
       </c>
       <c r="H29" s="17" t="n">
         <v>0.61</v>
@@ -2492,7 +2492,7 @@
         <v/>
       </c>
       <c r="J29" s="6" t="n">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="K29" s="20">
         <f>IF(I29&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2531,7 +2531,7 @@
         <v>0.5</v>
       </c>
       <c r="G30" s="18" t="n">
-        <v>0.081</v>
+        <v>0.059</v>
       </c>
       <c r="H30" s="17" t="n">
         <v>0.3</v>
@@ -2541,7 +2541,7 @@
         <v/>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.78</v>
+        <v>0.66</v>
       </c>
       <c r="K30" s="20">
         <f>IF(I30&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2580,7 +2580,7 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.064</v>
       </c>
       <c r="H31" s="17" t="n">
         <v>0.41</v>
@@ -2590,7 +2590,7 @@
         <v/>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K31" s="20">
         <f>IF(I31&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2629,7 +2629,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="18" t="n">
-        <v>0.106</v>
+        <v>0.077</v>
       </c>
       <c r="H32" s="17" t="n">
         <v>0.44</v>
@@ -2639,7 +2639,7 @@
         <v/>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.88</v>
+        <v>0.75</v>
       </c>
       <c r="K32" s="20">
         <f>IF(I32&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2678,7 +2678,7 @@
         <v>0.5</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0.112</v>
+        <v>0.081</v>
       </c>
       <c r="H33" s="17" t="n">
         <v>0.53</v>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
       <c r="J33" s="6" t="n">
-        <v>0.9</v>
+        <v>0.77</v>
       </c>
       <c r="K33" s="20">
         <f>IF(I33&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2727,7 +2727,7 @@
         <v>0.5</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>0.148</v>
+        <v>0.105</v>
       </c>
       <c r="H34" s="17" t="n">
         <v>0.55</v>
@@ -2737,7 +2737,7 @@
         <v/>
       </c>
       <c r="J34" s="6" t="n">
-        <v>1.01</v>
+        <v>0.87</v>
       </c>
       <c r="K34" s="20">
         <f>IF(I34&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2776,7 +2776,7 @@
         <v>0.5</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0.052</v>
+        <v>0.038</v>
       </c>
       <c r="H35" s="17" t="n">
         <v>0.3</v>
@@ -2786,7 +2786,7 @@
         <v/>
       </c>
       <c r="J35" s="6" t="n">
-        <v>0.62</v>
+        <v>0.52</v>
       </c>
       <c r="K35" s="20">
         <f>IF(I35&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2825,7 +2825,7 @@
         <v>1.72</v>
       </c>
       <c r="G36" s="18" t="n">
-        <v>0.036</v>
+        <v>0.026</v>
       </c>
       <c r="H36" s="17" t="n">
         <v>0.3</v>
@@ -2835,7 +2835,7 @@
         <v/>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0.93</v>
+        <v>0.78</v>
       </c>
       <c r="K36" s="20">
         <f>IF(I36&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2874,7 +2874,7 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0.166</v>
+        <v>0.118</v>
       </c>
       <c r="H37" s="17" t="n">
         <v>0.5</v>
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="J37" s="6" t="n">
-        <v>1.06</v>
+        <v>0.92</v>
       </c>
       <c r="K37" s="20">
         <f>IF(I37&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2923,7 +2923,7 @@
         <v>0.5</v>
       </c>
       <c r="G38" s="18" t="n">
-        <v>0.218</v>
+        <v>0.153</v>
       </c>
       <c r="H38" s="17" t="n">
         <v>0.59</v>
@@ -2933,7 +2933,7 @@
         <v/>
       </c>
       <c r="J38" s="6" t="n">
-        <v>1.16</v>
+        <v>1.02</v>
       </c>
       <c r="K38" s="20">
         <f>IF(I38&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2972,7 +2972,7 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0.218</v>
+        <v>0.153</v>
       </c>
       <c r="H39" s="17" t="n">
         <v>0.61</v>
@@ -2982,7 +2982,7 @@
         <v/>
       </c>
       <c r="J39" s="6" t="n">
-        <v>1.16</v>
+        <v>1.02</v>
       </c>
       <c r="K39" s="20">
         <f>IF(I39&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3021,7 +3021,7 @@
         <v>0.5</v>
       </c>
       <c r="G40" s="18" t="n">
-        <v>0.259</v>
+        <v>0.18</v>
       </c>
       <c r="H40" s="17" t="n">
         <v>0.62</v>
@@ -3031,7 +3031,7 @@
         <v/>
       </c>
       <c r="J40" s="6" t="n">
-        <v>1.23</v>
+        <v>1.09</v>
       </c>
       <c r="K40" s="20">
         <f>IF(I40&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3070,7 +3070,7 @@
         <v>0.5</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0.259</v>
+        <v>0.18</v>
       </c>
       <c r="H41" s="17" t="n">
         <v>0.73</v>
@@ -3080,7 +3080,7 @@
         <v/>
       </c>
       <c r="J41" s="6" t="n">
-        <v>1.23</v>
+        <v>1.09</v>
       </c>
       <c r="K41" s="20">
         <f>IF(I41&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3119,7 +3119,7 @@
         <v>0.5</v>
       </c>
       <c r="G42" s="18" t="n">
-        <v>0.341</v>
+        <v>0.234</v>
       </c>
       <c r="H42" s="17" t="n">
         <v>0.73</v>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
       <c r="J42" s="6" t="n">
-        <v>1.33</v>
+        <v>1.19</v>
       </c>
       <c r="K42" s="20">
         <f>IF(I42&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3168,7 +3168,7 @@
         <v>0.5</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0.395</v>
+        <v>0.269</v>
       </c>
       <c r="H43" s="17" t="n">
         <v>0.79</v>
@@ -3178,7 +3178,7 @@
         <v/>
       </c>
       <c r="J43" s="6" t="n">
-        <v>1.38</v>
+        <v>1.24</v>
       </c>
       <c r="K43" s="20">
         <f>IF(I43&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3217,7 +3217,7 @@
         <v>0.5</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>0.395</v>
+        <v>0.269</v>
       </c>
       <c r="H44" s="17" t="n">
         <v>0.7</v>
@@ -3227,7 +3227,7 @@
         <v/>
       </c>
       <c r="J44" s="6" t="n">
-        <v>1.38</v>
+        <v>1.24</v>
       </c>
       <c r="K44" s="20">
         <f>IF(I44&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3266,7 +3266,7 @@
         <v>0.5</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>0.396</v>
+        <v>0.27</v>
       </c>
       <c r="H45" s="17" t="n">
         <v>0.7</v>
@@ -3276,7 +3276,7 @@
         <v/>
       </c>
       <c r="J45" s="6" t="n">
-        <v>1.38</v>
+        <v>1.24</v>
       </c>
       <c r="K45" s="20">
         <f>IF(I45&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3315,7 +3315,7 @@
         <v>0.5</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>0.397</v>
+        <v>0.27</v>
       </c>
       <c r="H46" s="17" t="n">
         <v>0.74</v>
@@ -3325,7 +3325,7 @@
         <v/>
       </c>
       <c r="J46" s="6" t="n">
-        <v>1.38</v>
+        <v>1.24</v>
       </c>
       <c r="K46" s="20">
         <f>IF(I46&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3364,7 +3364,7 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>0.399</v>
+        <v>0.272</v>
       </c>
       <c r="H47" s="17" t="n">
         <v>0.74</v>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="J47" s="6" t="n">
-        <v>1.38</v>
+        <v>1.25</v>
       </c>
       <c r="K47" s="20">
         <f>IF(I47&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3413,7 +3413,7 @@
         <v>0.5</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>0.399</v>
+        <v>0.272</v>
       </c>
       <c r="H48" s="17" t="n">
         <v>0.77</v>
@@ -3423,7 +3423,7 @@
         <v/>
       </c>
       <c r="J48" s="6" t="n">
-        <v>1.38</v>
+        <v>1.25</v>
       </c>
       <c r="K48" s="20">
         <f>IF(I48&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3462,7 +3462,7 @@
         <v>0.5</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>0.404</v>
+        <v>0.275</v>
       </c>
       <c r="H49" s="17" t="n">
         <v>0.77</v>
@@ -3472,7 +3472,7 @@
         <v/>
       </c>
       <c r="J49" s="6" t="n">
-        <v>1.39</v>
+        <v>1.25</v>
       </c>
       <c r="K49" s="20">
         <f>IF(I49&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3511,7 +3511,7 @@
         <v>0.5</v>
       </c>
       <c r="G50" s="18" t="n">
-        <v>0.406</v>
+        <v>0.276</v>
       </c>
       <c r="H50" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3521,7 +3521,7 @@
         <v/>
       </c>
       <c r="J50" s="6" t="n">
-        <v>1.39</v>
+        <v>1.25</v>
       </c>
       <c r="K50" s="20">
         <f>IF(I50&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3560,7 +3560,7 @@
         <v>0.5</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>0.406</v>
+        <v>0.276</v>
       </c>
       <c r="H51" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3570,7 +3570,7 @@
         <v/>
       </c>
       <c r="J51" s="6" t="n">
-        <v>1.39</v>
+        <v>1.25</v>
       </c>
       <c r="K51" s="20">
         <f>IF(I51&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3609,7 +3609,7 @@
         <v>0.5</v>
       </c>
       <c r="G52" s="18" t="n">
-        <v>0.033</v>
+        <v>0.024</v>
       </c>
       <c r="H52" s="17" t="n">
         <v>0.3</v>
@@ -3619,7 +3619,7 @@
         <v/>
       </c>
       <c r="J52" s="6" t="n">
-        <v>0.48</v>
+        <v>0.4</v>
       </c>
       <c r="K52" s="20">
         <f>IF(I52&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3658,7 +3658,7 @@
         <v>0.5</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>0.105</v>
+        <v>0.075</v>
       </c>
       <c r="H53" s="17" t="n">
         <v>0.32</v>
@@ -3668,7 +3668,7 @@
         <v/>
       </c>
       <c r="J53" s="6" t="n">
-        <v>0.87</v>
+        <v>0.75</v>
       </c>
       <c r="K53" s="20">
         <f>IF(I53&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3707,7 +3707,7 @@
         <v>0.5</v>
       </c>
       <c r="G54" s="18" t="n">
-        <v>0.089</v>
+        <v>0.064</v>
       </c>
       <c r="H54" s="17" t="n">
         <v>0.3</v>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J54" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K54" s="20">
         <f>IF(I54&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3756,7 +3756,7 @@
         <v>0.5</v>
       </c>
       <c r="G55" s="18" t="n">
-        <v>0.075</v>
+        <v>0.055</v>
       </c>
       <c r="H55" s="17" t="n">
         <v>0.3</v>
@@ -3766,7 +3766,7 @@
         <v/>
       </c>
       <c r="J55" s="6" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="K55" s="20">
         <f>IF(I55&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3805,7 +3805,7 @@
         <v>0.5</v>
       </c>
       <c r="G56" s="18" t="n">
-        <v>0.082</v>
+        <v>0.06</v>
       </c>
       <c r="H56" s="17" t="n">
         <v>0.39</v>
@@ -3815,7 +3815,7 @@
         <v/>
       </c>
       <c r="J56" s="6" t="n">
-        <v>0.78</v>
+        <v>0.67</v>
       </c>
       <c r="K56" s="20">
         <f>IF(I56&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3854,7 +3854,7 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="18" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.062</v>
       </c>
       <c r="H57" s="17" t="n">
         <v>0.42</v>
@@ -3864,7 +3864,7 @@
         <v/>
       </c>
       <c r="J57" s="6" t="n">
-        <v>0.8</v>
+        <v>0.68</v>
       </c>
       <c r="K57" s="20">
         <f>IF(I57&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3903,7 +3903,7 @@
         <v>0.5</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>0.111</v>
+        <v>0.08</v>
       </c>
       <c r="H58" s="17" t="n">
         <v>0.42</v>
@@ -3913,7 +3913,7 @@
         <v/>
       </c>
       <c r="J58" s="6" t="n">
-        <v>0.9</v>
+        <v>0.77</v>
       </c>
       <c r="K58" s="20">
         <f>IF(I58&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3952,7 +3952,7 @@
         <v>0.5</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>0.111</v>
+        <v>0.08</v>
       </c>
       <c r="H59" s="17" t="n">
         <v>0.48</v>
@@ -3962,7 +3962,7 @@
         <v/>
       </c>
       <c r="J59" s="6" t="n">
-        <v>0.9</v>
+        <v>0.77</v>
       </c>
       <c r="K59" s="20">
         <f>IF(I59&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4001,7 +4001,7 @@
         <v>0.5</v>
       </c>
       <c r="G60" s="18" t="n">
-        <v>0.099</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H60" s="17" t="n">
         <v>0.2</v>
@@ -4011,7 +4011,7 @@
         <v/>
       </c>
       <c r="J60" s="6" t="n">
-        <v>0.85</v>
+        <v>0.73</v>
       </c>
       <c r="K60" s="20">
         <f>IF(I60&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4050,7 +4050,7 @@
         <v>0.5</v>
       </c>
       <c r="G61" s="18" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.051</v>
       </c>
       <c r="H61" s="17" t="n">
         <v>0.3</v>
@@ -4060,7 +4060,7 @@
         <v/>
       </c>
       <c r="J61" s="6" t="n">
-        <v>0.72</v>
+        <v>0.61</v>
       </c>
       <c r="K61" s="20">
         <f>IF(I61&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4099,7 +4099,7 @@
         <v>0.5</v>
       </c>
       <c r="G62" s="18" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.053</v>
       </c>
       <c r="H62" s="17" t="n">
         <v>0.38</v>
@@ -4109,7 +4109,7 @@
         <v/>
       </c>
       <c r="J62" s="6" t="n">
-        <v>0.73</v>
+        <v>0.62</v>
       </c>
       <c r="K62" s="20">
         <f>IF(I62&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4148,7 +4148,7 @@
         <v>0.5</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>0.113</v>
+        <v>0.081</v>
       </c>
       <c r="H63" s="17" t="n">
         <v>0.38</v>
@@ -4158,7 +4158,7 @@
         <v/>
       </c>
       <c r="J63" s="6" t="n">
-        <v>0.9</v>
+        <v>0.78</v>
       </c>
       <c r="K63" s="20">
         <f>IF(I63&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4197,7 +4197,7 @@
         <v>0.5</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>0.113</v>
+        <v>0.081</v>
       </c>
       <c r="H64" s="17" t="n">
         <v>0.49</v>
@@ -4207,7 +4207,7 @@
         <v/>
       </c>
       <c r="J64" s="6" t="n">
-        <v>0.9</v>
+        <v>0.78</v>
       </c>
       <c r="K64" s="20">
         <f>IF(I64&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4246,7 +4246,7 @@
         <v>0.5</v>
       </c>
       <c r="G65" s="18" t="n">
-        <v>0.153</v>
+        <v>0.108</v>
       </c>
       <c r="H65" s="17" t="n">
         <v>0.5</v>
@@ -4256,7 +4256,7 @@
         <v/>
       </c>
       <c r="J65" s="6" t="n">
-        <v>1.02</v>
+        <v>0.89</v>
       </c>
       <c r="K65" s="20">
         <f>IF(I65&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4295,7 +4295,7 @@
         <v>0.5</v>
       </c>
       <c r="G66" s="18" t="n">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
       <c r="H66" s="17" t="n">
         <v>0.52</v>
@@ -4305,7 +4305,7 @@
         <v/>
       </c>
       <c r="J66" s="6" t="n">
-        <v>1.13</v>
+        <v>0.99</v>
       </c>
       <c r="K66" s="20">
         <f>IF(I66&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4344,7 +4344,7 @@
         <v>0.5</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>0.352</v>
+        <v>0.241</v>
       </c>
       <c r="H67" s="17" t="n">
         <v>0.5600000000000001</v>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="J67" s="6" t="n">
-        <v>1.34</v>
+        <v>1.2</v>
       </c>
       <c r="K67" s="20">
         <f>IF(I67&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4393,7 +4393,7 @@
         <v>0.5</v>
       </c>
       <c r="G68" s="18" t="n">
-        <v>0.457</v>
+        <v>0.309</v>
       </c>
       <c r="H68" s="17" t="n">
         <v>0.62</v>
@@ -4403,7 +4403,7 @@
         <v/>
       </c>
       <c r="J68" s="6" t="n">
-        <v>1.42</v>
+        <v>1.29</v>
       </c>
       <c r="K68" s="20">
         <f>IF(I68&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4442,7 +4442,7 @@
         <v>0.5</v>
       </c>
       <c r="G69" s="18" t="n">
-        <v>0.483</v>
+        <v>0.326</v>
       </c>
       <c r="H69" s="17" t="n">
         <v>0.57</v>
@@ -4452,7 +4452,7 @@
         <v/>
       </c>
       <c r="J69" s="6" t="n">
-        <v>1.44</v>
+        <v>1.31</v>
       </c>
       <c r="K69" s="20">
         <f>IF(I69&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4491,7 +4491,7 @@
         <v>0.5</v>
       </c>
       <c r="G70" s="18" t="n">
-        <v>0.486</v>
+        <v>0.328</v>
       </c>
       <c r="H70" s="17" t="n">
         <v>0.63</v>
@@ -4501,7 +4501,7 @@
         <v/>
       </c>
       <c r="J70" s="6" t="n">
-        <v>1.44</v>
+        <v>1.31</v>
       </c>
       <c r="K70" s="20">
         <f>IF(I70&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4540,7 +4540,7 @@
         <v>0.5</v>
       </c>
       <c r="G71" s="18" t="n">
-        <v>0.486</v>
+        <v>0.328</v>
       </c>
       <c r="H71" s="17" t="n">
         <v>0.64</v>
@@ -4550,7 +4550,7 @@
         <v/>
       </c>
       <c r="J71" s="6" t="n">
-        <v>1.44</v>
+        <v>1.31</v>
       </c>
       <c r="K71" s="20">
         <f>IF(I71&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4589,7 +4589,7 @@
         <v>0.5</v>
       </c>
       <c r="G72" s="18" t="n">
-        <v>0.576</v>
+        <v>0.385</v>
       </c>
       <c r="H72" s="17" t="n">
         <v>0.64</v>
@@ -4599,7 +4599,7 @@
         <v/>
       </c>
       <c r="J72" s="6" t="n">
-        <v>1.49</v>
+        <v>1.37</v>
       </c>
       <c r="K72" s="20">
         <f>IF(I72&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4638,7 +4638,7 @@
         <v>0.5</v>
       </c>
       <c r="G73" s="18" t="n">
-        <v>0.078</v>
+        <v>0.057</v>
       </c>
       <c r="H73" s="17" t="n">
         <v>0.3</v>
@@ -4648,7 +4648,7 @@
         <v/>
       </c>
       <c r="J73" s="6" t="n">
-        <v>0.76</v>
+        <v>0.65</v>
       </c>
       <c r="K73" s="20">
         <f>IF(I73&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4687,7 +4687,7 @@
         <v>0.5</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>0.089</v>
+        <v>0.064</v>
       </c>
       <c r="H74" s="17" t="n">
         <v>0.3</v>
@@ -4697,7 +4697,7 @@
         <v/>
       </c>
       <c r="J74" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K74" s="20">
         <f>IF(I74&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4736,7 +4736,7 @@
         <v>0.5</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>0.092</v>
+        <v>0.066</v>
       </c>
       <c r="H75" s="17" t="n">
         <v>0.38</v>
@@ -4746,7 +4746,7 @@
         <v/>
       </c>
       <c r="J75" s="6" t="n">
-        <v>0.82</v>
+        <v>0.7</v>
       </c>
       <c r="K75" s="20">
         <f>IF(I75&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4785,7 +4785,7 @@
         <v>0.5</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>0.147</v>
+        <v>0.105</v>
       </c>
       <c r="H76" s="17" t="n">
         <v>0.35</v>
@@ -4795,7 +4795,7 @@
         <v/>
       </c>
       <c r="J76" s="6" t="n">
-        <v>1.01</v>
+        <v>0.87</v>
       </c>
       <c r="K76" s="20">
         <f>IF(I76&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4834,7 +4834,7 @@
         <v>0.5</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>0.148</v>
+        <v>0.105</v>
       </c>
       <c r="H77" s="17" t="n">
         <v>0.35</v>
@@ -4844,7 +4844,7 @@
         <v/>
       </c>
       <c r="J77" s="6" t="n">
-        <v>1.01</v>
+        <v>0.87</v>
       </c>
       <c r="K77" s="20">
         <f>IF(I77&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4883,7 +4883,7 @@
         <v>0.5</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>0.15</v>
+        <v>0.107</v>
       </c>
       <c r="H78" s="17" t="n">
         <v>0.35</v>
@@ -4893,7 +4893,7 @@
         <v/>
       </c>
       <c r="J78" s="6" t="n">
-        <v>1.02</v>
+        <v>0.88</v>
       </c>
       <c r="K78" s="20">
         <f>IF(I78&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4932,7 +4932,7 @@
         <v>0.5</v>
       </c>
       <c r="G79" s="18" t="n">
-        <v>0.196</v>
+        <v>0.138</v>
       </c>
       <c r="H79" s="17" t="n">
         <v>0.35</v>
@@ -4942,7 +4942,7 @@
         <v/>
       </c>
       <c r="J79" s="6" t="n">
-        <v>1.12</v>
+        <v>0.98</v>
       </c>
       <c r="K79" s="20">
         <f>IF(I79&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4981,7 +4981,7 @@
         <v>0.5</v>
       </c>
       <c r="G80" s="18" t="n">
-        <v>0.2</v>
+        <v>0.141</v>
       </c>
       <c r="H80" s="17" t="n">
         <v>0.45</v>
@@ -4991,7 +4991,7 @@
         <v/>
       </c>
       <c r="J80" s="6" t="n">
-        <v>1.13</v>
+        <v>0.99</v>
       </c>
       <c r="K80" s="20">
         <f>IF(I80&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5030,7 +5030,7 @@
         <v>0.5</v>
       </c>
       <c r="G81" s="18" t="n">
-        <v>0.075</v>
+        <v>0.054</v>
       </c>
       <c r="H81" s="17" t="n">
         <v>0.3</v>
@@ -5040,7 +5040,7 @@
         <v/>
       </c>
       <c r="J81" s="6" t="n">
-        <v>0.74</v>
+        <v>0.63</v>
       </c>
       <c r="K81" s="20">
         <f>IF(I81&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5079,7 +5079,7 @@
         <v>0.5</v>
       </c>
       <c r="G82" s="18" t="n">
-        <v>0.075</v>
+        <v>0.055</v>
       </c>
       <c r="H82" s="17" t="n">
         <v>0.36</v>
@@ -5089,7 +5089,7 @@
         <v/>
       </c>
       <c r="J82" s="6" t="n">
-        <v>0.75</v>
+        <v>0.63</v>
       </c>
       <c r="K82" s="20">
         <f>IF(I82&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5128,7 +5128,7 @@
         <v>0.58</v>
       </c>
       <c r="G83" s="18" t="n">
-        <v>0.144</v>
+        <v>0.102</v>
       </c>
       <c r="H83" s="17" t="n">
         <v>0.35</v>
@@ -5138,7 +5138,7 @@
         <v/>
       </c>
       <c r="J83" s="6" t="n">
-        <v>1.08</v>
+        <v>0.93</v>
       </c>
       <c r="K83" s="20">
         <f>IF(I83&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5177,7 +5177,7 @@
         <v>0.5</v>
       </c>
       <c r="G84" s="18" t="n">
-        <v>0.158</v>
+        <v>0.112</v>
       </c>
       <c r="H84" s="17" t="n">
         <v>0.35</v>
@@ -5187,7 +5187,7 @@
         <v/>
       </c>
       <c r="J84" s="6" t="n">
-        <v>1.04</v>
+        <v>0.9</v>
       </c>
       <c r="K84" s="20">
         <f>IF(I84&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5226,7 +5226,7 @@
         <v>0.5</v>
       </c>
       <c r="G85" s="18" t="n">
-        <v>0.113</v>
+        <v>0.081</v>
       </c>
       <c r="H85" s="17" t="n">
         <v>0.3</v>
@@ -5236,7 +5236,7 @@
         <v/>
       </c>
       <c r="J85" s="6" t="n">
-        <v>0.9</v>
+        <v>0.78</v>
       </c>
       <c r="K85" s="20">
         <f>IF(I85&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5275,7 +5275,7 @@
         <v>0.5</v>
       </c>
       <c r="G86" s="18" t="n">
-        <v>0.119</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="H86" s="17" t="n">
         <v>0.45</v>
@@ -5285,7 +5285,7 @@
         <v/>
       </c>
       <c r="J86" s="6" t="n">
-        <v>0.92</v>
+        <v>0.79</v>
       </c>
       <c r="K86" s="20">
         <f>IF(I86&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5324,7 +5324,7 @@
         <v>0.5</v>
       </c>
       <c r="G87" s="18" t="n">
-        <v>0.121</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H87" s="17" t="n">
         <v>0.46</v>
@@ -5334,7 +5334,7 @@
         <v/>
       </c>
       <c r="J87" s="6" t="n">
-        <v>0.93</v>
+        <v>0.8</v>
       </c>
       <c r="K87" s="20">
         <f>IF(I87&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5373,7 +5373,7 @@
         <v>0.5</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>0.121</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H88" s="17" t="n">
         <v>0.47</v>
@@ -5383,7 +5383,7 @@
         <v/>
       </c>
       <c r="J88" s="6" t="n">
-        <v>0.93</v>
+        <v>0.8</v>
       </c>
       <c r="K88" s="20">
         <f>IF(I88&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5422,7 +5422,7 @@
         <v>0.5</v>
       </c>
       <c r="G89" s="18" t="n">
-        <v>0.15</v>
+        <v>0.107</v>
       </c>
       <c r="H89" s="17" t="n">
         <v>0.4</v>
@@ -5432,7 +5432,7 @@
         <v/>
       </c>
       <c r="J89" s="6" t="n">
-        <v>1.02</v>
+        <v>0.88</v>
       </c>
       <c r="K89" s="20">
         <f>IF(I89&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5471,7 +5471,7 @@
         <v>0.5</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>0.15</v>
+        <v>0.107</v>
       </c>
       <c r="H90" s="17" t="n">
         <v>0.4</v>
@@ -5481,7 +5481,7 @@
         <v/>
       </c>
       <c r="J90" s="6" t="n">
-        <v>1.02</v>
+        <v>0.88</v>
       </c>
       <c r="K90" s="20">
         <f>IF(I90&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5520,7 +5520,7 @@
         <v>0.51</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>0.097</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H91" s="17" t="n">
         <v>0.2</v>
@@ -5530,7 +5530,7 @@
         <v/>
       </c>
       <c r="J91" s="6" t="n">
-        <v>0.86</v>
+        <v>0.73</v>
       </c>
       <c r="K91" s="20">
         <f>IF(I91&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5569,7 +5569,7 @@
         <v>0.5</v>
       </c>
       <c r="G92" s="18" t="n">
-        <v>0.098</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H92" s="17" t="n">
         <v>0.5</v>
@@ -5579,7 +5579,7 @@
         <v/>
       </c>
       <c r="J92" s="6" t="n">
-        <v>0.85</v>
+        <v>0.72</v>
       </c>
       <c r="K92" s="20">
         <f>IF(I92&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5618,7 +5618,7 @@
         <v>0.5</v>
       </c>
       <c r="G93" s="18" t="n">
-        <v>0.151</v>
+        <v>0.107</v>
       </c>
       <c r="H93" s="17" t="n">
         <v>0.5</v>
@@ -5628,7 +5628,7 @@
         <v/>
       </c>
       <c r="J93" s="6" t="n">
-        <v>1.02</v>
+        <v>0.88</v>
       </c>
       <c r="K93" s="20">
         <f>IF(I93&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5667,7 +5667,7 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="18" t="n">
-        <v>0.151</v>
+        <v>0.108</v>
       </c>
       <c r="H94" s="17" t="n">
         <v>0.4</v>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="J94" s="6" t="n">
-        <v>1.02</v>
+        <v>0.88</v>
       </c>
       <c r="K94" s="20">
         <f>IF(I94&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5716,7 +5716,7 @@
         <v>0.5</v>
       </c>
       <c r="G95" s="18" t="n">
-        <v>0.044</v>
+        <v>0.032</v>
       </c>
       <c r="H95" s="17" t="n">
         <v>0.3</v>
@@ -5726,7 +5726,7 @@
         <v/>
       </c>
       <c r="J95" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.47</v>
       </c>
       <c r="K95" s="20">
         <f>IF(I95&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5765,7 +5765,7 @@
         <v>0.5</v>
       </c>
       <c r="G96" s="18" t="n">
-        <v>0.044</v>
+        <v>0.032</v>
       </c>
       <c r="H96" s="17" t="n">
         <v>0.36</v>
@@ -5775,7 +5775,7 @@
         <v/>
       </c>
       <c r="J96" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.47</v>
       </c>
       <c r="K96" s="20">
         <f>IF(I96&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5814,7 +5814,7 @@
         <v>0.5</v>
       </c>
       <c r="G97" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.051</v>
       </c>
       <c r="H97" s="17" t="n">
         <v>0.36</v>
@@ -5824,7 +5824,7 @@
         <v/>
       </c>
       <c r="J97" s="6" t="n">
-        <v>0.72</v>
+        <v>0.61</v>
       </c>
       <c r="K97" s="20">
         <f>IF(I97&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5863,7 +5863,7 @@
         <v>0.5</v>
       </c>
       <c r="G98" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.051</v>
       </c>
       <c r="H98" s="17" t="n">
         <v>0.48</v>
@@ -5873,7 +5873,7 @@
         <v/>
       </c>
       <c r="J98" s="6" t="n">
-        <v>0.72</v>
+        <v>0.61</v>
       </c>
       <c r="K98" s="20">
         <f>IF(I98&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5912,7 +5912,7 @@
         <v>0.5</v>
       </c>
       <c r="G99" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.063</v>
       </c>
       <c r="H99" s="17" t="n">
         <v>0.49</v>
@@ -5922,7 +5922,7 @@
         <v/>
       </c>
       <c r="J99" s="6" t="n">
-        <v>0.8</v>
+        <v>0.68</v>
       </c>
       <c r="K99" s="20">
         <f>IF(I99&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5961,7 +5961,7 @@
         <v>0.5</v>
       </c>
       <c r="G100" s="18" t="n">
-        <v>0.036</v>
+        <v>0.026</v>
       </c>
       <c r="H100" s="17" t="n">
         <v>0.3</v>
@@ -5971,7 +5971,7 @@
         <v/>
       </c>
       <c r="J100" s="6" t="n">
-        <v>0.5</v>
+        <v>0.42</v>
       </c>
       <c r="K100" s="20">
         <f>IF(I100&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -6010,7 +6010,7 @@
         <v>0.5</v>
       </c>
       <c r="G101" s="18" t="n">
-        <v>0.036</v>
+        <v>0.026</v>
       </c>
       <c r="H101" s="17" t="n">
         <v>0.37</v>
@@ -6020,7 +6020,7 @@
         <v/>
       </c>
       <c r="J101" s="6" t="n">
-        <v>0.5</v>
+        <v>0.42</v>
       </c>
       <c r="K101" s="20">
         <f>IF(I101&gt;=0.05,"CUMPLE","NO CUMPLE")</f>

</xml_diff>

<commit_message>
Barranquita: superficies por tipo, metrado y especificaciones en formato CAR, anexo estadistico
Superficies dentro del cerco: techos (incluye aulas en diagonal, patio civico y losa multiusos
techados), areas libres de concreto, patio de maniobra y estacionamiento, areas verdes; C 0.761.
Metrado con las hojas del CAR Mujeres y los mismos totales; especificaciones con el motor de los
CAR; memoria hidrologica con el anexo de cuadros estadisticos. Planos sin cambios.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>I = 289 mm/h, C ponderado = 0.57, area total 9393 m2; menor borde libre 0.129 m en EJE-11 P-48-P-33 (Q 18.8 l/s, y 0.071, h 0.20)</t>
+          <t>I = 289 mm/h, C ponderado = 0.76, area total 9393 m2; menor borde libre 0.129 m en EJE-11 P-48-P-33 (Q 18.8 l/s, y 0.071, h 0.20)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>V max 1.62 m/s</t>
+          <t>V max 1.97 m/s</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>0.57</v>
+        <v>0.761</v>
       </c>
     </row>
     <row r="5">
@@ -1600,7 +1600,7 @@
         <v>0.5</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>0.073</v>
+        <v>0.094</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>0.3</v>
@@ -1610,7 +1610,7 @@
         <v/>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0.74</v>
+        <v>0.83</v>
       </c>
       <c r="K11" s="20">
         <f>IF(I11&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1649,7 +1649,7 @@
         <v>0.5</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>0.076</v>
+        <v>0.096</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>0.46</v>
@@ -1659,7 +1659,7 @@
         <v/>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.75</v>
+        <v>0.84</v>
       </c>
       <c r="K12" s="20">
         <f>IF(I12&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1698,7 +1698,7 @@
         <v>0.5</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0.062</v>
+        <v>0.083</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>0.3</v>
@@ -1708,7 +1708,7 @@
         <v/>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.68</v>
+        <v>0.78</v>
       </c>
       <c r="K13" s="20">
         <f>IF(I13&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1747,7 +1747,7 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>0.065</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>0.46</v>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="K14" s="20">
         <f>IF(I14&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1796,7 +1796,7 @@
         <v>0.5</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.073</v>
+        <v>0.103</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>0.46</v>
@@ -1806,7 +1806,7 @@
         <v/>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.74</v>
+        <v>0.87</v>
       </c>
       <c r="K15" s="20">
         <f>IF(I15&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1845,7 +1845,7 @@
         <v>2.92</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>0.061</v>
+        <v>0.09</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>0.52</v>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="J16" s="6" t="n">
-        <v>1.62</v>
+        <v>1.97</v>
       </c>
       <c r="K16" s="20">
         <f>IF(I16&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1894,7 +1894,7 @@
         <v>0.5</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>0.219</v>
+        <v>0.314</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>0.77</v>
@@ -1904,7 +1904,7 @@
         <v/>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1.17</v>
+        <v>1.3</v>
       </c>
       <c r="K17" s="20">
         <f>IF(I17&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1943,7 +1943,7 @@
         <v>0.5</v>
       </c>
       <c r="G18" s="18" t="n">
-        <v>0.219</v>
+        <v>0.314</v>
       </c>
       <c r="H18" s="17" t="n">
         <v>0.83</v>
@@ -1953,7 +1953,7 @@
         <v/>
       </c>
       <c r="J18" s="6" t="n">
-        <v>1.17</v>
+        <v>1.3</v>
       </c>
       <c r="K18" s="20">
         <f>IF(I18&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1992,7 +1992,7 @@
         <v>0.5</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>0.282</v>
+        <v>0.399</v>
       </c>
       <c r="H19" s="17" t="n">
         <v>0.83</v>
@@ -2002,7 +2002,7 @@
         <v/>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1.26</v>
+        <v>1.38</v>
       </c>
       <c r="K19" s="20">
         <f>IF(I19&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2041,7 +2041,7 @@
         <v>0.5</v>
       </c>
       <c r="G20" s="18" t="n">
-        <v>0.282</v>
+        <v>0.399</v>
       </c>
       <c r="H20" s="17" t="n">
         <v>0.79</v>
@@ -2051,7 +2051,7 @@
         <v/>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.26</v>
+        <v>1.38</v>
       </c>
       <c r="K20" s="20">
         <f>IF(I20&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2090,7 +2090,7 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>0.317</v>
+        <v>0.448</v>
       </c>
       <c r="H21" s="17" t="n">
         <v>0.79</v>
@@ -2100,7 +2100,7 @@
         <v/>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1.3</v>
+        <v>1.42</v>
       </c>
       <c r="K21" s="20">
         <f>IF(I21&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2139,7 +2139,7 @@
         <v>0.5</v>
       </c>
       <c r="G22" s="18" t="n">
-        <v>0.058</v>
+        <v>0.091</v>
       </c>
       <c r="H22" s="17" t="n">
         <v>0.3</v>
@@ -2149,7 +2149,7 @@
         <v/>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.65</v>
+        <v>0.82</v>
       </c>
       <c r="K22" s="20">
         <f>IF(I22&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2188,7 +2188,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0.073</v>
+        <v>0.077</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>0.3</v>
@@ -2198,7 +2198,7 @@
         <v/>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="K23" s="20">
         <f>IF(I23&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2237,7 +2237,7 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="18" t="n">
-        <v>0.078</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>0.43</v>
@@ -2247,7 +2247,7 @@
         <v/>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.76</v>
+        <v>0.79</v>
       </c>
       <c r="K24" s="20">
         <f>IF(I24&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2286,7 +2286,7 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>0.079</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H25" s="17" t="n">
         <v>0.47</v>
@@ -2296,7 +2296,7 @@
         <v/>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="K25" s="20">
         <f>IF(I25&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2335,7 +2335,7 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="18" t="n">
-        <v>0.098</v>
+        <v>0.104</v>
       </c>
       <c r="H26" s="17" t="n">
         <v>0.48</v>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="K26" s="20">
         <f>IF(I26&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2384,7 +2384,7 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0.115</v>
+        <v>0.129</v>
       </c>
       <c r="H27" s="17" t="n">
         <v>0.49</v>
@@ -2394,7 +2394,7 @@
         <v/>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0.91</v>
+        <v>0.96</v>
       </c>
       <c r="K27" s="20">
         <f>IF(I27&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2433,7 +2433,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="18" t="n">
-        <v>0.122</v>
+        <v>0.139</v>
       </c>
       <c r="H28" s="17" t="n">
         <v>0.57</v>
@@ -2443,7 +2443,7 @@
         <v/>
       </c>
       <c r="J28" s="6" t="n">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="K28" s="20">
         <f>IF(I28&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2482,7 +2482,7 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0.145</v>
+        <v>0.186</v>
       </c>
       <c r="H29" s="17" t="n">
         <v>0.61</v>
@@ -2492,7 +2492,7 @@
         <v/>
       </c>
       <c r="J29" s="6" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="K29" s="20">
         <f>IF(I29&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2629,7 +2629,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="18" t="n">
-        <v>0.077</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H32" s="17" t="n">
         <v>0.44</v>
@@ -2639,7 +2639,7 @@
         <v/>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.75</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K32" s="20">
         <f>IF(I32&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2678,7 +2678,7 @@
         <v>0.5</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0.081</v>
+        <v>0.093</v>
       </c>
       <c r="H33" s="17" t="n">
         <v>0.53</v>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
       <c r="J33" s="6" t="n">
-        <v>0.77</v>
+        <v>0.83</v>
       </c>
       <c r="K33" s="20">
         <f>IF(I33&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2727,7 +2727,7 @@
         <v>0.5</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>0.105</v>
+        <v>0.135</v>
       </c>
       <c r="H34" s="17" t="n">
         <v>0.55</v>
@@ -2737,7 +2737,7 @@
         <v/>
       </c>
       <c r="J34" s="6" t="n">
-        <v>0.87</v>
+        <v>0.97</v>
       </c>
       <c r="K34" s="20">
         <f>IF(I34&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2825,7 +2825,7 @@
         <v>1.72</v>
       </c>
       <c r="G36" s="18" t="n">
-        <v>0.026</v>
+        <v>0.029</v>
       </c>
       <c r="H36" s="17" t="n">
         <v>0.3</v>
@@ -2835,7 +2835,7 @@
         <v/>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0.78</v>
+        <v>0.83</v>
       </c>
       <c r="K36" s="20">
         <f>IF(I36&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2874,7 +2874,7 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0.118</v>
+        <v>0.165</v>
       </c>
       <c r="H37" s="17" t="n">
         <v>0.5</v>
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="J37" s="6" t="n">
-        <v>0.92</v>
+        <v>1.05</v>
       </c>
       <c r="K37" s="20">
         <f>IF(I37&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2923,7 +2923,7 @@
         <v>0.5</v>
       </c>
       <c r="G38" s="18" t="n">
-        <v>0.153</v>
+        <v>0.219</v>
       </c>
       <c r="H38" s="17" t="n">
         <v>0.59</v>
@@ -2933,7 +2933,7 @@
         <v/>
       </c>
       <c r="J38" s="6" t="n">
-        <v>1.02</v>
+        <v>1.16</v>
       </c>
       <c r="K38" s="20">
         <f>IF(I38&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2972,7 +2972,7 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0.153</v>
+        <v>0.219</v>
       </c>
       <c r="H39" s="17" t="n">
         <v>0.61</v>
@@ -2982,7 +2982,7 @@
         <v/>
       </c>
       <c r="J39" s="6" t="n">
-        <v>1.02</v>
+        <v>1.17</v>
       </c>
       <c r="K39" s="20">
         <f>IF(I39&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3021,7 +3021,7 @@
         <v>0.5</v>
       </c>
       <c r="G40" s="18" t="n">
-        <v>0.18</v>
+        <v>0.246</v>
       </c>
       <c r="H40" s="17" t="n">
         <v>0.62</v>
@@ -3031,7 +3031,7 @@
         <v/>
       </c>
       <c r="J40" s="6" t="n">
-        <v>1.09</v>
+        <v>1.21</v>
       </c>
       <c r="K40" s="20">
         <f>IF(I40&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3070,7 +3070,7 @@
         <v>0.5</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0.18</v>
+        <v>0.246</v>
       </c>
       <c r="H41" s="17" t="n">
         <v>0.73</v>
@@ -3080,7 +3080,7 @@
         <v/>
       </c>
       <c r="J41" s="6" t="n">
-        <v>1.09</v>
+        <v>1.21</v>
       </c>
       <c r="K41" s="20">
         <f>IF(I41&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3119,7 +3119,7 @@
         <v>0.5</v>
       </c>
       <c r="G42" s="18" t="n">
-        <v>0.234</v>
+        <v>0.304</v>
       </c>
       <c r="H42" s="17" t="n">
         <v>0.73</v>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
       <c r="J42" s="6" t="n">
-        <v>1.19</v>
+        <v>1.29</v>
       </c>
       <c r="K42" s="20">
         <f>IF(I42&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3168,7 +3168,7 @@
         <v>0.5</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0.269</v>
+        <v>0.338</v>
       </c>
       <c r="H43" s="17" t="n">
         <v>0.79</v>
@@ -3178,7 +3178,7 @@
         <v/>
       </c>
       <c r="J43" s="6" t="n">
-        <v>1.24</v>
+        <v>1.32</v>
       </c>
       <c r="K43" s="20">
         <f>IF(I43&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3217,7 +3217,7 @@
         <v>0.5</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>0.269</v>
+        <v>0.338</v>
       </c>
       <c r="H44" s="17" t="n">
         <v>0.7</v>
@@ -3227,7 +3227,7 @@
         <v/>
       </c>
       <c r="J44" s="6" t="n">
-        <v>1.24</v>
+        <v>1.32</v>
       </c>
       <c r="K44" s="20">
         <f>IF(I44&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3266,7 +3266,7 @@
         <v>0.5</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>0.27</v>
+        <v>0.338</v>
       </c>
       <c r="H45" s="17" t="n">
         <v>0.7</v>
@@ -3276,7 +3276,7 @@
         <v/>
       </c>
       <c r="J45" s="6" t="n">
-        <v>1.24</v>
+        <v>1.33</v>
       </c>
       <c r="K45" s="20">
         <f>IF(I45&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3315,7 +3315,7 @@
         <v>0.5</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>0.27</v>
+        <v>0.339</v>
       </c>
       <c r="H46" s="17" t="n">
         <v>0.74</v>
@@ -3325,7 +3325,7 @@
         <v/>
       </c>
       <c r="J46" s="6" t="n">
-        <v>1.24</v>
+        <v>1.33</v>
       </c>
       <c r="K46" s="20">
         <f>IF(I46&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3364,7 +3364,7 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>0.272</v>
+        <v>0.34</v>
       </c>
       <c r="H47" s="17" t="n">
         <v>0.74</v>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="J47" s="6" t="n">
-        <v>1.25</v>
+        <v>1.33</v>
       </c>
       <c r="K47" s="20">
         <f>IF(I47&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3413,7 +3413,7 @@
         <v>0.5</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>0.272</v>
+        <v>0.34</v>
       </c>
       <c r="H48" s="17" t="n">
         <v>0.77</v>
@@ -3423,7 +3423,7 @@
         <v/>
       </c>
       <c r="J48" s="6" t="n">
-        <v>1.25</v>
+        <v>1.33</v>
       </c>
       <c r="K48" s="20">
         <f>IF(I48&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3462,7 +3462,7 @@
         <v>0.5</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>0.275</v>
+        <v>0.343</v>
       </c>
       <c r="H49" s="17" t="n">
         <v>0.77</v>
@@ -3472,7 +3472,7 @@
         <v/>
       </c>
       <c r="J49" s="6" t="n">
-        <v>1.25</v>
+        <v>1.33</v>
       </c>
       <c r="K49" s="20">
         <f>IF(I49&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3511,7 +3511,7 @@
         <v>0.5</v>
       </c>
       <c r="G50" s="18" t="n">
-        <v>0.276</v>
+        <v>0.344</v>
       </c>
       <c r="H50" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3521,7 +3521,7 @@
         <v/>
       </c>
       <c r="J50" s="6" t="n">
-        <v>1.25</v>
+        <v>1.33</v>
       </c>
       <c r="K50" s="20">
         <f>IF(I50&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3560,7 +3560,7 @@
         <v>0.5</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>0.276</v>
+        <v>0.344</v>
       </c>
       <c r="H51" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3570,7 +3570,7 @@
         <v/>
       </c>
       <c r="J51" s="6" t="n">
-        <v>1.25</v>
+        <v>1.33</v>
       </c>
       <c r="K51" s="20">
         <f>IF(I51&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3609,7 +3609,7 @@
         <v>0.5</v>
       </c>
       <c r="G52" s="18" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="H52" s="17" t="n">
         <v>0.3</v>
@@ -3619,7 +3619,7 @@
         <v/>
       </c>
       <c r="J52" s="6" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
       <c r="K52" s="20">
         <f>IF(I52&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3658,7 +3658,7 @@
         <v>0.5</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>0.075</v>
+        <v>0.119</v>
       </c>
       <c r="H53" s="17" t="n">
         <v>0.32</v>
@@ -3668,7 +3668,7 @@
         <v/>
       </c>
       <c r="J53" s="6" t="n">
-        <v>0.75</v>
+        <v>0.92</v>
       </c>
       <c r="K53" s="20">
         <f>IF(I53&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3707,7 +3707,7 @@
         <v>0.5</v>
       </c>
       <c r="G54" s="18" t="n">
-        <v>0.064</v>
+        <v>0.093</v>
       </c>
       <c r="H54" s="17" t="n">
         <v>0.3</v>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J54" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.83</v>
       </c>
       <c r="K54" s="20">
         <f>IF(I54&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3756,7 +3756,7 @@
         <v>0.5</v>
       </c>
       <c r="G55" s="18" t="n">
-        <v>0.055</v>
+        <v>0.063</v>
       </c>
       <c r="H55" s="17" t="n">
         <v>0.3</v>
@@ -3766,7 +3766,7 @@
         <v/>
       </c>
       <c r="J55" s="6" t="n">
-        <v>0.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K55" s="20">
         <f>IF(I55&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3805,7 +3805,7 @@
         <v>0.5</v>
       </c>
       <c r="G56" s="18" t="n">
-        <v>0.06</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H56" s="17" t="n">
         <v>0.39</v>
@@ -3815,7 +3815,7 @@
         <v/>
       </c>
       <c r="J56" s="6" t="n">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="K56" s="20">
         <f>IF(I56&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3854,7 +3854,7 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="18" t="n">
-        <v>0.062</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H57" s="17" t="n">
         <v>0.42</v>
@@ -3864,7 +3864,7 @@
         <v/>
       </c>
       <c r="J57" s="6" t="n">
-        <v>0.68</v>
+        <v>0.73</v>
       </c>
       <c r="K57" s="20">
         <f>IF(I57&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3903,7 +3903,7 @@
         <v>0.5</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>0.08</v>
+        <v>0.089</v>
       </c>
       <c r="H58" s="17" t="n">
         <v>0.42</v>
@@ -3913,7 +3913,7 @@
         <v/>
       </c>
       <c r="J58" s="6" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K58" s="20">
         <f>IF(I58&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3952,7 +3952,7 @@
         <v>0.5</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>0.08</v>
+        <v>0.089</v>
       </c>
       <c r="H59" s="17" t="n">
         <v>0.48</v>
@@ -3962,7 +3962,7 @@
         <v/>
       </c>
       <c r="J59" s="6" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K59" s="20">
         <f>IF(I59&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4050,7 +4050,7 @@
         <v>0.5</v>
       </c>
       <c r="G61" s="18" t="n">
-        <v>0.051</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H61" s="17" t="n">
         <v>0.3</v>
@@ -4060,7 +4060,7 @@
         <v/>
       </c>
       <c r="J61" s="6" t="n">
-        <v>0.61</v>
+        <v>0.72</v>
       </c>
       <c r="K61" s="20">
         <f>IF(I61&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4099,7 +4099,7 @@
         <v>0.5</v>
       </c>
       <c r="G62" s="18" t="n">
-        <v>0.053</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H62" s="17" t="n">
         <v>0.38</v>
@@ -4109,7 +4109,7 @@
         <v/>
       </c>
       <c r="J62" s="6" t="n">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="K62" s="20">
         <f>IF(I62&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4148,7 +4148,7 @@
         <v>0.5</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>0.081</v>
+        <v>0.111</v>
       </c>
       <c r="H63" s="17" t="n">
         <v>0.38</v>
@@ -4158,7 +4158,7 @@
         <v/>
       </c>
       <c r="J63" s="6" t="n">
-        <v>0.78</v>
+        <v>0.9</v>
       </c>
       <c r="K63" s="20">
         <f>IF(I63&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4197,7 +4197,7 @@
         <v>0.5</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>0.081</v>
+        <v>0.111</v>
       </c>
       <c r="H64" s="17" t="n">
         <v>0.49</v>
@@ -4207,7 +4207,7 @@
         <v/>
       </c>
       <c r="J64" s="6" t="n">
-        <v>0.78</v>
+        <v>0.9</v>
       </c>
       <c r="K64" s="20">
         <f>IF(I64&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4246,7 +4246,7 @@
         <v>0.5</v>
       </c>
       <c r="G65" s="18" t="n">
-        <v>0.108</v>
+        <v>0.161</v>
       </c>
       <c r="H65" s="17" t="n">
         <v>0.5</v>
@@ -4256,7 +4256,7 @@
         <v/>
       </c>
       <c r="J65" s="6" t="n">
-        <v>0.89</v>
+        <v>1.04</v>
       </c>
       <c r="K65" s="20">
         <f>IF(I65&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4295,7 +4295,7 @@
         <v>0.5</v>
       </c>
       <c r="G66" s="18" t="n">
-        <v>0.14</v>
+        <v>0.202</v>
       </c>
       <c r="H66" s="17" t="n">
         <v>0.52</v>
@@ -4305,7 +4305,7 @@
         <v/>
       </c>
       <c r="J66" s="6" t="n">
-        <v>0.99</v>
+        <v>1.13</v>
       </c>
       <c r="K66" s="20">
         <f>IF(I66&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4344,7 +4344,7 @@
         <v>0.5</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>0.241</v>
+        <v>0.306</v>
       </c>
       <c r="H67" s="17" t="n">
         <v>0.5600000000000001</v>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="J67" s="6" t="n">
-        <v>1.2</v>
+        <v>1.29</v>
       </c>
       <c r="K67" s="20">
         <f>IF(I67&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4393,7 +4393,7 @@
         <v>0.5</v>
       </c>
       <c r="G68" s="18" t="n">
-        <v>0.309</v>
+        <v>0.372</v>
       </c>
       <c r="H68" s="17" t="n">
         <v>0.62</v>
@@ -4403,7 +4403,7 @@
         <v/>
       </c>
       <c r="J68" s="6" t="n">
-        <v>1.29</v>
+        <v>1.36</v>
       </c>
       <c r="K68" s="20">
         <f>IF(I68&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4442,7 +4442,7 @@
         <v>0.5</v>
       </c>
       <c r="G69" s="18" t="n">
-        <v>0.326</v>
+        <v>0.389</v>
       </c>
       <c r="H69" s="17" t="n">
         <v>0.57</v>
@@ -4452,7 +4452,7 @@
         <v/>
       </c>
       <c r="J69" s="6" t="n">
-        <v>1.31</v>
+        <v>1.37</v>
       </c>
       <c r="K69" s="20">
         <f>IF(I69&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4491,7 +4491,7 @@
         <v>0.5</v>
       </c>
       <c r="G70" s="18" t="n">
-        <v>0.328</v>
+        <v>0.39</v>
       </c>
       <c r="H70" s="17" t="n">
         <v>0.63</v>
@@ -4501,7 +4501,7 @@
         <v/>
       </c>
       <c r="J70" s="6" t="n">
-        <v>1.31</v>
+        <v>1.37</v>
       </c>
       <c r="K70" s="20">
         <f>IF(I70&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4540,7 +4540,7 @@
         <v>0.5</v>
       </c>
       <c r="G71" s="18" t="n">
-        <v>0.328</v>
+        <v>0.39</v>
       </c>
       <c r="H71" s="17" t="n">
         <v>0.64</v>
@@ -4550,7 +4550,7 @@
         <v/>
       </c>
       <c r="J71" s="6" t="n">
-        <v>1.31</v>
+        <v>1.37</v>
       </c>
       <c r="K71" s="20">
         <f>IF(I71&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4589,7 +4589,7 @@
         <v>0.5</v>
       </c>
       <c r="G72" s="18" t="n">
-        <v>0.385</v>
+        <v>0.447</v>
       </c>
       <c r="H72" s="17" t="n">
         <v>0.64</v>
@@ -4599,7 +4599,7 @@
         <v/>
       </c>
       <c r="J72" s="6" t="n">
-        <v>1.37</v>
+        <v>1.42</v>
       </c>
       <c r="K72" s="20">
         <f>IF(I72&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4638,7 +4638,7 @@
         <v>0.5</v>
       </c>
       <c r="G73" s="18" t="n">
-        <v>0.057</v>
+        <v>0.074</v>
       </c>
       <c r="H73" s="17" t="n">
         <v>0.3</v>
@@ -4648,7 +4648,7 @@
         <v/>
       </c>
       <c r="J73" s="6" t="n">
-        <v>0.65</v>
+        <v>0.74</v>
       </c>
       <c r="K73" s="20">
         <f>IF(I73&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4736,7 +4736,7 @@
         <v>0.5</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>0.066</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H75" s="17" t="n">
         <v>0.38</v>
@@ -4746,7 +4746,7 @@
         <v/>
       </c>
       <c r="J75" s="6" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="K75" s="20">
         <f>IF(I75&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4785,7 +4785,7 @@
         <v>0.5</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>0.105</v>
+        <v>0.116</v>
       </c>
       <c r="H76" s="17" t="n">
         <v>0.35</v>
@@ -4795,7 +4795,7 @@
         <v/>
       </c>
       <c r="J76" s="6" t="n">
-        <v>0.87</v>
+        <v>0.91</v>
       </c>
       <c r="K76" s="20">
         <f>IF(I76&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4834,7 +4834,7 @@
         <v>0.5</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>0.105</v>
+        <v>0.116</v>
       </c>
       <c r="H77" s="17" t="n">
         <v>0.35</v>
@@ -4844,7 +4844,7 @@
         <v/>
       </c>
       <c r="J77" s="6" t="n">
-        <v>0.87</v>
+        <v>0.91</v>
       </c>
       <c r="K77" s="20">
         <f>IF(I77&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4883,7 +4883,7 @@
         <v>0.5</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>0.107</v>
+        <v>0.117</v>
       </c>
       <c r="H78" s="17" t="n">
         <v>0.35</v>
@@ -4893,7 +4893,7 @@
         <v/>
       </c>
       <c r="J78" s="6" t="n">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="K78" s="20">
         <f>IF(I78&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4932,7 +4932,7 @@
         <v>0.5</v>
       </c>
       <c r="G79" s="18" t="n">
-        <v>0.138</v>
+        <v>0.147</v>
       </c>
       <c r="H79" s="17" t="n">
         <v>0.35</v>
@@ -4942,7 +4942,7 @@
         <v/>
       </c>
       <c r="J79" s="6" t="n">
-        <v>0.98</v>
+        <v>1.01</v>
       </c>
       <c r="K79" s="20">
         <f>IF(I79&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4981,7 +4981,7 @@
         <v>0.5</v>
       </c>
       <c r="G80" s="18" t="n">
-        <v>0.141</v>
+        <v>0.151</v>
       </c>
       <c r="H80" s="17" t="n">
         <v>0.45</v>
@@ -4991,7 +4991,7 @@
         <v/>
       </c>
       <c r="J80" s="6" t="n">
-        <v>0.99</v>
+        <v>1.02</v>
       </c>
       <c r="K80" s="20">
         <f>IF(I80&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5618,7 +5618,7 @@
         <v>0.5</v>
       </c>
       <c r="G93" s="18" t="n">
-        <v>0.107</v>
+        <v>0.129</v>
       </c>
       <c r="H93" s="17" t="n">
         <v>0.5</v>
@@ -5628,7 +5628,7 @@
         <v/>
       </c>
       <c r="J93" s="6" t="n">
-        <v>0.88</v>
+        <v>0.96</v>
       </c>
       <c r="K93" s="20">
         <f>IF(I93&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5667,7 +5667,7 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="18" t="n">
-        <v>0.108</v>
+        <v>0.129</v>
       </c>
       <c r="H94" s="17" t="n">
         <v>0.4</v>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="J94" s="6" t="n">
-        <v>0.88</v>
+        <v>0.96</v>
       </c>
       <c r="K94" s="20">
         <f>IF(I94&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5716,7 +5716,7 @@
         <v>0.5</v>
       </c>
       <c r="G95" s="18" t="n">
-        <v>0.032</v>
+        <v>0.037</v>
       </c>
       <c r="H95" s="17" t="n">
         <v>0.3</v>
@@ -5726,7 +5726,7 @@
         <v/>
       </c>
       <c r="J95" s="6" t="n">
-        <v>0.47</v>
+        <v>0.51</v>
       </c>
       <c r="K95" s="20">
         <f>IF(I95&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5765,7 +5765,7 @@
         <v>0.5</v>
       </c>
       <c r="G96" s="18" t="n">
-        <v>0.032</v>
+        <v>0.037</v>
       </c>
       <c r="H96" s="17" t="n">
         <v>0.36</v>
@@ -5775,7 +5775,7 @@
         <v/>
       </c>
       <c r="J96" s="6" t="n">
-        <v>0.47</v>
+        <v>0.51</v>
       </c>
       <c r="K96" s="20">
         <f>IF(I96&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5814,7 +5814,7 @@
         <v>0.5</v>
       </c>
       <c r="G97" s="18" t="n">
-        <v>0.051</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H97" s="17" t="n">
         <v>0.36</v>
@@ -5824,7 +5824,7 @@
         <v/>
       </c>
       <c r="J97" s="6" t="n">
-        <v>0.61</v>
+        <v>0.73</v>
       </c>
       <c r="K97" s="20">
         <f>IF(I97&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5863,7 +5863,7 @@
         <v>0.5</v>
       </c>
       <c r="G98" s="18" t="n">
-        <v>0.051</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H98" s="17" t="n">
         <v>0.48</v>
@@ -5873,7 +5873,7 @@
         <v/>
       </c>
       <c r="J98" s="6" t="n">
-        <v>0.61</v>
+        <v>0.73</v>
       </c>
       <c r="K98" s="20">
         <f>IF(I98&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5912,7 +5912,7 @@
         <v>0.5</v>
       </c>
       <c r="G99" s="18" t="n">
-        <v>0.063</v>
+        <v>0.089</v>
       </c>
       <c r="H99" s="17" t="n">
         <v>0.49</v>
@@ -5922,7 +5922,7 @@
         <v/>
       </c>
       <c r="J99" s="6" t="n">
-        <v>0.68</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K99" s="20">
         <f>IF(I99&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5961,7 +5961,7 @@
         <v>0.5</v>
       </c>
       <c r="G100" s="18" t="n">
-        <v>0.026</v>
+        <v>0.038</v>
       </c>
       <c r="H100" s="17" t="n">
         <v>0.3</v>
@@ -5971,7 +5971,7 @@
         <v/>
       </c>
       <c r="J100" s="6" t="n">
-        <v>0.42</v>
+        <v>0.52</v>
       </c>
       <c r="K100" s="20">
         <f>IF(I100&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -6010,7 +6010,7 @@
         <v>0.5</v>
       </c>
       <c r="G101" s="18" t="n">
-        <v>0.026</v>
+        <v>0.038</v>
       </c>
       <c r="H101" s="17" t="n">
         <v>0.37</v>
@@ -6020,7 +6020,7 @@
         <v/>
       </c>
       <c r="J101" s="6" t="n">
-        <v>0.42</v>
+        <v>0.52</v>
       </c>
       <c r="K101" s="20">
         <f>IF(I101&gt;=0.05,"CUMPLE","NO CUMPLE")</f>

</xml_diff>

<commit_message>
Barranquita: analisis estadistico en el formato del usuario (plantilla CAR Varones)
Excel ANALISIS_ESTADISTICO generado desde la plantilla del usuario con LibreOffice (mismas hojas,
formulas y graficos) con la serie de Pongo de Caynarachi 1989-2013. hidrologia_b usa los mismos
metodos de la hoja (K-S, LP3 de Kite, Gumbel yn/sn, modelo de Bell): se adopta Log Pearson III,
P24 169.27 mm, I 293.18 mm/h. Verificacion, memorias y memoria de calculo regenerados; planos y
metrado sin cambios.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/CUADRO_TRAMOS_CUNETAS_IE0590_BARRANQUITA.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>I = 289 mm/h, C ponderado = 0.76, area total 9393 m2; menor borde libre 0.129 m en EJE-11 P-48-P-33 (Q 18.8 l/s, y 0.071, h 0.20)</t>
+          <t>I = 293 mm/h, C ponderado = 0.76, area total 9393 m2; menor borde libre 0.128 m en EJE-11 P-48-P-33 (Q 19.1 l/s, y 0.072, h 0.20)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>V max 1.97 m/s</t>
+          <t>V max 1.98 m/s</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>288.63</v>
+        <v>293.18</v>
       </c>
     </row>
     <row r="6">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>166.64</v>
+        <v>169.27</v>
       </c>
     </row>
     <row r="7">
@@ -1502,7 +1502,7 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>I: tc = 10 min, TR = 25 anos, P10 = 48.11 mm (estacion Pongo de Caynarachi, SENAMHI 003317, 1989-2013; Dick y Peschke). Area tributaria: cada m2 dentro del cerco a la cuneta mas cercana.</t>
+          <t>I: tc = 10 min, TR = 25 anos, P10 = 48.86 mm (estacion Pongo de Caynarachi, SENAMHI 003317, 1989-2013; Dick y Peschke). Area tributaria: cada m2 dentro del cerco a la cuneta mas cercana.</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
         <v>0.5</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>0.094</v>
+        <v>0.095</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>0.3</v>
@@ -1649,7 +1649,7 @@
         <v>0.5</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>0.096</v>
+        <v>0.097</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>0.46</v>
@@ -1698,7 +1698,7 @@
         <v>0.5</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0.083</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>0.3</v>
@@ -1708,7 +1708,7 @@
         <v/>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="K13" s="20">
         <f>IF(I13&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1747,7 +1747,7 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>0.46</v>
@@ -1796,7 +1796,7 @@
         <v>0.5</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.103</v>
+        <v>0.104</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>0.46</v>
@@ -1845,7 +1845,7 @@
         <v>2.92</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>0.09</v>
+        <v>0.091</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>0.52</v>
@@ -1855,7 +1855,7 @@
         <v/>
       </c>
       <c r="J16" s="6" t="n">
-        <v>1.97</v>
+        <v>1.98</v>
       </c>
       <c r="K16" s="20">
         <f>IF(I16&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -1894,7 +1894,7 @@
         <v>0.5</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>0.314</v>
+        <v>0.318</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>0.77</v>
@@ -1943,7 +1943,7 @@
         <v>0.5</v>
       </c>
       <c r="G18" s="18" t="n">
-        <v>0.314</v>
+        <v>0.318</v>
       </c>
       <c r="H18" s="17" t="n">
         <v>0.83</v>
@@ -1992,7 +1992,7 @@
         <v>0.5</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>0.399</v>
+        <v>0.404</v>
       </c>
       <c r="H19" s="17" t="n">
         <v>0.83</v>
@@ -2002,7 +2002,7 @@
         <v/>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="K19" s="20">
         <f>IF(I19&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2041,7 +2041,7 @@
         <v>0.5</v>
       </c>
       <c r="G20" s="18" t="n">
-        <v>0.399</v>
+        <v>0.405</v>
       </c>
       <c r="H20" s="17" t="n">
         <v>0.79</v>
@@ -2051,7 +2051,7 @@
         <v/>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="K20" s="20">
         <f>IF(I20&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2090,7 +2090,7 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>0.448</v>
+        <v>0.453</v>
       </c>
       <c r="H21" s="17" t="n">
         <v>0.79</v>
@@ -2139,7 +2139,7 @@
         <v>0.5</v>
       </c>
       <c r="G22" s="18" t="n">
-        <v>0.091</v>
+        <v>0.092</v>
       </c>
       <c r="H22" s="17" t="n">
         <v>0.3</v>
@@ -2188,7 +2188,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0.077</v>
+        <v>0.078</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>0.3</v>
@@ -2198,7 +2198,7 @@
         <v/>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="K23" s="20">
         <f>IF(I23&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2286,7 +2286,7 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="H25" s="17" t="n">
         <v>0.47</v>
@@ -2335,7 +2335,7 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="18" t="n">
-        <v>0.104</v>
+        <v>0.105</v>
       </c>
       <c r="H26" s="17" t="n">
         <v>0.48</v>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="K26" s="20">
         <f>IF(I26&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2384,7 +2384,7 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0.129</v>
+        <v>0.131</v>
       </c>
       <c r="H27" s="17" t="n">
         <v>0.49</v>
@@ -2433,7 +2433,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="18" t="n">
-        <v>0.139</v>
+        <v>0.141</v>
       </c>
       <c r="H28" s="17" t="n">
         <v>0.57</v>
@@ -2482,7 +2482,7 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0.186</v>
+        <v>0.188</v>
       </c>
       <c r="H29" s="17" t="n">
         <v>0.61</v>
@@ -2492,7 +2492,7 @@
         <v/>
       </c>
       <c r="J29" s="6" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="K29" s="20">
         <f>IF(I29&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2531,7 +2531,7 @@
         <v>0.5</v>
       </c>
       <c r="G30" s="18" t="n">
-        <v>0.059</v>
+        <v>0.06</v>
       </c>
       <c r="H30" s="17" t="n">
         <v>0.3</v>
@@ -2580,7 +2580,7 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0.064</v>
+        <v>0.065</v>
       </c>
       <c r="H31" s="17" t="n">
         <v>0.41</v>
@@ -2629,7 +2629,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="18" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.089</v>
       </c>
       <c r="H32" s="17" t="n">
         <v>0.44</v>
@@ -2678,7 +2678,7 @@
         <v>0.5</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0.093</v>
+        <v>0.094</v>
       </c>
       <c r="H33" s="17" t="n">
         <v>0.53</v>
@@ -2727,7 +2727,7 @@
         <v>0.5</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>0.135</v>
+        <v>0.136</v>
       </c>
       <c r="H34" s="17" t="n">
         <v>0.55</v>
@@ -2737,7 +2737,7 @@
         <v/>
       </c>
       <c r="J34" s="6" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="K34" s="20">
         <f>IF(I34&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2776,7 +2776,7 @@
         <v>0.5</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0.038</v>
+        <v>0.039</v>
       </c>
       <c r="H35" s="17" t="n">
         <v>0.3</v>
@@ -2786,7 +2786,7 @@
         <v/>
       </c>
       <c r="J35" s="6" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="K35" s="20">
         <f>IF(I35&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2874,7 +2874,7 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0.165</v>
+        <v>0.167</v>
       </c>
       <c r="H37" s="17" t="n">
         <v>0.5</v>
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="J37" s="6" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="K37" s="20">
         <f>IF(I37&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2923,7 +2923,7 @@
         <v>0.5</v>
       </c>
       <c r="G38" s="18" t="n">
-        <v>0.219</v>
+        <v>0.221</v>
       </c>
       <c r="H38" s="17" t="n">
         <v>0.59</v>
@@ -2933,7 +2933,7 @@
         <v/>
       </c>
       <c r="J38" s="6" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="K38" s="20">
         <f>IF(I38&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -2972,7 +2972,7 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0.219</v>
+        <v>0.222</v>
       </c>
       <c r="H39" s="17" t="n">
         <v>0.61</v>
@@ -3021,7 +3021,7 @@
         <v>0.5</v>
       </c>
       <c r="G40" s="18" t="n">
-        <v>0.246</v>
+        <v>0.249</v>
       </c>
       <c r="H40" s="17" t="n">
         <v>0.62</v>
@@ -3070,7 +3070,7 @@
         <v>0.5</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0.246</v>
+        <v>0.249</v>
       </c>
       <c r="H41" s="17" t="n">
         <v>0.73</v>
@@ -3119,7 +3119,7 @@
         <v>0.5</v>
       </c>
       <c r="G42" s="18" t="n">
-        <v>0.304</v>
+        <v>0.308</v>
       </c>
       <c r="H42" s="17" t="n">
         <v>0.73</v>
@@ -3168,7 +3168,7 @@
         <v>0.5</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0.338</v>
+        <v>0.342</v>
       </c>
       <c r="H43" s="17" t="n">
         <v>0.79</v>
@@ -3178,7 +3178,7 @@
         <v/>
       </c>
       <c r="J43" s="6" t="n">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="K43" s="20">
         <f>IF(I43&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3217,7 +3217,7 @@
         <v>0.5</v>
       </c>
       <c r="G44" s="18" t="n">
-        <v>0.338</v>
+        <v>0.342</v>
       </c>
       <c r="H44" s="17" t="n">
         <v>0.7</v>
@@ -3227,7 +3227,7 @@
         <v/>
       </c>
       <c r="J44" s="6" t="n">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="K44" s="20">
         <f>IF(I44&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3266,7 +3266,7 @@
         <v>0.5</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>0.338</v>
+        <v>0.343</v>
       </c>
       <c r="H45" s="17" t="n">
         <v>0.7</v>
@@ -3315,7 +3315,7 @@
         <v>0.5</v>
       </c>
       <c r="G46" s="18" t="n">
-        <v>0.339</v>
+        <v>0.343</v>
       </c>
       <c r="H46" s="17" t="n">
         <v>0.74</v>
@@ -3364,7 +3364,7 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>0.34</v>
+        <v>0.344</v>
       </c>
       <c r="H47" s="17" t="n">
         <v>0.74</v>
@@ -3413,7 +3413,7 @@
         <v>0.5</v>
       </c>
       <c r="G48" s="18" t="n">
-        <v>0.34</v>
+        <v>0.345</v>
       </c>
       <c r="H48" s="17" t="n">
         <v>0.77</v>
@@ -3462,7 +3462,7 @@
         <v>0.5</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>0.343</v>
+        <v>0.348</v>
       </c>
       <c r="H49" s="17" t="n">
         <v>0.77</v>
@@ -3472,7 +3472,7 @@
         <v/>
       </c>
       <c r="J49" s="6" t="n">
-        <v>1.33</v>
+        <v>1.34</v>
       </c>
       <c r="K49" s="20">
         <f>IF(I49&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3511,7 +3511,7 @@
         <v>0.5</v>
       </c>
       <c r="G50" s="18" t="n">
-        <v>0.344</v>
+        <v>0.349</v>
       </c>
       <c r="H50" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3521,7 +3521,7 @@
         <v/>
       </c>
       <c r="J50" s="6" t="n">
-        <v>1.33</v>
+        <v>1.34</v>
       </c>
       <c r="K50" s="20">
         <f>IF(I50&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3560,7 +3560,7 @@
         <v>0.5</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>0.344</v>
+        <v>0.349</v>
       </c>
       <c r="H51" s="17" t="n">
         <v>0.8100000000000001</v>
@@ -3570,7 +3570,7 @@
         <v/>
       </c>
       <c r="J51" s="6" t="n">
-        <v>1.33</v>
+        <v>1.34</v>
       </c>
       <c r="K51" s="20">
         <f>IF(I51&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3609,7 +3609,7 @@
         <v>0.5</v>
       </c>
       <c r="G52" s="18" t="n">
-        <v>0.025</v>
+        <v>0.026</v>
       </c>
       <c r="H52" s="17" t="n">
         <v>0.3</v>
@@ -3658,7 +3658,7 @@
         <v>0.5</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>0.119</v>
+        <v>0.12</v>
       </c>
       <c r="H53" s="17" t="n">
         <v>0.32</v>
@@ -3668,7 +3668,7 @@
         <v/>
       </c>
       <c r="J53" s="6" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="K53" s="20">
         <f>IF(I53&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3707,7 +3707,7 @@
         <v>0.5</v>
       </c>
       <c r="G54" s="18" t="n">
-        <v>0.093</v>
+        <v>0.094</v>
       </c>
       <c r="H54" s="17" t="n">
         <v>0.3</v>
@@ -3756,7 +3756,7 @@
         <v>0.5</v>
       </c>
       <c r="G55" s="18" t="n">
-        <v>0.063</v>
+        <v>0.064</v>
       </c>
       <c r="H55" s="17" t="n">
         <v>0.3</v>
@@ -3815,7 +3815,7 @@
         <v/>
       </c>
       <c r="J56" s="6" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="K56" s="20">
         <f>IF(I56&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -3854,7 +3854,7 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H57" s="17" t="n">
         <v>0.42</v>
@@ -3903,7 +3903,7 @@
         <v>0.5</v>
       </c>
       <c r="G58" s="18" t="n">
-        <v>0.089</v>
+        <v>0.09</v>
       </c>
       <c r="H58" s="17" t="n">
         <v>0.42</v>
@@ -3952,7 +3952,7 @@
         <v>0.5</v>
       </c>
       <c r="G59" s="18" t="n">
-        <v>0.089</v>
+        <v>0.09</v>
       </c>
       <c r="H59" s="17" t="n">
         <v>0.48</v>
@@ -4001,7 +4001,7 @@
         <v>0.5</v>
       </c>
       <c r="G60" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H60" s="17" t="n">
         <v>0.2</v>
@@ -4050,7 +4050,7 @@
         <v>0.5</v>
       </c>
       <c r="G61" s="18" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H61" s="17" t="n">
         <v>0.3</v>
@@ -4060,7 +4060,7 @@
         <v/>
       </c>
       <c r="J61" s="6" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="K61" s="20">
         <f>IF(I61&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4099,7 +4099,7 @@
         <v>0.5</v>
       </c>
       <c r="G62" s="18" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.073</v>
       </c>
       <c r="H62" s="17" t="n">
         <v>0.38</v>
@@ -4109,7 +4109,7 @@
         <v/>
       </c>
       <c r="J62" s="6" t="n">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="K62" s="20">
         <f>IF(I62&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4148,7 +4148,7 @@
         <v>0.5</v>
       </c>
       <c r="G63" s="18" t="n">
-        <v>0.111</v>
+        <v>0.112</v>
       </c>
       <c r="H63" s="17" t="n">
         <v>0.38</v>
@@ -4197,7 +4197,7 @@
         <v>0.5</v>
       </c>
       <c r="G64" s="18" t="n">
-        <v>0.111</v>
+        <v>0.112</v>
       </c>
       <c r="H64" s="17" t="n">
         <v>0.49</v>
@@ -4246,7 +4246,7 @@
         <v>0.5</v>
       </c>
       <c r="G65" s="18" t="n">
-        <v>0.161</v>
+        <v>0.163</v>
       </c>
       <c r="H65" s="17" t="n">
         <v>0.5</v>
@@ -4256,7 +4256,7 @@
         <v/>
       </c>
       <c r="J65" s="6" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
       <c r="K65" s="20">
         <f>IF(I65&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4295,7 +4295,7 @@
         <v>0.5</v>
       </c>
       <c r="G66" s="18" t="n">
-        <v>0.202</v>
+        <v>0.204</v>
       </c>
       <c r="H66" s="17" t="n">
         <v>0.52</v>
@@ -4305,7 +4305,7 @@
         <v/>
       </c>
       <c r="J66" s="6" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="K66" s="20">
         <f>IF(I66&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4344,7 +4344,7 @@
         <v>0.5</v>
       </c>
       <c r="G67" s="18" t="n">
-        <v>0.306</v>
+        <v>0.31</v>
       </c>
       <c r="H67" s="17" t="n">
         <v>0.5600000000000001</v>
@@ -4393,7 +4393,7 @@
         <v>0.5</v>
       </c>
       <c r="G68" s="18" t="n">
-        <v>0.372</v>
+        <v>0.377</v>
       </c>
       <c r="H68" s="17" t="n">
         <v>0.62</v>
@@ -4442,7 +4442,7 @@
         <v>0.5</v>
       </c>
       <c r="G69" s="18" t="n">
-        <v>0.389</v>
+        <v>0.394</v>
       </c>
       <c r="H69" s="17" t="n">
         <v>0.57</v>
@@ -4452,7 +4452,7 @@
         <v/>
       </c>
       <c r="J69" s="6" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="K69" s="20">
         <f>IF(I69&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4491,7 +4491,7 @@
         <v>0.5</v>
       </c>
       <c r="G70" s="18" t="n">
-        <v>0.39</v>
+        <v>0.395</v>
       </c>
       <c r="H70" s="17" t="n">
         <v>0.63</v>
@@ -4501,7 +4501,7 @@
         <v/>
       </c>
       <c r="J70" s="6" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="K70" s="20">
         <f>IF(I70&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4540,7 +4540,7 @@
         <v>0.5</v>
       </c>
       <c r="G71" s="18" t="n">
-        <v>0.39</v>
+        <v>0.395</v>
       </c>
       <c r="H71" s="17" t="n">
         <v>0.64</v>
@@ -4550,7 +4550,7 @@
         <v/>
       </c>
       <c r="J71" s="6" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="K71" s="20">
         <f>IF(I71&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4589,7 +4589,7 @@
         <v>0.5</v>
       </c>
       <c r="G72" s="18" t="n">
-        <v>0.447</v>
+        <v>0.453</v>
       </c>
       <c r="H72" s="17" t="n">
         <v>0.64</v>
@@ -4687,7 +4687,7 @@
         <v>0.5</v>
       </c>
       <c r="G74" s="18" t="n">
-        <v>0.064</v>
+        <v>0.065</v>
       </c>
       <c r="H74" s="17" t="n">
         <v>0.3</v>
@@ -4736,7 +4736,7 @@
         <v>0.5</v>
       </c>
       <c r="G75" s="18" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H75" s="17" t="n">
         <v>0.38</v>
@@ -4785,7 +4785,7 @@
         <v>0.5</v>
       </c>
       <c r="G76" s="18" t="n">
-        <v>0.116</v>
+        <v>0.117</v>
       </c>
       <c r="H76" s="17" t="n">
         <v>0.35</v>
@@ -4795,7 +4795,7 @@
         <v/>
       </c>
       <c r="J76" s="6" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="K76" s="20">
         <f>IF(I76&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4834,7 +4834,7 @@
         <v>0.5</v>
       </c>
       <c r="G77" s="18" t="n">
-        <v>0.116</v>
+        <v>0.117</v>
       </c>
       <c r="H77" s="17" t="n">
         <v>0.35</v>
@@ -4844,7 +4844,7 @@
         <v/>
       </c>
       <c r="J77" s="6" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="K77" s="20">
         <f>IF(I77&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -4883,7 +4883,7 @@
         <v>0.5</v>
       </c>
       <c r="G78" s="18" t="n">
-        <v>0.117</v>
+        <v>0.119</v>
       </c>
       <c r="H78" s="17" t="n">
         <v>0.35</v>
@@ -4932,7 +4932,7 @@
         <v>0.5</v>
       </c>
       <c r="G79" s="18" t="n">
-        <v>0.147</v>
+        <v>0.149</v>
       </c>
       <c r="H79" s="17" t="n">
         <v>0.35</v>
@@ -4981,7 +4981,7 @@
         <v>0.5</v>
       </c>
       <c r="G80" s="18" t="n">
-        <v>0.151</v>
+        <v>0.152</v>
       </c>
       <c r="H80" s="17" t="n">
         <v>0.45</v>
@@ -5030,7 +5030,7 @@
         <v>0.5</v>
       </c>
       <c r="G81" s="18" t="n">
-        <v>0.054</v>
+        <v>0.055</v>
       </c>
       <c r="H81" s="17" t="n">
         <v>0.3</v>
@@ -5040,7 +5040,7 @@
         <v/>
       </c>
       <c r="J81" s="6" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="K81" s="20">
         <f>IF(I81&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5089,7 +5089,7 @@
         <v/>
       </c>
       <c r="J82" s="6" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="K82" s="20">
         <f>IF(I82&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5128,7 +5128,7 @@
         <v>0.58</v>
       </c>
       <c r="G83" s="18" t="n">
-        <v>0.102</v>
+        <v>0.103</v>
       </c>
       <c r="H83" s="17" t="n">
         <v>0.35</v>
@@ -5138,7 +5138,7 @@
         <v/>
       </c>
       <c r="J83" s="6" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K83" s="20">
         <f>IF(I83&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5177,7 +5177,7 @@
         <v>0.5</v>
       </c>
       <c r="G84" s="18" t="n">
-        <v>0.112</v>
+        <v>0.113</v>
       </c>
       <c r="H84" s="17" t="n">
         <v>0.35</v>
@@ -5226,7 +5226,7 @@
         <v>0.5</v>
       </c>
       <c r="G85" s="18" t="n">
-        <v>0.081</v>
+        <v>0.082</v>
       </c>
       <c r="H85" s="17" t="n">
         <v>0.3</v>
@@ -5275,7 +5275,7 @@
         <v>0.5</v>
       </c>
       <c r="G86" s="18" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H86" s="17" t="n">
         <v>0.45</v>
@@ -5285,7 +5285,7 @@
         <v/>
       </c>
       <c r="J86" s="6" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="K86" s="20">
         <f>IF(I86&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5324,7 +5324,7 @@
         <v>0.5</v>
       </c>
       <c r="G87" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H87" s="17" t="n">
         <v>0.46</v>
@@ -5373,7 +5373,7 @@
         <v>0.5</v>
       </c>
       <c r="G88" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H88" s="17" t="n">
         <v>0.47</v>
@@ -5383,7 +5383,7 @@
         <v/>
       </c>
       <c r="J88" s="6" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K88" s="20">
         <f>IF(I88&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5422,7 +5422,7 @@
         <v>0.5</v>
       </c>
       <c r="G89" s="18" t="n">
-        <v>0.107</v>
+        <v>0.108</v>
       </c>
       <c r="H89" s="17" t="n">
         <v>0.4</v>
@@ -5432,7 +5432,7 @@
         <v/>
       </c>
       <c r="J89" s="6" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="K89" s="20">
         <f>IF(I89&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5471,7 +5471,7 @@
         <v>0.5</v>
       </c>
       <c r="G90" s="18" t="n">
-        <v>0.107</v>
+        <v>0.108</v>
       </c>
       <c r="H90" s="17" t="n">
         <v>0.4</v>
@@ -5481,7 +5481,7 @@
         <v/>
       </c>
       <c r="J90" s="6" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="K90" s="20">
         <f>IF(I90&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5520,7 +5520,7 @@
         <v>0.51</v>
       </c>
       <c r="G91" s="18" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H91" s="17" t="n">
         <v>0.2</v>
@@ -5530,7 +5530,7 @@
         <v/>
       </c>
       <c r="J91" s="6" t="n">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="K91" s="20">
         <f>IF(I91&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5579,7 +5579,7 @@
         <v/>
       </c>
       <c r="J92" s="6" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="K92" s="20">
         <f>IF(I92&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5618,7 +5618,7 @@
         <v>0.5</v>
       </c>
       <c r="G93" s="18" t="n">
-        <v>0.129</v>
+        <v>0.131</v>
       </c>
       <c r="H93" s="17" t="n">
         <v>0.5</v>
@@ -5667,7 +5667,7 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="18" t="n">
-        <v>0.129</v>
+        <v>0.131</v>
       </c>
       <c r="H94" s="17" t="n">
         <v>0.4</v>
@@ -5775,7 +5775,7 @@
         <v/>
       </c>
       <c r="J96" s="6" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="K96" s="20">
         <f>IF(I96&gt;=0.05,"CUMPLE","NO CUMPLE")</f>
@@ -5814,7 +5814,7 @@
         <v>0.5</v>
       </c>
       <c r="G97" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H97" s="17" t="n">
         <v>0.36</v>
@@ -5863,7 +5863,7 @@
         <v>0.5</v>
       </c>
       <c r="G98" s="18" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H98" s="17" t="n">
         <v>0.48</v>
@@ -5912,7 +5912,7 @@
         <v>0.5</v>
       </c>
       <c r="G99" s="18" t="n">
-        <v>0.089</v>
+        <v>0.09</v>
       </c>
       <c r="H99" s="17" t="n">
         <v>0.49</v>

</xml_diff>